<commit_message>
Update consolidated ablation review workbook
</commit_message>
<xml_diff>
--- a/analysis/jamia_revision_ablation/Lumen_All_New_Ablation_Review_Pairs.xlsx
+++ b/analysis/jamia_revision_ablation/Lumen_All_New_Ablation_Review_Pairs.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All New Pairs" sheetId="1" r:id="R8536a03bb156456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All New Pairs" sheetId="1" r:id="R754eeea57a3f4fb8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12878,7 +12878,7 @@
         <x:v>Andrew Dunbar</x:v>
       </x:c>
       <x:c r="I461" s="9" t="str">
-        <x:v>The patient is not merely missing routine screening information: there is a directly documented systemic exclusion—ischemic heart disease. In addition, the available ophthalmic diagnosis does not establish the trial-defining condition of neovascular glaucoma. Formal eye evaluation could resolve the latter, but it would not remove the known cardiovascular exclusion.</x:v>
+        <x:v>The patient is not merely missing routine screening information: there is a directly documented systemic exclusion, ischemic heart disease. In addition, the available ophthalmic diagnosis does not establish the trial-defining condition of neovascular glaucoma. Formal eye evaluation could resolve the latter, but it would not remove the known cardiovascular exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="462" ht="58" customHeight="1">
@@ -22578,7 +22578,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I803" s="9" t="str">
-        <x:v>CAD coded explicitly without angina pectoris; trial requires symptomatic angina with objective ischemia. No culprit lesion requiring stenting and no PCI/IVUS — angiography led to TAVR for aortic stenosis. Frailty burden also questionable against 2-year TVF endpoint.</x:v>
+        <x:v>CAD coded explicitly without angina pectoris; trial requires symptomatic angina with objective ischemia. No culprit lesion requiring stenting and no PCI/IVUS, angiography led to TAVR for aortic stenosis. Frailty burden also questionable against 2-year TVF endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="804" ht="58" customHeight="1">
@@ -22607,7 +22607,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I804" s="9" t="str">
-        <x:v>Age 71 exceeds the 18–70 window stated in all three enrollment arms; elderly subjects also explicitly excluded. Documented atrial fibrillation separately invalidates beat-to-beat HRV, the study's primary measurement. HbA1c 5.4% would otherwise place her in the non-diabetic comparator arm. Registry age field (min 8, no max) conflicts with criteria text — criteria text weighted.</x:v>
+        <x:v>Age 71 exceeds the 18–70 window stated in all three enrollment arms; elderly subjects also explicitly excluded. Documented atrial fibrillation separately invalidates beat-to-beat HRV, the study's primary measurement. HbA1c 5.4% would otherwise place her in the non-diabetic comparator arm. Registry age field (min 8, no max) conflicts with criteria text, criteria text weighted.</x:v>
       </x:c>
     </x:row>
     <x:row r="805" ht="58" customHeight="1">
@@ -22665,7 +22665,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I806" s="9" t="str">
-        <x:v>Meets age (71 vs ≤75) and has documented essential hypertension; contrast tolerance and eGFR both favorable. Fails because HF + AF + CAD require beta blockade, incompatible with the mandated 6-month ARB/CCB ± thiazide standardized regimen. Dementia with Lewy bodies raises orthostatic hypotension risk (explicit exclusion) and compliance concerns. No BP values or medication list in record — confidence set to Medium accordingly.</x:v>
+        <x:v>Meets age (71 vs ≤75) and has documented essential hypertension; contrast tolerance and eGFR both favorable. Fails because HF + AF + CAD require beta blockade, incompatible with the mandated 6-month ARB/CCB ± thiazide standardized regimen. Dementia with Lewy bodies raises orthostatic hypotension risk (explicit exclusion) and compliance concerns. No BP values or medication list in record, confidence set to Medium accordingly.</x:v>
       </x:c>
     </x:row>
     <x:row r="807" ht="58" customHeight="1">
@@ -22719,7 +22719,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I808" s="9" t="str">
-        <x:v>Most permissive protocol reviewed for this patient — age ≥21 with no ceiling, only moderate calcification required, minimal exclusions — and the calcified coronary lesion substrate is documented. Fails solely because enrollment requires patients undergoing elective/planned PCI; her angiogram led to TAVR, not coronary intervention. No intravascular imaging available to assess the 180° calcium arc criterion.</x:v>
+        <x:v>Most permissive protocol reviewed for this patient, age ≥21 with no ceiling, only moderate calcification required, minimal exclusions, and the calcified coronary lesion substrate is documented. Fails solely because enrollment requires patients undergoing elective/planned PCI; her angiogram led to TAVR, not coronary intervention. No intravascular imaging available to assess the 180° calcium arc criterion.</x:v>
       </x:c>
     </x:row>
     <x:row r="809" ht="58" customHeight="1">
@@ -22748,7 +22748,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I809" s="9" t="str">
-        <x:v>Clears age (71 vs &lt;75), renal function (CKD 1–2), documented coronary calcification, contrast tolerance, hypothyroid not hyper, and no prior stent/CABG (high-priority exclusion avoided). Missing CCTA treated as obtainable per soft-item standard. Fails on comorbidity: no indication for the required repeat coronary angiography, and dementia with Lewy bodies plus AF undermine cardiac MRI cooperation and ECG gating — engaging the grade III–IV heart function and MRI-intolerance exclusions.</x:v>
+        <x:v>Clears age (71 vs &lt;75), renal function (CKD 1–2), documented coronary calcification, contrast tolerance, hypothyroid not hyper, and no prior stent/CABG (high-priority exclusion avoided). Missing CCTA treated as obtainable per soft-item standard. Fails on comorbidity: no indication for the required repeat coronary angiography, and dementia with Lewy bodies plus AF undermine cardiac MRI cooperation and ECG gating, engaging the grade III–IV heart function and MRI-intolerance exclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="810" ht="58" customHeight="1">
@@ -22775,7 +22775,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I810" s="9" t="str">
-        <x:v>Calcified coronary lesion documented and BMI 27.0–27.9 clears the &gt;35 exclusion outright. Fails because the study requires IVUS traversal of a calcified culprit lesion during coronary catheterization — no IVUS, no PCI, no designated culprit lesion; her angiogram led to TAVR. Dementia with Lewy bodies also engages the EU vulnerable-population exclusion for legally incapacitated adults.</x:v>
+        <x:v>Calcified coronary lesion documented and BMI 27.0–27.9 clears the &gt;35 exclusion outright. Fails because the study requires IVUS traversal of a calcified culprit lesion during coronary catheterization, no IVUS, no PCI, no designated culprit lesion; her angiogram led to TAVR. Dementia with Lewy bodies also engages the EU vulnerable-population exclusion for legally incapacitated adults.</x:v>
       </x:c>
     </x:row>
     <x:row r="811" ht="58" customHeight="1">
@@ -22802,7 +22802,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I811" s="9" t="str">
-        <x:v>Procedure record (endovascular cardiac ablation, cardiac mapping, TEE) plus documented AF and heart failure places him directly in the trial's EPU/PVI population; T2DM not required, so non-diabetic status is fine. Clears all evaluable exclusions — Hb 12.5–15.8, no acute infection, troponin normal, no mechanical valve or transplant, creatinine stable. Rated Medium not High because it is unclear whether a qualifying procedure is upcoming vs. already performed, and NTproBNP 7235 leaves the recent-HF-hospitalization exclusion open.</x:v>
+        <x:v>Procedure record (endovascular cardiac ablation, cardiac mapping, TEE) plus documented AF and heart failure places him directly in the trial's EPU/PVI population; T2DM not required, so non-diabetic status is fine. Clears all evaluable exclusions, Hb 12.5–15.8, no acute infection, troponin normal, no mechanical valve or transplant, creatinine stable. Rated Medium not High because it is unclear whether a qualifying procedure is upcoming vs. already performed, and NTproBNP 7235 leaves the recent-HF-hospitalization exclusion open.</x:v>
       </x:c>
     </x:row>
     <x:row r="812" ht="58" customHeight="1">
@@ -22831,7 +22831,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I812" s="9" t="str">
-        <x:v>Atrial fibrillation is explicitly named in the exclusion criteria as a disqualifying serious medical condition; he has it documented and underwent ablation with mapping and TEE for it. Trial requires LVEF ≥50% — no EF in record, but cardiomegaly, NTproBNP 7235, and a 51M smoker phenotype argue for reduced rather than preserved function. eGFR clears the &gt;30 threshold cleanly and no secondary hypertension. Rated Medium because the AF exclusion is investigator-discretionary and he may be in post-ablation sinus rhythm; retrieving the echo EF would resolve this pair definitively.</x:v>
+        <x:v>Atrial fibrillation is explicitly named in the exclusion criteria as a disqualifying serious medical condition; he has it documented and underwent ablation with mapping and TEE for it. Trial requires LVEF ≥50%, no EF in record, but cardiomegaly, NTproBNP 7235, and a 51M smoker phenotype argue for reduced rather than preserved function. eGFR clears the &gt;30 threshold cleanly and no secondary hypertension. Rated Medium because the AF exclusion is investigator-discretionary and he may be in post-ablation sinus rhythm; retrieving the echo EF would resolve this pair definitively.</x:v>
       </x:c>
     </x:row>
     <x:row r="813" ht="58" customHeight="1">
@@ -22860,7 +22860,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I813" s="9" t="str">
-        <x:v>Trial enrolls patients scheduled for laparoscopic hepatectomy; patient has no hepatic pathology and no planned abdominal surgery — his entire procedure record is cardiac. Independently triggers the high-priority active cardiac conditions exclusion on three counts: history of CHF, significant arrhythmia (AF, ablated), and probable decompensation (NTproBNP 7235). Bilirubin 1.1 mg/dL is the only hepatic criterion he passes.</x:v>
+        <x:v>Trial enrolls patients scheduled for laparoscopic hepatectomy; patient has no hepatic pathology and no planned abdominal surgery, his entire procedure record is cardiac. Independently triggers the high-priority active cardiac conditions exclusion on three counts: history of CHF, significant arrhythmia (AF, ablated), and probable decompensation (NTproBNP 7235). Bilirubin 1.1 mg/dL is the only hepatic criterion he passes.</x:v>
       </x:c>
     </x:row>
     <x:row r="814" ht="58" customHeight="1">
@@ -22889,7 +22889,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I814" s="9" t="str">
-        <x:v>"History of atrial fibrillation" is a standalone high-priority exclusion; patient has documented AF status post catheter ablation with mapping and TEE — categorical and unambiguous. Also likely triggers NYHA III–IV/reduced EF, structural heart disease (cardiomegaly), loop diuretic use, and ≥2 antihypertensive exclusions. Trial targets uncomplicated grade 1–2 hypertension on ≤1 agent; he is a complex cardiac patient (NTproBNP 7235, cardiomegaly, 2nd-degree AV block). Age 51 and hypertension diagnosis are the only criteria he clears.</x:v>
+        <x:v>"History of atrial fibrillation" is a standalone high-priority exclusion; patient has documented AF status post catheter ablation with mapping and TEE, categorical and unambiguous. Also likely triggers NYHA III–IV/reduced EF, structural heart disease (cardiomegaly), loop diuretic use, and ≥2 antihypertensive exclusions. Trial targets uncomplicated grade 1–2 hypertension on ≤1 agent; he is a complex cardiac patient (NTproBNP 7235, cardiomegaly, 2nd-degree AV block). Age 51 and hypertension diagnosis are the only criteria he clears.</x:v>
       </x:c>
     </x:row>
     <x:row r="815" ht="58" customHeight="1">
@@ -22916,7 +22916,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I815" s="9" t="str">
-        <x:v>Observational hypertension registry with minimal participation burden — no drug, procedure, or washout. Documented primary hypertension with no secondary cause; no psychiatric diagnosis. Sole open item is the untresholded "liver and kidney dysfunction" exclusion: ALT 55 / AST 53 (mild, congestive pattern, normal bilirubin and alk phos) and creatinine 1.3–1.6 giving eGFR ~48–62, stable across 5 draws. Read permissively given no drug exposure or procedural risk. Site is a single hospital in Xinjiang, China — treated as logistical per review standard, not weighted.</x:v>
+        <x:v>Observational hypertension registry with minimal participation burden, no drug, procedure, or washout. Documented primary hypertension with no secondary cause; no psychiatric diagnosis. Sole open item is the untresholded "liver and kidney dysfunction" exclusion: ALT 55 / AST 53 (mild, congestive pattern, normal bilirubin and alk phos) and creatinine 1.3–1.6 giving eGFR ~48–62, stable across 5 draws. Read permissively given no drug exposure or procedural risk. Site is a single hospital in Xinjiang, China, treated as logistical per review standard, not weighted.</x:v>
       </x:c>
     </x:row>
     <x:row r="816" ht="58" customHeight="1">
@@ -22943,7 +22943,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I816" s="9" t="str">
-        <x:v>Digital self-management app added to usual care — no drug, procedure, or washout, and notably NO cardiac exclusions, so the AF and heart failure that disqualified PAIR-000862 and 000864 are irrelevant here. Documented primary hypertension, no secondary cause; mild stable renal impairment (eGFR ~48–62) read as cardiorenal rather than causative. Low confidence because both decisive criteria depend on absent data: no BP values anywhere (needs office SBP ≥140 and home ≥135), and likely &gt;triple antihypertensive combination given HF+AF+HTN regimen. High screen-failure risk.</x:v>
+        <x:v>Digital self-management app added to usual care, no drug, procedure, or washout, and notably NO cardiac exclusions, so the AF and heart failure that disqualified PAIR-000862 and 000864 are irrelevant here. Documented primary hypertension, no secondary cause; mild stable renal impairment (eGFR ~48–62) read as cardiorenal rather than causative. Low confidence because both decisive criteria depend on absent data: no BP values anywhere (needs office SBP ≥140 and home ≥135), and likely &gt;triple antihypertensive combination given HF+AF+HTN regimen. High screen-failure risk.</x:v>
       </x:c>
     </x:row>
     <x:row r="817" ht="58" customHeight="1">
@@ -22970,7 +22970,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I817" s="9" t="str">
-        <x:v>Community health behavior intervention, no drug/procedure and no cardiac exclusions. Both high-priority inclusions met (age 51 vs 18–80; intact language and communication) and the sole high-priority exclusion — impaired memory, behavioral, or language ability — clearly absent, as he has no cognitive or psychiatric diagnosis. Documented tobacco use disorder makes him a substantively good fit. Open items are lower priority: no BP values to grade mild-to-moderate severity, and community residency unconfirmed given a "residential institution" place-of-occurrence code in his record.</x:v>
+        <x:v>Community health behavior intervention, no drug/procedure and no cardiac exclusions. Both high-priority inclusions met (age 51 vs 18–80; intact language and communication) and the sole high-priority exclusion, impaired memory, behavioral, or language ability, clearly absent, as he has no cognitive or psychiatric diagnosis. Documented tobacco use disorder makes him a substantively good fit. Open items are lower priority: no BP values to grade mild-to-moderate severity, and community residency unconfirmed given a "residential institution" place-of-occurrence code in his record.</x:v>
       </x:c>
     </x:row>
     <x:row r="818" ht="58" customHeight="1">
@@ -22999,7 +22999,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I818" s="9" t="str">
-        <x:v>Trial requires newly diagnosed, antihypertensive-naive primary hypertension randomized to first-line metoprolol, ramipril, or amlodipine. Patient has established cardiovascular disease — heart failure (NTproBNP 7235), cardiomegaly indicating chronic remodeling, AF, and 2nd-degree AV block — with a digoxin level confirming existing cardiac pharmacotherapy. Also a safety issue: metoprolol arm is hazardous with 2nd-degree AV block, and the other two arms would leave HF/AF undertreated. Clears the high-priority balance criteria (no neurological, vestibular, orthopedic, or psychiatric conditions) and has no secondary hypertension.</x:v>
+        <x:v>Trial requires newly diagnosed, antihypertensive-naive primary hypertension randomized to first-line metoprolol, ramipril, or amlodipine. Patient has established cardiovascular disease, heart failure (NTproBNP 7235), cardiomegaly indicating chronic remodeling, AF, and 2nd-degree AV block, with a digoxin level confirming existing cardiac pharmacotherapy. Also a safety issue: metoprolol arm is hazardous with 2nd-degree AV block, and the other two arms would leave HF/AF undertreated. Clears the high-priority balance criteria (no neurological, vestibular, orthopedic, or psychiatric conditions) and has no secondary hypertension.</x:v>
       </x:c>
     </x:row>
     <x:row r="819" ht="58" customHeight="1">
@@ -23028,7 +23028,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I819" s="9" t="str">
-        <x:v>Two explicitly named exclusions hit with affirmative documentation: atrial fibrillation (documented, status post ablation with mapping and TEE) and oral anticoagulant use (INR 1.3–3.3 with PT 15.1–32.9 sec across 4 draws — lab-proven VKA therapy). Also likely triggers LVEF &lt;55% (NTproBNP 7235, cardiomegaly) and indispensable beta-blocker/MRA use given HF and AF, neither of which is in the perindopril/indapamide/amlodipine fixed combination. Clears eGFR &gt;30 and no secondary hypertension or valvular disease.</x:v>
+        <x:v>Two explicitly named exclusions hit with affirmative documentation: atrial fibrillation (documented, status post ablation with mapping and TEE) and oral anticoagulant use (INR 1.3–3.3 with PT 15.1–32.9 sec across 4 draws, lab-proven VKA therapy). Also likely triggers LVEF &lt;55% (NTproBNP 7235, cardiomegaly) and indispensable beta-blocker/MRA use given HF and AF, neither of which is in the perindopril/indapamide/amlodipine fixed combination. Clears eGFR &gt;30 and no secondary hypertension or valvular disease.</x:v>
       </x:c>
     </x:row>
     <x:row r="820" ht="58" customHeight="1">
@@ -23057,7 +23057,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I820" s="9" t="str">
-        <x:v>Has the target diagnosis and clears eGFR &gt;30, no severe hyperkalemia history (max K 5.1), and no AF exclusion in this protocol. Fails on disease state: trial requires chronic STABLE heart failure, NYHA I–II, optimal volume status, decompensation-free 60 days. NTproBNP 7235 with congestive transaminitis (ALT 55/AST 53, normal bili) and creatinine 1.3–1.6 argues against euvolemia. IV aldosterone infusion also engages the "high risk" safety exclusion in a possibly congested patient. Recent ablation with labile INR undermines the 8-week medication stability requirement. Note: potentially time-limited — worth re-screening once optimized.</x:v>
+        <x:v>Has the target diagnosis and clears eGFR &gt;30, no severe hyperkalemia history (max K 5.1), and no AF exclusion in this protocol. Fails on disease state: trial requires chronic STABLE heart failure, NYHA I–II, optimal volume status, decompensation-free 60 days. NTproBNP 7235 with congestive transaminitis (ALT 55/AST 53, normal bili) and creatinine 1.3–1.6 argues against euvolemia. IV aldosterone infusion also engages the "high risk" safety exclusion in a possibly congested patient. Recent ablation with labile INR undermines the 8-week medication stability requirement. Note: potentially time-limited, worth re-screening once optimized.</x:v>
       </x:c>
     </x:row>
     <x:row r="821" ht="58" customHeight="1">
@@ -23144,7 +23144,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I823" s="9" t="str">
-        <x:v>Trial targets CAD and he has it, with no recent MI or PCI. Clears BMI (32.0–32.9 vs &gt;42), hemoglobin, potassium, and creatinine thresholds cleanly. Fails on comorbidity: trial requires CPET without orthopedic limitation, and he has bilateral hip/knee replacements, lumbar-lumbosacral fusion of 2–3 vertebrae, arthrodesis, spinal stenosis, spondylolisthesis, spondylosis, osteoarthrosis, and chronic pain — triggering both the inclusion criterion and the "unable to exercise" exclusion. Persistent AF also excluded, evidenced by electric cardioversion. COPD raises the severe lung disease exclusion.</x:v>
+        <x:v>Trial targets CAD and he has it, with no recent MI or PCI. Clears BMI (32.0–32.9 vs &gt;42), hemoglobin, potassium, and creatinine thresholds cleanly. Fails on comorbidity: trial requires CPET without orthopedic limitation, and he has bilateral hip/knee replacements, lumbar-lumbosacral fusion of 2–3 vertebrae, arthrodesis, spinal stenosis, spondylolisthesis, spondylosis, osteoarthrosis, and chronic pain, triggering both the inclusion criterion and the "unable to exercise" exclusion. Persistent AF also excluded, evidenced by electric cardioversion. COPD raises the severe lung disease exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="824" ht="58" customHeight="1">
@@ -23173,7 +23173,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I824" s="9" t="str">
-        <x:v>Trial requires severe symptomatic aortic stenosis with TAVI scheduled. Patient has no valvular disease of any kind — and his echocardiogram was performed with no valve pathology coded, so this is an informed absence rather than missing data. No TAVI or valve procedure documented; only cardiac procedure is external cardioversion. Meets age ≥60 and clears the spironolactone-relevant safety thresholds cleanly (creatinine 0.7–1.1, potassium 3.7–4.6). Possible EF &lt;35% with MRA indication would be a further concern in a genuine candidate.</x:v>
+        <x:v>Trial requires severe symptomatic aortic stenosis with TAVI scheduled. Patient has no valvular disease of any kind, and his echocardiogram was performed with no valve pathology coded, so this is an informed absence rather than missing data. No TAVI or valve procedure documented; only cardiac procedure is external cardioversion. Meets age ≥60 and clears the spironolactone-relevant safety thresholds cleanly (creatinine 0.7–1.1, potassium 3.7–4.6). Possible EF &lt;35% with MRA indication would be a further concern in a genuine candidate.</x:v>
       </x:c>
     </x:row>
     <x:row r="825" ht="58" customHeight="1">
@@ -23202,7 +23202,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I825" s="9" t="str">
-        <x:v>Trial randomizes at the time of type 1 MI treated with PCI plus drug-eluting stent. Patient has CAD but no MI, no PCI, no stent, and no troponin values anywhere in his lab panel — no biochemical basis for infarction. Independently and permanently excluded by "indication for oral anticoagulation": long-term anticoagulant use is an explicit diagnosis code, with three indications (AF, prior VTE, acute proximal DVT). Would likely have met the PRECISE-DAPT ≥25 high bleeding risk criterion (age 68, platelets 83–159, thrombocytopenia).</x:v>
+        <x:v>Trial randomizes at the time of type 1 MI treated with PCI plus drug-eluting stent. Patient has CAD but no MI, no PCI, no stent, and no troponin values anywhere in his lab panel, no biochemical basis for infarction. Independently and permanently excluded by "indication for oral anticoagulation": long-term anticoagulant use is an explicit diagnosis code, with three indications (AF, prior VTE, acute proximal DVT). Would likely have met the PRECISE-DAPT ≥25 high bleeding risk criterion (age 68, platelets 83–159, thrombocytopenia).</x:v>
       </x:c>
     </x:row>
     <x:row r="826" ht="58" customHeight="1">
@@ -23231,7 +23231,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I826" s="9" t="str">
-        <x:v>Observational study of patients who already underwent intracoronary acetylcholine provocative testing at CAG — stated as both an inclusion criterion and, in negative form, as the first exclusion. Patient has never had coronary angiography; procedures are cardioversion, echo, and two lumbar fusions. Neither INOCA nor MINOCA establishable: no troponin anywhere in his lab panel, no documented angina or inducible ischemia, no angiographic anatomy. Documented CAD also sits against a population defined by non-obstructive arteries. Only criterion met is age ≥18.</x:v>
+        <x:v>Observational study of patients who already underwent intracoronary acetylcholine provocative testing at CAG, stated as both an inclusion criterion and, in negative form, as the first exclusion. Patient has never had coronary angiography; procedures are cardioversion, echo, and two lumbar fusions. Neither INOCA nor MINOCA establishable: no troponin anywhere in his lab panel, no documented angina or inducible ischemia, no angiographic anatomy. Documented CAD also sits against a population defined by non-obstructive arteries. Only criterion met is age ≥18.</x:v>
       </x:c>
     </x:row>
     <x:row r="827" ht="58" customHeight="1">
@@ -23258,7 +23258,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I827" s="9" t="str">
-        <x:v>Observational echo study of atriogenic secondary tricuspid regurgitation in persistent/permanent AF. Target rhythm satisfied on procedural evidence — electric cardioversion indicates persistent AF. All five exclusions cleanly absent (no pacemaker/ICD, no valve surgery, no transplant, no organic TR, not pregnant); prior echo confirms an obtainable acoustic window. Low confidence because two inclusion thresholds are unmeasured and at genuine risk: LVEF &gt;50% against documented heart failure and other cardiomyopathies, and PASP &lt;50 mmHg against COPD plus heart failure. Both resolved by the study's own baseline echo. No NTproBNP in record and normal creatinine argue against severe congestion.</x:v>
+        <x:v>Observational echo study of atriogenic secondary tricuspid regurgitation in persistent/permanent AF. Target rhythm satisfied on procedural evidence, electric cardioversion indicates persistent AF. All five exclusions cleanly absent (no pacemaker/ICD, no valve surgery, no transplant, no organic TR, not pregnant); prior echo confirms an obtainable acoustic window. Low confidence because two inclusion thresholds are unmeasured and at genuine risk: LVEF &gt;50% against documented heart failure and other cardiomyopathies, and PASP &lt;50 mmHg against COPD plus heart failure. Both resolved by the study's own baseline echo. No NTproBNP in record and normal creatinine argue against severe congestion.</x:v>
       </x:c>
     </x:row>
     <x:row r="828" ht="58" customHeight="1">
@@ -23312,7 +23312,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I829" s="9" t="str">
-        <x:v>Trial targets CHD with chronic heart failure and he has both. Excluded categorically by documented chronic hepatitis C, explicitly named in the exclusion criteria and standard for Phase Ib PK work. Also triggers "serious diseases of other systems": hepatic (hep C, albumin 3.0–3.5) and hematopoietic (thrombocytopenia, platelets 83–159, WBC to 3.0) — a picture suggestive of cirrhosis with hypersplenism. Coded "other cardiomyopathies" sits against the non-ischemic HF etiology exclusion. Clears transaminases (&lt;3× ULN), eGFR, potassium, and glycemic thresholds. Borderline on anemia (Hb 11–15 vs 12.0 g/dL floor).</x:v>
+        <x:v>Trial targets CHD with chronic heart failure and he has both. Excluded categorically by documented chronic hepatitis C, explicitly named in the exclusion criteria and standard for Phase Ib PK work. Also triggers "serious diseases of other systems": hepatic (hep C, albumin 3.0–3.5) and hematopoietic (thrombocytopenia, platelets 83–159, WBC to 3.0), a picture suggestive of cirrhosis with hypersplenism. Coded "other cardiomyopathies" sits against the non-ischemic HF etiology exclusion. Clears transaminases (&lt;3× ULN), eGFR, potassium, and glycemic thresholds. Borderline on anemia (Hb 11–15 vs 12.0 g/dL floor).</x:v>
       </x:c>
     </x:row>
     <x:row r="830" ht="58" customHeight="1">
@@ -23341,7 +23341,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I830" s="9" t="str">
-        <x:v>BMI explicitly coded as 32.0–32.9 against an exclusion at ≥30 kg/m² — the cleanest documented threshold failure in the set, requiring no inference. Also fails the procedural gate: trial randomizes ablation strategy at first-time catheter ablation, and he has had cardioversion only, with no ablation documented or planned. High-priority thromboembolism-within-6-months exclusion likely triggered by coded acute proximal DVT. Clears age (68 vs ≤75), transaminases (&lt;3× ULN), renal function, anticoagulant tolerance, and no prior ablation. LVEF, left atrial diameter, and AF duration all unmeasured.</x:v>
+        <x:v>BMI explicitly coded as 32.0–32.9 against an exclusion at ≥30 kg/m², the cleanest documented threshold failure in the set, requiring no inference. Also fails the procedural gate: trial randomizes ablation strategy at first-time catheter ablation, and he has had cardioversion only, with no ablation documented or planned. High-priority thromboembolism-within-6-months exclusion likely triggered by coded acute proximal DVT. Clears age (68 vs ≤75), transaminases (&lt;3× ULN), renal function, anticoagulant tolerance, and no prior ablation. LVEF, left atrial diameter, and AF duration all unmeasured.</x:v>
       </x:c>
     </x:row>
     <x:row r="831" ht="58" customHeight="1">
@@ -23370,7 +23370,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I831" s="9" t="str">
-        <x:v>Trial requires hypertrophic obstructive cardiomyopathy plus ≥12 weeks of stable mavacamten. Patient's cardiac code is "Other cardiomyopathies" — a residual ICD category distinct from the hypertrophic forms — with no LVH, outflow obstruction, or septal findings documented; his phenotype is ischemic/hypertensive. Mavacamten is licensed only for obstructive HCM, so the drug prerequisite is downstream of a disease he lacks and cannot be met by screening. Intervention is 6 weeks of supervised endurance/resistance training plus CPET, unachievable given bilateral hip/knee replacements, lumbar fusion, spinal stenosis, chronic pain, and COPD. Notably clears the AF exclusion — persistent AF but anticoagulated (INR 1.0–1.8).</x:v>
+        <x:v>Trial requires hypertrophic obstructive cardiomyopathy plus ≥12 weeks of stable mavacamten. Patient's cardiac code is "Other cardiomyopathies", a residual ICD category distinct from the hypertrophic forms, with no LVH, outflow obstruction, or septal findings documented; his phenotype is ischemic/hypertensive. Mavacamten is licensed only for obstructive HCM, so the drug prerequisite is downstream of a disease he lacks and cannot be met by screening. Intervention is 6 weeks of supervised endurance/resistance training plus CPET, unachievable given bilateral hip/knee replacements, lumbar fusion, spinal stenosis, chronic pain, and COPD. Notably clears the AF exclusion, persistent AF but anticoagulated (INR 1.0–1.8).</x:v>
       </x:c>
     </x:row>
     <x:row r="832" ht="58" customHeight="1">
@@ -23397,7 +23397,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I832" s="9" t="str">
-        <x:v>Study compares lead-placement techniques during a PPM/ICD implant occurring as routine care; short criteria list and he clears all stated exclusions. Device indication not documented but plausible: heart failure, other cardiomyopathies, sudden_cardiac_death tag, unspecified tachycardia; EF &lt;35% would make primary-prevention ICD a guideline indication. Persistent AF exclusion is conditional on cardioversion being contraindicated — his completed electric cardioversion demonstrates it is not. Creatinine 0.7–1.1 clears the &gt;3.0 threshold cleanly (contrast used). Low confidence: device indication unconfirmed. Note thrombocytopenia (platelets 83–159) on dual antithrombotic therapy — pocket hematoma risk, periprocedural rather than eligibility.</x:v>
+        <x:v>Study compares lead-placement techniques during a PPM/ICD implant occurring as routine care; short criteria list and he clears all stated exclusions. Device indication not documented but plausible: heart failure, other cardiomyopathies, sudden_cardiac_death tag, unspecified tachycardia; EF &lt;35% would make primary-prevention ICD a guideline indication. Persistent AF exclusion is conditional on cardioversion being contraindicated, his completed electric cardioversion demonstrates it is not. Creatinine 0.7–1.1 clears the &gt;3.0 threshold cleanly (contrast used). Low confidence: device indication unconfirmed. Note thrombocytopenia (platelets 83–159) on dual antithrombotic therapy, pocket hematoma risk, periprocedural rather than eligibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="833" ht="58" customHeight="1">
@@ -23455,7 +23455,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I834" s="9" t="str">
-        <x:v>eGFR fits the 20–60 window (creatinine 1.1–1.7, age 79M) and CKD is documented — the one criterion met. Excluded by life-expectancy &lt;2 years: encounter for palliative care and DNR status both explicitly coded, with advanced Alzheimer's, bilateral post-stroke hemiplegia, communicating hydrocephalus, aspiration pneumonitis, and tube feeding. Also excluded for inability to comply — aphasia, dysarthria, encephalopathy, physical restraints — in a 6-month blinded trial with cognitive, depression, and QoL endpoints. Fails the stable-antihyperglycemic requirement: glucose 49–1000 mg/dL, HbA1c 6.7–11.5%, "NIDDM UNCONTROLLED" coded. Possible recent MI (troponin to 0.22, subendocardial infarction subsequent episode) and stroke within the 12-week window.</x:v>
+        <x:v>eGFR fits the 20–60 window (creatinine 1.1–1.7, age 79M) and CKD is documented, the one criterion met. Excluded by life-expectancy &lt;2 years: encounter for palliative care and DNR status both explicitly coded, with advanced Alzheimer's, bilateral post-stroke hemiplegia, communicating hydrocephalus, aspiration pneumonitis, and tube feeding. Also excluded for inability to comply, aphasia, dysarthria, encephalopathy, physical restraints, in a 6-month blinded trial with cognitive, depression, and QoL endpoints. Fails the stable-antihyperglycemic requirement: glucose 49–1000 mg/dL, HbA1c 6.7–11.5%, "NIDDM UNCONTROLLED" coded. Possible recent MI (troponin to 0.22, subendocardial infarction subsequent episode) and stroke within the 12-week window.</x:v>
       </x:c>
     </x:row>
     <x:row r="835" ht="58" customHeight="1">
@@ -23542,7 +23542,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I837" s="9" t="str">
-        <x:v>Qualifying MI history is genuine (subendocardial infarction, initial and subsequent episodes; troponin T to 0.22) and this is a history requirement rather than an acute window. Excluded by "uncontrolled diabetes" — NIDDM UNCONTROLLED explicitly coded, glucose 49–1000 mg/dL, HbA1c 6.7–11.5%. Cannot consent (Alzheimer's, aphasia, encephalopathy, physical restraints) or complete assessments: 6-minute walk test unperformable with bilateral post-stroke hemiplegia, symptom diary uncompletable. Palliative care encounter and DNR status against a 6-month protocol with monthly visits. Likely triggers the endoscopic-procedure-within-6-months exclusion (colonoscopy, EGD, spinal tap, CVC). Notably clears TB (tuberculin reaction coded WITHOUT active TB), no NYHA IV heart failure, no active cancer, no carotid intervention. NOTE: trial's exclusion_criteria array is empty in source — all exclusions parsed into the inclusion array.</x:v>
+        <x:v>Qualifying MI history is genuine (subendocardial infarction, initial and subsequent episodes; troponin T to 0.22) and this is a history requirement rather than an acute window. Excluded by "uncontrolled diabetes", NIDDM UNCONTROLLED explicitly coded, glucose 49–1000 mg/dL, HbA1c 6.7–11.5%. Cannot consent (Alzheimer's, aphasia, encephalopathy, physical restraints) or complete assessments: 6-minute walk test unperformable with bilateral post-stroke hemiplegia, symptom diary uncompletable. Palliative care encounter and DNR status against a 6-month protocol with monthly visits. Likely triggers the endoscopic-procedure-within-6-months exclusion (colonoscopy, EGD, spinal tap, CVC). Notably clears TB (tuberculin reaction coded WITHOUT active TB), no NYHA IV heart failure, no active cancer, no carotid intervention. NOTE: trial's exclusion_criteria array is empty in source, all exclusions parsed into the inclusion array.</x:v>
       </x:c>
     </x:row>
     <x:row r="838" ht="58" customHeight="1">
@@ -23571,7 +23571,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I838" s="9" t="str">
-        <x:v>Trial targets high-risk PRIMARY prevention patients; he has established clinical ASCVD (subendocardial MI initial and subsequent, left MCA embolic infarct, atherosclerotic coronary disease). All three qualifying routes fail — ASCVD Risk Estimator is primary-prevention only, "subclinical" atherosclerosis excludes clinically manifest disease, and the diabetes route requires stable HbA1c &lt;8.5% against his 6.7–11.5%. Same value affirmatively triggers the uncontrolled-diabetes exclusion (&gt;8.5%). Age criterion uniquely requires ability to "provide self-consent," foreclosing surrogate consent — Alzheimer's, aphasia, encephalopathy, physical restraints. Palliative care and DNR status trigger investigator-unsuitability in a 12-month protocol with 5 visits, 3 injections, and surveys. LDL 125–128 and non-HDL ~143–149 would otherwise have qualified.</x:v>
+        <x:v>Trial targets high-risk PRIMARY prevention patients; he has established clinical ASCVD (subendocardial MI initial and subsequent, left MCA embolic infarct, atherosclerotic coronary disease). All three qualifying routes fail, ASCVD Risk Estimator is primary-prevention only, "subclinical" atherosclerosis excludes clinically manifest disease, and the diabetes route requires stable HbA1c &lt;8.5% against his 6.7–11.5%. Same value affirmatively triggers the uncontrolled-diabetes exclusion (&gt;8.5%). Age criterion uniquely requires ability to "provide self-consent," foreclosing surrogate consent, Alzheimer's, aphasia, encephalopathy, physical restraints. Palliative care and DNR status trigger investigator-unsuitability in a 12-month protocol with 5 visits, 3 injections, and surveys. LDL 125–128 and non-HDL ~143–149 would otherwise have qualified.</x:v>
       </x:c>
     </x:row>
     <x:row r="839" ht="58" customHeight="1">
@@ -23600,7 +23600,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I839" s="9" t="str">
-        <x:v>Case-control study with five population groups: four require ages 18–35, the fifth (older adults) requires 65–75. He is 79 — outside all of them. Older adults group also requires being free of cognitive or mental health disorders, directly contradicted by Alzheimer's disease plus multiple dementia and encephalopathy codes. Cannot undergo the required cardiorespiratory fitness testing or spirometry given bilateral post-stroke hemiplegia and physical restraints. Documented sleep disorder is sleep apnea, not insomnia. Would also fail metabolic syndrome criteria on their own terms — triglycerides 92–104 (&lt;150) and HDL 44 (&gt;40). Palliative care and DNR status coded.</x:v>
+        <x:v>Case-control study with five population groups: four require ages 18–35, the fifth (older adults) requires 65–75. He is 79, outside all of them. Older adults group also requires being free of cognitive or mental health disorders, directly contradicted by Alzheimer's disease plus multiple dementia and encephalopathy codes. Cannot undergo the required cardiorespiratory fitness testing or spirometry given bilateral post-stroke hemiplegia and physical restraints. Documented sleep disorder is sleep apnea, not insomnia. Would also fail metabolic syndrome criteria on their own terms, triglycerides 92–104 (&lt;150) and HDL 44 (&gt;40). Palliative care and DNR status coded.</x:v>
       </x:c>
     </x:row>
     <x:row r="840" ht="58" customHeight="1">
@@ -23629,7 +23629,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I840" s="9" t="str">
-        <x:v>Age 79 exceeds the ≤75 high-priority ceiling. Registry structured age field reads min 4 / no maximum, contradicting the criteria text — a matcher reading structured fields would not catch this. Also: probable eGFR &lt;45 (creatinine 1.1–1.7 at age 79M, hypertensive CKD documented); palliative care encounter and DNR status trigger the &lt;1-year life expectancy and investigator-unsuitability exclusions; cannot consent (Alzheimer's, aphasia, encephalopathy, physical restraints); CKD raises suspected secondary hypertension against a trial premised on primary hypertension; coded subendocardial MI and left MCA embolic stroke bear on the recent-vascular-events exclusion. Clears Type 1 DM, contrast allergy, prior denervation, and the respiratory support exclusion (sleep apnea explicitly carved out).</x:v>
+        <x:v>Age 79 exceeds the ≤75 high-priority ceiling. Registry structured age field reads min 4 / no maximum, contradicting the criteria text, a matcher reading structured fields would not catch this. Also: probable eGFR &lt;45 (creatinine 1.1–1.7 at age 79M, hypertensive CKD documented); palliative care encounter and DNR status trigger the &lt;1-year life expectancy and investigator-unsuitability exclusions; cannot consent (Alzheimer's, aphasia, encephalopathy, physical restraints); CKD raises suspected secondary hypertension against a trial premised on primary hypertension; coded subendocardial MI and left MCA embolic stroke bear on the recent-vascular-events exclusion. Clears Type 1 DM, contrast allergy, prior denervation, and the respiratory support exclusion (sleep apnea explicitly carved out).</x:v>
       </x:c>
     </x:row>
     <x:row r="841" ht="58" customHeight="1">
@@ -23658,7 +23658,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I841" s="9" t="str">
-        <x:v>Trial enrolls prostate cancer patients receiving radiation plus 6 months ADT. Patient has benign prostatic hyperplasia without obstruction — no malignancy, no prostatectomy, no radiation, no ADT, no PSA in his lab panel. Meets male and age criteria (79, exactly at the 30–79 ceiling). Independently excluded by poorly controlled diabetes ("NIDDM UNCONTROLLED," glucose 49–1000, HbA1c 6.7–11.5) and by inability to undergo time-restricted eating given enteral tube feeding after aspiration pneumonitis. ECOG would be 4 (bilateral hemiplegia, restraints, palliative care) against required 0–2; aphasia bars the language and app-based food diary requirements. Clears GLP1-RA contraindications — CKD is not end-stage.</x:v>
+        <x:v>Trial enrolls prostate cancer patients receiving radiation plus 6 months ADT. Patient has benign prostatic hyperplasia without obstruction, no malignancy, no prostatectomy, no radiation, no ADT, no PSA in his lab panel. Meets male and age criteria (79, exactly at the 30–79 ceiling). Independently excluded by poorly controlled diabetes ("NIDDM UNCONTROLLED," glucose 49–1000, HbA1c 6.7–11.5) and by inability to undergo time-restricted eating given enteral tube feeding after aspiration pneumonitis. ECOG would be 4 (bilateral hemiplegia, restraints, palliative care) against required 0–2; aphasia bars the language and app-based food diary requirements. Clears GLP1-RA contraindications, CKD is not end-stage.</x:v>
       </x:c>
     </x:row>
     <x:row r="842" ht="58" customHeight="1">
@@ -23685,7 +23685,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I842" s="9" t="str">
-        <x:v>Strong fit for cardiorenal syndrome population: heart failure (NTproBNP 3062) with CKD from diabetic nephropathy ("NIDDM W/RENAL MANIF"), plus secondary pulmonary hypertension. eGFR clears the ≥15 floor comfortably (creatinine 0.7–1.4 at 74F). Intact consent capacity — no cognitive impairment. All stated exclusions absent: no hepatorenal syndrome (LFTs normal), no kidney malformation, not pregnant, potassium 3.8–4.5 clears the visit-2 hypokalemia floor. Medium confidence pending two items: loop diuretic dose ≥40 mg/day furosemide is undocumented but clinically near-certain, and MRI feasibility needs checking given left knee prosthesis, right femoral IM hardware, and BMI 40.0–44.9 — hardware is distal to the imaging field and likely MR-conditional. Recent femoral and periprosthetic fractures with Hgb nadir 5.8 affect visit timing, not eligibility. NOTE: trial's exclusion_criteria array is empty in source.</x:v>
+        <x:v>Strong fit for cardiorenal syndrome population: heart failure (NTproBNP 3062) with CKD from diabetic nephropathy ("NIDDM W/RENAL MANIF"), plus secondary pulmonary hypertension. eGFR clears the ≥15 floor comfortably (creatinine 0.7–1.4 at 74F). Intact consent capacity, no cognitive impairment. All stated exclusions absent: no hepatorenal syndrome (LFTs normal), no kidney malformation, not pregnant, potassium 3.8–4.5 clears the visit-2 hypokalemia floor. Medium confidence pending two items: loop diuretic dose ≥40 mg/day furosemide is undocumented but clinically near-certain, and MRI feasibility needs checking given left knee prosthesis, right femoral IM hardware, and BMI 40.0–44.9, hardware is distal to the imaging field and likely MR-conditional. Recent femoral and periprosthetic fractures with Hgb nadir 5.8 affect visit timing, not eligibility. NOTE: trial's exclusion_criteria array is empty in source.</x:v>
       </x:c>
     </x:row>
     <x:row r="843" ht="58" customHeight="1">
@@ -23714,7 +23714,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I843" s="9" t="str">
-        <x:v>Has the chronic substrate — heart failure (NTproBNP 3062) with CKD from diabetic nephropathy — but not the acute state the trial requires. Protocol enrolls hypervolemic patients admitted with acutely decompensated HF and diuretic resistance; her record codes dehydration and iatrogenic hypotension, indicating volume depletion, and her admission narrative is orthopedic/infectious (open femoral fracture with ORIF, acute posthemorrhagic anemia Hgb nadir 5.8, E. coli and Klebsiella UTI). Recurrent urinary infection engages the SGLT2i genitourinary infection exclusion. Severe anemia plus hypotension raise the general safety exclusion. Clears type 1 DM, DKA, liver disease, dialysis, and GI absorption exclusions; protocol explicitly permits acute creatinine rise.</x:v>
+        <x:v>Has the chronic substrate, heart failure (NTproBNP 3062) with CKD from diabetic nephropathy, but not the acute state the trial requires. Protocol enrolls hypervolemic patients admitted with acutely decompensated HF and diuretic resistance; her record codes dehydration and iatrogenic hypotension, indicating volume depletion, and her admission narrative is orthopedic/infectious (open femoral fracture with ORIF, acute posthemorrhagic anemia Hgb nadir 5.8, E. coli and Klebsiella UTI). Recurrent urinary infection engages the SGLT2i genitourinary infection exclusion. Severe anemia plus hypotension raise the general safety exclusion. Clears type 1 DM, DKA, liver disease, dialysis, and GI absorption exclusions; protocol explicitly permits acute creatinine rise.</x:v>
       </x:c>
     </x:row>
     <x:row r="844" ht="58" customHeight="1">
@@ -23741,7 +23741,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I844" s="9" t="str">
-        <x:v>Pro-BNP criterion met affirmatively — NTproBNP 3062 ng/L against a &gt;800 threshold, ~3.8x margin, satisfying the elevated_bnp required signal; more significant still given BMI 40.0–44.9, since obesity suppresses natriuretic peptides. Age and consent capacity clear (no cognitive impairment; MDD documented but not capacity-impairing). Sole exclusion is investigator discretion, and the intervention is non-invasive ultrasound with no drug — so her anemia (Hgb nadir 5.8), UTI, and recent femoral ORIF weigh far less than they did against empagliflozin in PAIR-000894. Open item: whether admission carried a clinical ADHF diagnosis, since the dominant narrative is fall with open femoral fracture; postoperative decompensation is plausible given hypoxemia, pulmonary collapse, atelectasis, and the coded dehydration/iatrogenic hypotension may reflect over-diuresis.</x:v>
+        <x:v>Pro-BNP criterion met affirmatively, NTproBNP 3062 ng/L against a &gt;800 threshold, ~3.8x margin, satisfying the elevated_bnp required signal; more significant still given BMI 40.0–44.9, since obesity suppresses natriuretic peptides. Age and consent capacity clear (no cognitive impairment; MDD documented but not capacity-impairing). Sole exclusion is investigator discretion, and the intervention is non-invasive ultrasound with no drug, so her anemia (Hgb nadir 5.8), UTI, and recent femoral ORIF weigh far less than they did against empagliflozin in PAIR-000894. Open item: whether admission carried a clinical ADHF diagnosis, since the dominant narrative is fall with open femoral fracture; postoperative decompensation is plausible given hypoxemia, pulmonary collapse, atelectasis, and the coded dehydration/iatrogenic hypotension may reflect over-diuresis.</x:v>
       </x:c>
     </x:row>
     <x:row r="845" ht="58" customHeight="1">
@@ -23770,7 +23770,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I845" s="9" t="str">
-        <x:v>Closed-cohort follow-up study — eligibility is membership in the STONE cohort of 4,094 Shanghai residents recruited 2016–2017, not clinical characteristics. She is not a member and cannot become one; the qualifying baseline assessment window closed eight years ago, so no screening can establish eligibility. Both exclusions (moved away, lost to contact) presuppose membership and are inapplicable. Note the disease fit is otherwise excellent — she has cardiovascular, kidney, metabolic, thyroid, and bone-metabolism disease, covering nearly the trial's full registered condition list — which is precisely why a clinically-driven matcher would rank this pairing highly.</x:v>
+        <x:v>Closed-cohort follow-up study, eligibility is membership in the STONE cohort of 4,094 Shanghai residents recruited 2016–2017, not clinical characteristics. She is not a member and cannot become one; the qualifying baseline assessment window closed eight years ago, so no screening can establish eligibility. Both exclusions (moved away, lost to contact) presuppose membership and are inapplicable. Note the disease fit is otherwise excellent, she has cardiovascular, kidney, metabolic, thyroid, and bone-metabolism disease, covering nearly the trial's full registered condition list, which is precisely why a clinically-driven matcher would rank this pairing highly.</x:v>
       </x:c>
     </x:row>
     <x:row r="846" ht="58" customHeight="1">
@@ -23799,7 +23799,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I846" s="9" t="str">
-        <x:v>Excellent disease and demographic fit — CHF with NTproBNP 3062 plus CKD from diabetic nephropathy, age 74 inside the 18–75 window, and all three HF subtypes accepted so the missing EF is not a barrier. Fails on current state: trial requires STABLE chronic HF, and she is an acutely ill inpatient (open femoral fracture with ORIF, acute posthemorrhagic anemia Hgb nadir 5.8, dehydration, iatrogenic hypotension). Active infectious disease at enrollment explicitly excluded and affirmatively coded (UTI, E. coli, Klebsiella) — also confounding, since the five study biomarkers are inflammatory and complement mediators. Creatinine 0.7–1.4 with hyaline casts raises the AKI-within-3-months exclusion; breast cancer history bears on the high-priority 5-year oncologic exclusion, timing unknown. Clears dialysis/kidney surgery, autoimmune disease (gout is not autoimmune), liver dysfunction, and consent capacity. Time-limited rather than categorical — revisit after recovery, but note the 75-year ceiling.</x:v>
+        <x:v>Excellent disease and demographic fit, CHF with NTproBNP 3062 plus CKD from diabetic nephropathy, age 74 inside the 18–75 window, and all three HF subtypes accepted so the missing EF is not a barrier. Fails on current state: trial requires STABLE chronic HF, and she is an acutely ill inpatient (open femoral fracture with ORIF, acute posthemorrhagic anemia Hgb nadir 5.8, dehydration, iatrogenic hypotension). Active infectious disease at enrollment explicitly excluded and affirmatively coded (UTI, E. coli, Klebsiella), also confounding, since the five study biomarkers are inflammatory and complement mediators. Creatinine 0.7–1.4 with hyaline casts raises the AKI-within-3-months exclusion; breast cancer history bears on the high-priority 5-year oncologic exclusion, timing unknown. Clears dialysis/kidney surgery, autoimmune disease (gout is not autoimmune), liver dysfunction, and consent capacity. Time-limited rather than categorical, revisit after recovery, but note the 75-year ceiling.</x:v>
       </x:c>
     </x:row>
     <x:row r="847" ht="58" customHeight="1">
@@ -23828,7 +23828,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I847" s="9" t="str">
-        <x:v>Meets age 18–75 (74) and the renal criterion (eGFR &lt;90 across her full creatinine range of 0.7–1.4). Fails on two affirmatively documented exclusions. Severe anemia: Hgb 5.8–11.5, Hct 19–35.2, acute posthemorrhagic anemia coded — unsafe for aerobic training. Osteoarticular disease impeding rehabilitation: open femoral fracture, right femoral shaft fracture, periprosthetic fracture around right knee prosthesis, left knee prosthesis, three femoral fixation procedures — against an intervention of brisk walking and cycling 3x weekly for 6 months. Also fails "low risk in exercise risk assessment" and "chronically stable"; MDD triggers the unqualified mental illness exclusion; hypothyroidism and pulmonary findings raise two further exclusions. HFrEF unconfirmed — no EF in record, and this trial requires reduced EF specifically. Aortic valve disorders unspecified; if moderate stenosis, independently exclusionary.</x:v>
+        <x:v>Meets age 18–75 (74) and the renal criterion (eGFR &lt;90 across her full creatinine range of 0.7–1.4). Fails on two affirmatively documented exclusions. Severe anemia: Hgb 5.8–11.5, Hct 19–35.2, acute posthemorrhagic anemia coded, unsafe for aerobic training. Osteoarticular disease impeding rehabilitation: open femoral fracture, right femoral shaft fracture, periprosthetic fracture around right knee prosthesis, left knee prosthesis, three femoral fixation procedures, against an intervention of brisk walking and cycling 3x weekly for 6 months. Also fails "low risk in exercise risk assessment" and "chronically stable"; MDD triggers the unqualified mental illness exclusion; hypothyroidism and pulmonary findings raise two further exclusions. HFrEF unconfirmed, no EF in record, and this trial requires reduced EF specifically. Aortic valve disorders unspecified; if moderate stenosis, independently exclusionary.</x:v>
       </x:c>
     </x:row>
     <x:row r="848" ht="58" customHeight="1">
@@ -23857,7 +23857,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I848" s="9" t="str">
-        <x:v>Postmortem molecular autopsy study — index case must be a DECEASED person aged birth–45 whose death was sudden and unexplained, enrolled via the medical examiner's office with family sequencing. Patient is alive (44 procedures, 281 creatinine draws, active inpatient record), age 70, and his condition is exhaustively explained (AML with allogeneic stem cell transplant, GVHD, severe sepsis, aspergillosis, VAP, respiratory failure). Also triggers the high-priority open-heart-surgery exclusion: 4+ vessel CABG with internal mammary graft and extracorporeal circulation. Further hits: prior MI, severe pulmonary disease, death attributable to chronic comorbidity. Notably clears morbid obesity (BMI coded 19–24, with cachexia), illicit drug use, alcohol abuse, HCM, and prior CVA.</x:v>
+        <x:v>Postmortem molecular autopsy study, index case must be a DECEASED person aged birth–45 whose death was sudden and unexplained, enrolled via the medical examiner's office with family sequencing. Patient is alive (44 procedures, 281 creatinine draws, active inpatient record), age 70, and his condition is exhaustively explained (AML with allogeneic stem cell transplant, GVHD, severe sepsis, aspergillosis, VAP, respiratory failure). Also triggers the high-priority open-heart-surgery exclusion: 4+ vessel CABG with internal mammary graft and extracorporeal circulation. Further hits: prior MI, severe pulmonary disease, death attributable to chronic comorbidity. Notably clears morbid obesity (BMI coded 19–24, with cachexia), illicit drug use, alcohol abuse, HCM, and prior CVA.</x:v>
       </x:c>
     </x:row>
     <x:row r="849" ht="58" customHeight="1">
@@ -23886,7 +23886,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I849" s="9" t="str">
-        <x:v>Strongest CAD inclusion fit in the review — satisfies all three routes (angiography with chronic total occlusion, MI history, and 4+ vessel CABG with IMA graft), plus age 70 in the 60–85 window and male sex. Fails on everything else. Not "stable CAD on optimal medical therapy": severe sepsis, acute respiratory failure, VAP, Pseudomonas pneumonia, aspergillosis, with Hgb 5.1–12.9, platelets 5–517, WBC 0.1–34.7, albumin 1.4–4.7. Cannot consent — toxic encephalopathy, semicoma/stupor, delirium, physical restraints. "Other relevant ongoing or recurrent illness" triggered by AML, allogeneic stem cell transplant, GVHD, MDS, pancytopenia. Inspiratory muscle testing unperformable with tracheostomy, prolonged mechanical ventilation, and interstitial pulmonary disease. Intermediate coronary syndrome (unstable angina) also coded. Possible testosterone replacement (testicular hypofunction, hormone panel) triggers the HRT exclusion.</x:v>
+        <x:v>Strongest CAD inclusion fit in the review, satisfies all three routes (angiography with chronic total occlusion, MI history, and 4+ vessel CABG with IMA graft), plus age 70 in the 60–85 window and male sex. Fails on everything else. Not "stable CAD on optimal medical therapy": severe sepsis, acute respiratory failure, VAP, Pseudomonas pneumonia, aspergillosis, with Hgb 5.1–12.9, platelets 5–517, WBC 0.1–34.7, albumin 1.4–4.7. Cannot consent, toxic encephalopathy, semicoma/stupor, delirium, physical restraints. "Other relevant ongoing or recurrent illness" triggered by AML, allogeneic stem cell transplant, GVHD, MDS, pancytopenia. Inspiratory muscle testing unperformable with tracheostomy, prolonged mechanical ventilation, and interstitial pulmonary disease. Intermediate coronary syndrome (unstable angina) also coded. Possible testosterone replacement (testicular hypofunction, hormone panel) triggers the HRT exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="850" ht="58" customHeight="1">
@@ -23915,7 +23915,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I850" s="9" t="str">
-        <x:v>Trial randomizes next diagnostic step for patients with newly identified obstructive CAD on CCTA; explicitly excludes "known CAD with previous MI, PCI, CABG." Patient hits both limbs — documented myocardial infarction and aortocoronary bypass of 4+ vessels with IMA graft plus extracorporeal circulation. No CCTA in his record; coronary anatomy characterized invasively. Four-vessel bypass and chronic total occlusion also suggest high-risk anatomy, separately excluded. Non-cardiac comorbidity exclusion triggered by AML, allogeneic stem cell transplant, GVHD, severe sepsis, aspergillosis, respiratory failure. Cannot verbally confirm understanding — toxic encephalopathy, semicoma/stupor, restraints, tracheostomy. Clears aspirin/clopidogrel/heparin tolerance and contrast anaphylaxis.</x:v>
+        <x:v>Trial randomizes next diagnostic step for patients with newly identified obstructive CAD on CCTA; explicitly excludes "known CAD with previous MI, PCI, CABG." Patient hits both limbs, documented myocardial infarction and aortocoronary bypass of 4+ vessels with IMA graft plus extracorporeal circulation. No CCTA in his record; coronary anatomy characterized invasively. Four-vessel bypass and chronic total occlusion also suggest high-risk anatomy, separately excluded. Non-cardiac comorbidity exclusion triggered by AML, allogeneic stem cell transplant, GVHD, severe sepsis, aspergillosis, respiratory failure. Cannot verbally confirm understanding, toxic encephalopathy, semicoma/stupor, restraints, tracheostomy. Clears aspirin/clopidogrel/heparin tolerance and contrast anaphylaxis.</x:v>
       </x:c>
     </x:row>
     <x:row r="851" ht="58" customHeight="1">
@@ -23944,7 +23944,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I851" s="9" t="str">
-        <x:v>Ischemic HF inclusion met three ways (MI, 4+ vessel CABG, coronary arteriography) plus age ≥45. Excluded by explicitly named prohibited concomitant drugs: cyclosporin appears as a monitored lab analyte (calcineurin inhibitor post allogeneic SCT with GVHD), and documented aspergillosis implies azole antifungal therapy. Both are CYP3A4/P-gp inhibitors — colchicine co-administration risks fatal toxicity. Also excluded by active malignancy: AML coded as not having achieved remission, blasts 1–38%, on chemotherapy, life expectancy &lt;2 years. Fails the ambulatory/stable-hospitalized requirement — mechanically ventilated ≥96h via tracheostomy with severe sepsis, no discharge in 72h. "Examination of participant in clinical trial" coded, raising the concurrent-experimental-agent exclusion. Clears eGFR (creatinine 0.1–1.5), cirrhosis, VAD/transplant, valvular disease.</x:v>
+        <x:v>Ischemic HF inclusion met three ways (MI, 4+ vessel CABG, coronary arteriography) plus age ≥45. Excluded by explicitly named prohibited concomitant drugs: cyclosporin appears as a monitored lab analyte (calcineurin inhibitor post allogeneic SCT with GVHD), and documented aspergillosis implies azole antifungal therapy. Both are CYP3A4/P-gp inhibitors, colchicine co-administration risks fatal toxicity. Also excluded by active malignancy: AML coded as not having achieved remission, blasts 1–38%, on chemotherapy, life expectancy &lt;2 years. Fails the ambulatory/stable-hospitalized requirement, mechanically ventilated ≥96h via tracheostomy with severe sepsis, no discharge in 72h. "Examination of participant in clinical trial" coded, raising the concurrent-experimental-agent exclusion. Clears eGFR (creatinine 0.1–1.5), cirrhosis, VAD/transplant, valvular disease.</x:v>
       </x:c>
     </x:row>
     <x:row r="852" ht="58" customHeight="1">
@@ -23973,7 +23973,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I852" s="9" t="str">
-        <x:v>Trial enrolls clear cell RCC with IVC tumor thrombus for neoadjuvant pembrolizumab/axitinib before nephrectomy. Patient has no renal malignancy — his cancer is AML with MDS, post allogeneic stem cell transplant. Also excluded by: additional active malignancy requiring treatment (AML not in remission, blasts 1–38%); immunodeficiency and immunosuppression (hypogammaglobulinemia, long-term steroids, cyclosporin levels) — a contraindication to checkpoint inhibition in a GVHD patient; active bleeding disorder (platelets nadir 5 K/uL, Hgb 5.1, pancytopenia) against a VEGF inhibitor; strong CYP3A4 inhibitors (cyclosporine, azoles for aspergillosis); ALT to 157 and AST to 131 exceeding 3× ULN; likely non-infectious pneumonitis (interstitial pulmonary disease). Requires ECOG 0 — he is ECOG 4 (semicoma, ventilated, restrained). Clears prior solid organ transplant (his was hematopoietic) and prior anti-PD-1/VEGF therapy.</x:v>
+        <x:v>Trial enrolls clear cell RCC with IVC tumor thrombus for neoadjuvant pembrolizumab/axitinib before nephrectomy. Patient has no renal malignancy, his cancer is AML with MDS, post allogeneic stem cell transplant. Also excluded by: additional active malignancy requiring treatment (AML not in remission, blasts 1–38%); immunodeficiency and immunosuppression (hypogammaglobulinemia, long-term steroids, cyclosporin levels), a contraindication to checkpoint inhibition in a GVHD patient; active bleeding disorder (platelets nadir 5 K/uL, Hgb 5.1, pancytopenia) against a VEGF inhibitor; strong CYP3A4 inhibitors (cyclosporine, azoles for aspergillosis); ALT to 157 and AST to 131 exceeding 3× ULN; likely non-infectious pneumonitis (interstitial pulmonary disease). Requires ECOG 0, he is ECOG 4 (semicoma, ventilated, restrained). Clears prior solid organ transplant (his was hematopoietic) and prior anti-PD-1/VEGF therapy.</x:v>
       </x:c>
     </x:row>
     <x:row r="853" ht="58" customHeight="1">
@@ -24002,7 +24002,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I853" s="9" t="str">
-        <x:v>Perioperative trial randomizing angiotensin II vs norepinephrine during cardiac surgery with CPB. Patient has historical 4+ vessel CABG with extracorporeal circulation but no current or planned operation, and redo cardiac surgery is not plausible — AML not in remission, GVHD post allogeneic SCT, severe sepsis, aspergillosis, tracheostomy with prolonged ventilation, cachexia, platelet nadir 5 K/uL. Updated procedure rule does not apply: barriers are independent and permanent. Cannot consent (toxic encephalopathy, semicoma, restraints). Likely already on vasopressor support — an explicit exclusion — given severe sepsis, hypovolemia, and arterial line. Probable pre-existing AKI (creatinine 0.1–1.5, granular casts 3/lpf, nephrotoxic exposure via vancomycin/tobramycin levels). AKI risk score computes to 4 (Hgb &lt;130 g/L = 2, creatinine &gt;1 = 2; age exactly 70 not &gt;70 = 0; BMI 19–24 = 0), short of the ≥5 threshold unless NYHA 4 applies. Clears eGFR &lt;20, dialysis, pulmonary hypertension, and the excluded surgery types.</x:v>
+        <x:v>Perioperative trial randomizing angiotensin II vs norepinephrine during cardiac surgery with CPB. Patient has historical 4+ vessel CABG with extracorporeal circulation but no current or planned operation, and redo cardiac surgery is not plausible, AML not in remission, GVHD post allogeneic SCT, severe sepsis, aspergillosis, tracheostomy with prolonged ventilation, cachexia, platelet nadir 5 K/uL. Updated procedure rule does not apply: barriers are independent and permanent. Cannot consent (toxic encephalopathy, semicoma, restraints). Likely already on vasopressor support, an explicit exclusion, given severe sepsis, hypovolemia, and arterial line. Probable pre-existing AKI (creatinine 0.1–1.5, granular casts 3/lpf, nephrotoxic exposure via vancomycin/tobramycin levels). AKI risk score computes to 4 (Hgb &lt;130 g/L = 2, creatinine &gt;1 = 2; age exactly 70 not &gt;70 = 0; BMI 19–24 = 0), short of the ≥5 threshold unless NYHA 4 applies. Clears eGFR &lt;20, dialysis, pulmonary hypertension, and the excluded surgery types.</x:v>
       </x:c>
     </x:row>
     <x:row r="854" ht="58" customHeight="1">
@@ -24031,7 +24031,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I854" s="9" t="str">
-        <x:v>Smartphone-delivered secondary prevention app for post-CABG/PCI patients. CABG history and hypertension fit, but likely fails the conjunctive comorbidity requirement — HbA1c 5.6–6.1% is below diabetic range with no diabetes diagnosis coded, and no dyslipidemia diagnosis despite measured LDL 113–151. Cannot satisfy the explicit "use of a smartphone" inclusion: toxic encephalopathy, semicoma/stupor, delirium, physical restraints, tracheostomy with ≥96h mechanical ventilation. Three exclusions hit affirmatively — history of heart failure (clinical tag, NTproBNP 90–826) and cardiac dysrhythmias; severe underlying condition (AML not in remission, blasts 1–38%, post allogeneic SCT); and cognitive/communication impairment with limitations in daily activities.</x:v>
+        <x:v>Smartphone-delivered secondary prevention app for post-CABG/PCI patients. CABG history and hypertension fit, but likely fails the conjunctive comorbidity requirement, HbA1c 5.6–6.1% is below diabetic range with no diabetes diagnosis coded, and no dyslipidemia diagnosis despite measured LDL 113–151. Cannot satisfy the explicit "use of a smartphone" inclusion: toxic encephalopathy, semicoma/stupor, delirium, physical restraints, tracheostomy with ≥96h mechanical ventilation. Three exclusions hit affirmatively, history of heart failure (clinical tag, NTproBNP 90–826) and cardiac dysrhythmias; severe underlying condition (AML not in remission, blasts 1–38%, post allogeneic SCT); and cognitive/communication impairment with limitations in daily activities.</x:v>
       </x:c>
     </x:row>
     <x:row r="855" ht="58" customHeight="1">
@@ -24060,7 +24060,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I855" s="9" t="str">
-        <x:v>Trial studies coronary microvascular disease, requiring normal epicardial arteries or stenosis &lt;20%. Patient has chronic total occlusion (100% stenosis), atherosclerotic native coronary disease, and 4+ vessel CABG — the anatomic opposite, and the condition microvascular angina is diagnosed by excluding. Also affirmatively excluded by previous MI and CABG (both limbs), and by history of heart failure (high-priority, clinical tag with NTproBNP 90–826). Probable hepatic/renal dysfunction exclusion (ALT to 157, AST to 131, albumin 1.4, granular casts). CAD coded "without angina pectoris," working against the anginal inclusion criterion. Notably this protocol permits guardian consent, so his encephalopathy would not have been the barrier.</x:v>
+        <x:v>Trial studies coronary microvascular disease, requiring normal epicardial arteries or stenosis &lt;20%. Patient has chronic total occlusion (100% stenosis), atherosclerotic native coronary disease, and 4+ vessel CABG, the anatomic opposite, and the condition microvascular angina is diagnosed by excluding. Also affirmatively excluded by previous MI and CABG (both limbs), and by history of heart failure (high-priority, clinical tag with NTproBNP 90–826). Probable hepatic/renal dysfunction exclusion (ALT to 157, AST to 131, albumin 1.4, granular casts). CAD coded "without angina pectoris," working against the anginal inclusion criterion. Notably this protocol permits guardian consent, so his encephalopathy would not have been the barrier.</x:v>
       </x:c>
     </x:row>
     <x:row r="856" ht="58" customHeight="1">
@@ -24089,7 +24089,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I856" s="9" t="str">
-        <x:v>Trial recruits patients undergoing CCTA for SUSPECTED stable CAD; excludes known CAD via prior MI, PCI, CABG, or ≥50% angiographic lesion. Patient hits three limbs — MI tag, 4+ vessel CABG with IMA graft, and chronic total occlusion (100% stenosis) documented on coronary arteriography. Also fails age: criterion is 30 to &lt;70 and he is exactly 70 (registry structured fields show no maximum, so a matcher reading structured data would miss this). Not undergoing CCTA; unable to provide written consent (toxic encephalopathy, semicoma, restraints, tracheostomy). Pulmonary conditions capable of explaining symptoms (interstitial lung disease, VAP, aspergillosis, respiratory failure) engage the significant-condition exclusion. Swedish social security requirement treated as logistical, not weighted.</x:v>
+        <x:v>Trial recruits patients undergoing CCTA for SUSPECTED stable CAD; excludes known CAD via prior MI, PCI, CABG, or ≥50% angiographic lesion. Patient hits three limbs, MI tag, 4+ vessel CABG with IMA graft, and chronic total occlusion (100% stenosis) documented on coronary arteriography. Also fails age: criterion is 30 to &lt;70 and he is exactly 70 (registry structured fields show no maximum, so a matcher reading structured data would miss this). Not undergoing CCTA; unable to provide written consent (toxic encephalopathy, semicoma, restraints, tracheostomy). Pulmonary conditions capable of explaining symptoms (interstitial lung disease, VAP, aspergillosis, respiratory failure) engage the significant-condition exclusion. Swedish social security requirement treated as logistical, not weighted.</x:v>
       </x:c>
     </x:row>
     <x:row r="857" ht="58" customHeight="1">
@@ -24118,7 +24118,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I857" s="9" t="str">
-        <x:v>AI scoring of surgeon technique during IMA-to-LAD anastomosis; requires a patient undergoing first-time isolated CABG, with intraoperative video as the data source. Patient has already had single internal mammary-coronary artery bypass within a 4+ vessel CABG with extracorporeal circulation — first-time status is permanently unattainable, and a redo is a different operation. No current or planned surgery, and redo bypass is not feasible given AML not in remission, GVHD, severe sepsis, ventilator dependence via tracheostomy, and platelet nadir 5 K/uL. Also affirmatively excluded by transaminases &gt;3× ULN (ALT to 157, AST to 131). Cannot provide written consent (toxic encephalopathy, semicoma, restraints). Clears contrast/angiography contraindications.</x:v>
+        <x:v>AI scoring of surgeon technique during IMA-to-LAD anastomosis; requires a patient undergoing first-time isolated CABG, with intraoperative video as the data source. Patient has already had single internal mammary-coronary artery bypass within a 4+ vessel CABG with extracorporeal circulation, first-time status is permanently unattainable, and a redo is a different operation. No current or planned surgery, and redo bypass is not feasible given AML not in remission, GVHD, severe sepsis, ventilator dependence via tracheostomy, and platelet nadir 5 K/uL. Also affirmatively excluded by transaminases &gt;3× ULN (ALT to 157, AST to 131). Cannot provide written consent (toxic encephalopathy, semicoma, restraints). Clears contrast/angiography contraindications.</x:v>
       </x:c>
     </x:row>
     <x:row r="858" ht="58" customHeight="1">
@@ -24147,7 +24147,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I858" s="9" t="str">
-        <x:v>Meets age 45–75 (70) and the IHD criteria (MI tag, intermediate coronary syndrome, CABG). Fails on exclusions that are affirmatively documented: chemotherapy for cancer within 2 years (AML, chemo infusion, allogeneic SCT); ICU hospitalisation within 6 months for non-ischaemic reasons (≥96h invasive ventilation, tracheostomy, arterial line, sepsis); interstitial pulmonary disease with respiratory insufficiency; and medical contraindication to exercise. Cannot meet NYHA I–II or "no physical limitations for exercise" — semicoma, ventilator, restraints, cachexia, platelets nadir 5, Hgb nadir 5.1. Spanish speaking fluency impossible with tracheostomy and encephalopathy. Clears eGFR &lt;30, BMI ≥40 (coded 19–24), uncontrolled diabetes (HbA1c 5.6–6.1), and implantable devices (temporary pacing wires only, discontinued).</x:v>
+        <x:v>Meets age 45–75 (70) and the IHD criteria (MI tag, intermediate coronary syndrome, CABG). Fails on exclusions that are affirmatively documented: chemotherapy for cancer within 2 years (AML, chemo infusion, allogeneic SCT); ICU hospitalisation within 6 months for non-ischaemic reasons (≥96h invasive ventilation, tracheostomy, arterial line, sepsis); interstitial pulmonary disease with respiratory insufficiency; and medical contraindication to exercise. Cannot meet NYHA I–II or "no physical limitations for exercise", semicoma, ventilator, restraints, cachexia, platelets nadir 5, Hgb nadir 5.1. Spanish speaking fluency impossible with tracheostomy and encephalopathy. Clears eGFR &lt;30, BMI ≥40 (coded 19–24), uncontrolled diabetes (HbA1c 5.6–6.1), and implantable devices (temporary pacing wires only, discontinued).</x:v>
       </x:c>
     </x:row>
     <x:row r="859" ht="58" customHeight="1">
@@ -24176,7 +24176,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I859" s="9" t="str">
-        <x:v>Genuine disease and demographic fit — "Insomnia, unspecified" is documented (the trial's actual target condition) and age 70 falls inside the older adults band of 65–75. Fails on the group's sole requirement, freedom from cognitive or mental health disorders: toxic encephalopathy, semicoma/stupor, delirium, physical restraints, plus anxiety state, anxiety disorder, depressive disorder, and major depressive disorder. Also excluded by respiratory disease preventing exercise — interstitial pulmonary disease, acute respiratory failure, VAP, Pseudomonas and aspergillosis pneumonia, tracheostomy with ≥96h invasive ventilation; spirometry and cardiorespiratory fitness testing both unperformable. All four other enrolment groups require ages 18–35. Contrast with PAIR-000890, where the same trial failed on age (79).</x:v>
+        <x:v>Genuine disease and demographic fit, "Insomnia, unspecified" is documented (the trial's actual target condition) and age 70 falls inside the older adults band of 65–75. Fails on the group's sole requirement, freedom from cognitive or mental health disorders: toxic encephalopathy, semicoma/stupor, delirium, physical restraints, plus anxiety state, anxiety disorder, depressive disorder, and major depressive disorder. Also excluded by respiratory disease preventing exercise, interstitial pulmonary disease, acute respiratory failure, VAP, Pseudomonas and aspergillosis pneumonia, tracheostomy with ≥96h invasive ventilation; spirometry and cardiorespiratory fitness testing both unperformable. All four other enrolment groups require ages 18–35. Contrast with PAIR-000890, where the same trial failed on age (79).</x:v>
       </x:c>
     </x:row>
     <x:row r="860" ht="58" customHeight="1">
@@ -24205,7 +24205,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I860" s="9" t="str">
-        <x:v>Trial enrols hypertrophic cardiomyopathy phenotypes (sarcomeric, non-sarcomeric, Fabry, amyloid), plus first-degree relatives and mutation carriers. Patient has no cardiomyopathy of any kind coded, no LVH or outflow findings on his echocardiogram, no family history, no genetic testing — all three inclusion routes fail. Also triggers the trial's SOLE exclusion on all three limbs: prior MI (clinical tag, intermediate coronary syndrome), prior revascularization (4+ vessel CABG with IMA graft), and coronary stenosis ≥50% (chronic total occlusion on invasive arteriography). Cannot provide written consent (toxic encephalopathy, semicoma, restraints, tracheostomy).</x:v>
+        <x:v>Trial enrols hypertrophic cardiomyopathy phenotypes (sarcomeric, non-sarcomeric, Fabry, amyloid), plus first-degree relatives and mutation carriers. Patient has no cardiomyopathy of any kind coded, no LVH or outflow findings on his echocardiogram, no family history, no genetic testing, all three inclusion routes fail. Also triggers the trial's SOLE exclusion on all three limbs: prior MI (clinical tag, intermediate coronary syndrome), prior revascularization (4+ vessel CABG with IMA graft), and coronary stenosis ≥50% (chronic total occlusion on invasive arteriography). Cannot provide written consent (toxic encephalopathy, semicoma, restraints, tracheostomy).</x:v>
       </x:c>
     </x:row>
     <x:row r="861" ht="58" customHeight="1">
@@ -24234,7 +24234,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I861" s="9" t="str">
-        <x:v>Fails on enrolment timing: study captures prehospital scene data by HEMS crews, and his record carries subsequent-encounter codes for both the MVC and the subdural haemorrhage, with a completed course of 24–96h invasive ventilation followed by extubation and enteral feeding. Scene data cannot be collected retrospectively. No HEMS transport documented. Medium confidence — the barrier is temporal rather than clinical, and the exact interval since injury is not determinable from the record. Long-term anticoagulation (INR 1.1–1.7, PTT to 130.1) is clinically relevant to his bleeding but not an eligibility factor here.</x:v>
+        <x:v>Fails on enrolment timing: study captures prehospital scene data by HEMS crews, and his record carries subsequent-encounter codes for both the MVC and the subdural haemorrhage, with a completed course of 24–96h invasive ventilation followed by extubation and enteral feeding. Scene data cannot be collected retrospectively. No HEMS transport documented. Medium confidence, the barrier is temporal rather than clinical, and the exact interval since injury is not determinable from the record. Long-term anticoagulation (INR 1.1–1.7, PTT to 130.1) is clinically relevant to his bleeding but not an eligibility factor here.</x:v>
       </x:c>
     </x:row>
     <x:row r="862" ht="58" customHeight="1">
@@ -24263,7 +24263,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I862" s="9" t="str">
-        <x:v>Trial enrols aneurysmal SAH confirmed by angiography and secured by clipping or coiling, within 72h of rupture. Patient's haemorrhages are explicitly TRAUMATIC (subarachnoid, subdural, and cerebral) following a motor vehicle collision — a distinct entity with no aneurysm, no angiography, and no securing procedure. His thoracic aortic aneurysm is unrelated to intracranial disease. Hunt-Hess grading is not applicable to traumatic bleeding. Also triggers the high-priority exclusion for SVT "including atrial fibrillation" — AF clinical tag with long-term anticoagulation and INR 1.1–1.7; mechanistically significant given documented bradycardia and a vagal-stimulation intervention. 72-hour window passed (subsequent-encounter codes, completed ventilation and extubation). Protocol permits LAR consent, so his aphasia and encephalopathy were not the barrier.</x:v>
+        <x:v>Trial enrols aneurysmal SAH confirmed by angiography and secured by clipping or coiling, within 72h of rupture. Patient's haemorrhages are explicitly TRAUMATIC (subarachnoid, subdural, and cerebral) following a motor vehicle collision, a distinct entity with no aneurysm, no angiography, and no securing procedure. His thoracic aortic aneurysm is unrelated to intracranial disease. Hunt-Hess grading is not applicable to traumatic bleeding. Also triggers the high-priority exclusion for SVT "including atrial fibrillation", AF clinical tag with long-term anticoagulation and INR 1.1–1.7; mechanistically significant given documented bradycardia and a vagal-stimulation intervention. 72-hour window passed (subsequent-encounter codes, completed ventilation and extubation). Protocol permits LAR consent, so his aphasia and encephalopathy were not the barrier.</x:v>
       </x:c>
     </x:row>
     <x:row r="863" ht="58" customHeight="1">
@@ -24292,7 +24292,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I863" s="9" t="str">
-        <x:v>Meets only the age criterion (80, floor of 40). Cannot consent or be MMSE-tested — toxic encephalopathy, aphasia, dysarthria/anarthria, other symbolic dysfunctions, physical restraints. Cellulitis of right upper limb triggers the high-priority open wounds/skin lesions exclusion, directly relevant to repeated water immersion. Recent major health change exclusion triggered by MVC trauma, traumatic cerebral/SAH/subdural haemorrhage, 24–96h invasive ventilation, pneumonia, aspiration pneumonitis. Unstable CVD exclusion triggered by cerebral infarction. Documented hypotension argues against the 115–159 mmHg SBP entry range. Protein-calorie malnutrition with albumin 2.4–3.9 fails weight stability. Likely on thyroid medication (hypothyroidism coded, TSH and T4 in panel), a named interfering class. Clears BMI &gt;40 (coded 22.0–22.9) and blood-draw tolerance (62 draws documented).</x:v>
+        <x:v>Meets only the age criterion (80, floor of 40). Cannot consent or be MMSE-tested, toxic encephalopathy, aphasia, dysarthria/anarthria, other symbolic dysfunctions, physical restraints. Cellulitis of right upper limb triggers the high-priority open wounds/skin lesions exclusion, directly relevant to repeated water immersion. Recent major health change exclusion triggered by MVC trauma, traumatic cerebral/SAH/subdural haemorrhage, 24–96h invasive ventilation, pneumonia, aspiration pneumonitis. Unstable CVD exclusion triggered by cerebral infarction. Documented hypotension argues against the 115–159 mmHg SBP entry range. Protein-calorie malnutrition with albumin 2.4–3.9 fails weight stability. Likely on thyroid medication (hypothyroidism coded, TSH and T4 in panel), a named interfering class. Clears BMI &gt;40 (coded 22.0–22.9) and blood-draw tolerance (62 draws documented).</x:v>
       </x:c>
     </x:row>
     <x:row r="864" ht="58" customHeight="1">
@@ -24321,7 +24321,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I864" s="9" t="str">
-        <x:v>Trial enrols comatose survivors of out-of-hospital cardiac arrest for individualized cerebral perfusion targeting, with neuron-specific enolase as the hypoxic-ischemic injury biomarker. No cardiac arrest or ROSC anywhere in the record — his brain injury is traumatic (cerebral, subarachnoid, and subdural haemorrhage after a motor vehicle collision), a different mechanism and pathology. Coma status itself ambiguous: toxic encephalopathy, aphasia, anarthria, restraints, but progressed to extubation. Also excluded by age — exactly 80 against a ≥80 exclusion. Registry structured age field reads min 21 with no maximum, so the ceiling is invisible to a matcher reading structured data (4th such instance in this review). No care limitations documented</x:v>
+        <x:v>Trial enrols comatose survivors of out-of-hospital cardiac arrest for individualized cerebral perfusion targeting, with neuron-specific enolase as the hypoxic-ischemic injury biomarker. No cardiac arrest or ROSC anywhere in the record, his brain injury is traumatic (cerebral, subarachnoid, and subdural haemorrhage after a motor vehicle collision), a different mechanism and pathology. Coma status itself ambiguous: toxic encephalopathy, aphasia, anarthria, restraints, but progressed to extubation. Also excluded by age, exactly 80 against a ≥80 exclusion. Registry structured age field reads min 21 with no maximum, so the ceiling is invisible to a matcher reading structured data (4th such instance in this review). No care limitations documented</x:v>
       </x:c>
     </x:row>
     <x:row r="865" ht="58" customHeight="1">
@@ -24350,7 +24350,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I865" s="9" t="str">
-        <x:v>Trial requires prevalent ESRD on maintenance thrice-weekly hemodialysis &gt;90 days. Patient carries a chronic_kidney_disease tag but creatinine is 0.7–1.5 mg/dL across 62 draws (eGFR roughly 45–95 at age 80M) with normal potassium and sodium — mild-to-moderate CKD, not end-stage. No dialysis, AV access, or renal replacement therapy among his ten procedures. Not a satisfiable prerequisite: the &gt;90-day maintenance requirement is a durable treatment state he does not need and could not reach near-term. Also excluded by inability to provide written informed consent — toxic encephalopathy, aphasia, dysarthria/anarthria, physical restraints after traumatic intracranial haemorrhage. Clears the haemoglobin floor (9.9–15.4) and pregnancy.</x:v>
+        <x:v>Trial requires prevalent ESRD on maintenance thrice-weekly hemodialysis &gt;90 days. Patient carries a chronic_kidney_disease tag but creatinine is 0.7–1.5 mg/dL across 62 draws (eGFR roughly 45–95 at age 80M) with normal potassium and sodium, mild-to-moderate CKD, not end-stage. No dialysis, AV access, or renal replacement therapy among his ten procedures. Not a satisfiable prerequisite: the &gt;90-day maintenance requirement is a durable treatment state he does not need and could not reach near-term. Also excluded by inability to provide written informed consent, toxic encephalopathy, aphasia, dysarthria/anarthria, physical restraints after traumatic intracranial haemorrhage. Clears the haemoglobin floor (9.9–15.4) and pregnancy.</x:v>
       </x:c>
     </x:row>
     <x:row r="866" ht="58" customHeight="1">
@@ -24379,7 +24379,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I866" s="9" t="str">
-        <x:v>Prevention trial for NEW-ONSET atrial fibrillation in critically ill ICU patients; excludes active AF at enrolment. Patient has established, treated AF — clinical tag plus long-term anticoagulants with INR 1.1–1.7 across 20 draws — so he cannot contribute to a new-onset endpoint. Meets the ICU entry route (invasive ventilation 24–96h for acute respiratory failure with hypoxia) and age. Also past the 18-hour enrolment window, with ventilation completed and extubation performed. Ventilation may have been for airway protection after isolated head trauma, which the protocol names as an exclusion example — his traumatic cerebral, subarachnoid, and subdural haemorrhages fit, though genuine respiratory pathology (pneumonia, aspiration pneumonitis, atelectasis) coexists. Not on dialysis, not palliative, not a cardiac surgery patient.</x:v>
+        <x:v>Prevention trial for NEW-ONSET atrial fibrillation in critically ill ICU patients; excludes active AF at enrolment. Patient has established, treated AF, clinical tag plus long-term anticoagulants with INR 1.1–1.7 across 20 draws, so he cannot contribute to a new-onset endpoint. Meets the ICU entry route (invasive ventilation 24–96h for acute respiratory failure with hypoxia) and age. Also past the 18-hour enrolment window, with ventilation completed and extubation performed. Ventilation may have been for airway protection after isolated head trauma, which the protocol names as an exclusion example, his traumatic cerebral, subarachnoid, and subdural haemorrhages fit, though genuine respiratory pathology (pneumonia, aspiration pneumonitis, atelectasis) coexists. Not on dialysis, not palliative, not a cardiac surgery patient.</x:v>
       </x:c>
     </x:row>
     <x:row r="867" ht="58" customHeight="1">
@@ -24408,7 +24408,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I867" s="9" t="str">
-        <x:v>Two-cohort MCG calibration study (healthy volunteers, chest pain patients); both arms specify ages 18–79 and he is 80, closing every route. Registry structured age field reads min 18 / no maximum — 5th instance in this review of a permissive structured field masking a stated ceiling. Fails healthy arm on cardiovascular history (AF, cerebral infarction, prior TIA, thoracic aortic aneurysm, hypertension) and on normal ECG requirement. Fails patient arm on absence of chest pain, angina, or ACS — no troponin in his panel. Multiple exclusions triggered: unresolved AF, hypothyroidism, acute respiratory illness with ventilation, abnormal liver function (ALT 23–276, AST 16–150), active infection (pneumonia, cellulitis, vancomycin level), trauma with physical disability, and inability to cooperate with MCG (aphasia, encephalopathy, restraints). Clears the BMI band (22.0–22.9 against &gt;30 or &lt;18).</x:v>
+        <x:v>Two-cohort MCG calibration study (healthy volunteers, chest pain patients); both arms specify ages 18–79 and he is 80, closing every route. Registry structured age field reads min 18 / no maximum, 5th instance in this review of a permissive structured field masking a stated ceiling. Fails healthy arm on cardiovascular history (AF, cerebral infarction, prior TIA, thoracic aortic aneurysm, hypertension) and on normal ECG requirement. Fails patient arm on absence of chest pain, angina, or ACS, no troponin in his panel. Multiple exclusions triggered: unresolved AF, hypothyroidism, acute respiratory illness with ventilation, abnormal liver function (ALT 23–276, AST 16–150), active infection (pneumonia, cellulitis, vancomycin level), trauma with physical disability, and inability to cooperate with MCG (aphasia, encephalopathy, restraints). Clears the BMI band (22.0–22.9 against &gt;30 or &lt;18).</x:v>
       </x:c>
     </x:row>
     <x:row r="868" ht="58" customHeight="1">
@@ -24437,7 +24437,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I868" s="9" t="str">
-        <x:v>CAR-T trial for relapsed/refractory multiple myeloma. Patient has no plasma cell disorder — no M-protein, free light chains, marrow plasma cells, or haematologic malignancy anywhere in his record; only oncologic entry is remote personal history of prostate cancer. Age 80 exceeds the 18–75 ceiling (registry age_max again null). Triggers the high-priority CNS disease exclusion emphatically — traumatic cerebral, subarachnoid, and subdural haemorrhage, cerebral infarction, prior TIA, toxic encephalopathy, aphasia — mechanistically critical given CAR-T neurotoxicity risk. Fails organ function: ALT 23–276 (~6.9× ULN) and AST 16–150 (~3.75× ULN) against a 3× ceiling. ECOG would be 4 against a required 0–2. Active infection exclusion triggered (pneumonia, cellulitis, vancomycin level). Protocol permits guardian consent, so encephalopathy was not the consent barrier.</x:v>
+        <x:v>CAR-T trial for relapsed/refractory multiple myeloma. Patient has no plasma cell disorder, no M-protein, free light chains, marrow plasma cells, or haematologic malignancy anywhere in his record; only oncologic entry is remote personal history of prostate cancer. Age 80 exceeds the 18–75 ceiling (registry age_max again null). Triggers the high-priority CNS disease exclusion emphatically, traumatic cerebral, subarachnoid, and subdural haemorrhage, cerebral infarction, prior TIA, toxic encephalopathy, aphasia, mechanistically critical given CAR-T neurotoxicity risk. Fails organ function: ALT 23–276 (~6.9× ULN) and AST 16–150 (~3.75× ULN) against a 3× ceiling. ECOG would be 4 against a required 0–2. Active infection exclusion triggered (pneumonia, cellulitis, vancomycin level). Protocol permits guardian consent, so encephalopathy was not the consent barrier.</x:v>
       </x:c>
     </x:row>
     <x:row r="869" ht="58" customHeight="1">
@@ -24495,7 +24495,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I870" s="9" t="str">
-        <x:v>First pair in this patient's series where inclusion criteria are MET — age ≥22 and history of cardiovascular disease (cerebral infarction, prior TIA, thoracic aortic aneurysm, AF, hypertension). Fails on the forced expiration exclusion, both limbs: technically inadequate because aphasia, anarthria, toxic encephalopathy, other symbolic dysfunctions, and physical restraints make the manoeuvre uninstructable; and unsafe because forced expiration raises intracranial pressure in a patient with recent traumatic cerebral, subarachnoid, and subdural haemorrhage. Respiratory reserve also compromised (acute respiratory failure with hypoxia, pneumonia, aspiration pneumonitis, atelectasis, recent 24–96h ventilation). Clears all other exclusions — no pacemaker/ICD, no terminal illness, no cardiothoracic surgery, no retinal disease or eye surgery, hypotensive rather than hypertensive, no tremors. Potentially time-limited if command-following recovers.</x:v>
+        <x:v>First pair in this patient's series where inclusion criteria are MET, age ≥22 and history of cardiovascular disease (cerebral infarction, prior TIA, thoracic aortic aneurysm, AF, hypertension). Fails on the forced expiration exclusion, both limbs: technically inadequate because aphasia, anarthria, toxic encephalopathy, other symbolic dysfunctions, and physical restraints make the manoeuvre uninstructable; and unsafe because forced expiration raises intracranial pressure in a patient with recent traumatic cerebral, subarachnoid, and subdural haemorrhage. Respiratory reserve also compromised (acute respiratory failure with hypoxia, pneumonia, aspiration pneumonitis, atelectasis, recent 24–96h ventilation). Clears all other exclusions, no pacemaker/ICD, no terminal illness, no cardiothoracic surgery, no retinal disease or eye surgery, hypotensive rather than hypertensive, no tremors. Potentially time-limited if command-following recovers.</x:v>
       </x:c>
     </x:row>
     <x:row r="871" ht="58" customHeight="1">
@@ -24522,7 +24522,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I871" s="9" t="str">
-        <x:v>First genuine CTO PCI patient in the review — chronic total occlusion of coronary artery coded, with PTCA, drug-eluting stent insertion, single vessel procedure, coronary arteriography, and left heart catheterization all documented, plus long-term antiplatelet therapy. Age 52 and no cognitive barrier to consent. Low confidence because the trial's sole exclusion is contraindication to adenosine and he has documented asthma (unspecified type and severity) — adenosine causes bronchospasm and is required for the FFR/CFR/IMR components; only RFR is adenosine-free, and the primary endpoint compares the two. Asthma severity assessment is the decisive screening item and could flip this to No. Secondary question: he also has 4+ vessel CABG with IMA graft and recent post-op course (ventilation, extubation, arterial line), so the sequence and interval between PCI and bypass must be established to confirm the post-PCI physiology window is still open.</x:v>
+        <x:v>First genuine CTO PCI patient in the review, chronic total occlusion of coronary artery coded, with PTCA, drug-eluting stent insertion, single vessel procedure, coronary arteriography, and left heart catheterization all documented, plus long-term antiplatelet therapy. Age 52 and no cognitive barrier to consent. Low confidence because the trial's sole exclusion is contraindication to adenosine and he has documented asthma (unspecified type and severity), adenosine causes bronchospasm and is required for the FFR/CFR/IMR components; only RFR is adenosine-free, and the primary endpoint compares the two. Asthma severity assessment is the decisive screening item and could flip this to No. Secondary question: he also has 4+ vessel CABG with IMA graft and recent post-op course (ventilation, extubation, arterial line), so the sequence and interval between PCI and bypass must be established to confirm the post-PCI physiology window is still open.</x:v>
       </x:c>
     </x:row>
     <x:row r="872" ht="58" customHeight="1">
@@ -24551,7 +24551,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I872" s="9" t="str">
-        <x:v>Trial treats acute coronary artery perforation with a covered stent, enrolling in the cath lab at the moment of perforation. No perforation, pericardial effusion, tamponade, or haemopericardium documented; haemoglobin 10.8–15.4 with no acute blood loss anaemia. His interventional history (PTCA, drug-eluting stents, 4+ vessel CABG, coronary arteriography) is what drew the pairing and represents perforation risk, not occurrence. Not a satisfiable prerequisite — a perforation is an adverse event, not a schedulable procedure. Clears every stated exclusion: on long-term antiplatelet therapy, tolerates contrast and cobalt-chromium stents, no compliance concerns, no IABP/ECMO requirement.</x:v>
+        <x:v>Trial treats acute coronary artery perforation with a covered stent, enrolling in the cath lab at the moment of perforation. No perforation, pericardial effusion, tamponade, or haemopericardium documented; haemoglobin 10.8–15.4 with no acute blood loss anaemia. His interventional history (PTCA, drug-eluting stents, 4+ vessel CABG, coronary arteriography) is what drew the pairing and represents perforation risk, not occurrence. Not a satisfiable prerequisite, a perforation is an adverse event, not a schedulable procedure. Clears every stated exclusion: on long-term antiplatelet therapy, tolerates contrast and cobalt-chromium stents, no compliance concerns, no IABP/ECMO requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="873" ht="58" customHeight="1">
@@ -24580,7 +24580,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I873" s="9" t="str">
-        <x:v>Clinical population fit is genuine — intermediate coronary syndrome (unstable angina) plus documented PTCA, drug-eluting stent insertion, and single-vessel intervention, unlike PAIR-000853 where the same trial failed a patient coded "without angina pectoris." Excluded at patient level by prior CABG: aortocoronary bypass of 4+ vessels, IMA graft, and extracorporeal circulation, with cabg clinical tag. Chronic total occlusion separately excluded at lesion level — the same finding that qualified him for ULTRA-CTO at PAIR-000924. Clears antiplatelet tolerance, STEMI, cardiogenic shock, and life expectancy; LVEF unknown but no heart failure coded.</x:v>
+        <x:v>Clinical population fit is genuine, intermediate coronary syndrome (unstable angina) plus documented PTCA, drug-eluting stent insertion, and single-vessel intervention, unlike PAIR-000853 where the same trial failed a patient coded "without angina pectoris." Excluded at patient level by prior CABG: aortocoronary bypass of 4+ vessels, IMA graft, and extracorporeal circulation, with cabg clinical tag. Chronic total occlusion separately excluded at lesion level, the same finding that qualified him for ULTRA-CTO at PAIR-000924. Clears antiplatelet tolerance, STEMI, cardiogenic shock, and life expectancy; LVEF unknown but no heart failure coded.</x:v>
       </x:c>
     </x:row>
     <x:row r="874" ht="58" customHeight="1">
@@ -24609,7 +24609,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I874" s="9" t="str">
-        <x:v>Meets ALL inclusion criteria — age 52, intermediate coronary syndrome establishing symptomatic ischaemia, and chronic total occlusion of coronary artery documented (CTO is by definition ≥3 months). Excluded solely by history of coronary artery bypass grafting: 4+ vessel aortocoronary bypass, IMA graft, extracorporeal circulation, cabg clinical tag. Mechanistically sound exclusion — grafts supply the occluded territory and alter both collateral formation and outcome, the study's two endpoints. PCI-within-3-months exclusion may also apply (PTCA and DES documented, undated). Clears eGFR (creatinine 0–1.0), NYHA ≥3 heart failure (none coded), malignancy, immune disorders, and pulmonary heart disease.</x:v>
+        <x:v>Meets ALL inclusion criteria, age 52, intermediate coronary syndrome establishing symptomatic ischaemia, and chronic total occlusion of coronary artery documented (CTO is by definition ≥3 months). Excluded solely by history of coronary artery bypass grafting: 4+ vessel aortocoronary bypass, IMA graft, extracorporeal circulation, cabg clinical tag. Mechanistically sound exclusion, grafts supply the occluded territory and alter both collateral formation and outcome, the study's two endpoints. PCI-within-3-months exclusion may also apply (PTCA and DES documented, undated). Clears eGFR (creatinine 0–1.0), NYHA ≥3 heart failure (none coded), malignancy, immune disorders, and pulmonary heart disease.</x:v>
       </x:c>
     </x:row>
     <x:row r="875" ht="58" customHeight="1">
@@ -24636,7 +24636,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I875" s="9" t="str">
-        <x:v>Key distinction from PAIR-000926 and 000927: this trial has NO blanket prior-CABG exclusion — only "target lesion located in bypass graft" and "CTO in the study target vessel," both lesion-level. His 4-vessel CABG and CTO therefore do not categorically disqualify him. Meets age ≥19, suspected ischaemic heart disease (CAD, intermediate coronary syndrome), verbal consent capacity, and has demonstrably stentable anatomy (PTCA, DES, single vessel procedure) with antiplatelet tolerance. Clears all bleeding exclusions (INR 1.0–1.2, platelets 169–252, no bleeding events), life expectancy, and STEMI. Low confidence: entry requires a current 50–90% index stenosis, which is unestablished — his CTO is 100% and outside that band. High-priority concern is angiography-derived FFR eligibility, technically questionable in bypassed anatomy with competitive graft flow and CTO collaterals.</x:v>
+        <x:v>Key distinction from PAIR-000926 and 000927: this trial has NO blanket prior-CABG exclusion, only "target lesion located in bypass graft" and "CTO in the study target vessel," both lesion-level. His 4-vessel CABG and CTO therefore do not categorically disqualify him. Meets age ≥19, suspected ischaemic heart disease (CAD, intermediate coronary syndrome), verbal consent capacity, and has demonstrably stentable anatomy (PTCA, DES, single vessel procedure) with antiplatelet tolerance. Clears all bleeding exclusions (INR 1.0–1.2, platelets 169–252, no bleeding events), life expectancy, and STEMI. Low confidence: entry requires a current 50–90% index stenosis, which is unestablished, his CTO is 100% and outside that band. High-priority concern is angiography-derived FFR eligibility, technically questionable in bypassed anatomy with competitive graft flow and CTO collaterals.</x:v>
       </x:c>
     </x:row>
     <x:row r="876" ht="58" customHeight="1">
@@ -24663,7 +24663,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I876" s="9" t="str">
-        <x:v>Coronary sinus reducer for no-option refractory angina. His trajectory fits the population — CAD with chronic total occlusion, prior DES PCI and 4+ vessel CABG with IMA graft, intermediate coronary syndrome indicating symptomatic ischaemia; exhausted revascularization is the route into reducer candidacy rather than a bar. Clears all four exclusions: no heart failure coded (argues against EF &lt;35%), creatinine 0–1.0 (eGFR far above 30), asthma rather than GOLD D COPD. Hyperaemic-agent concern is resolvable — regadenoson carries bronchospasm risk in asthma, but the protocol names papaverine as an alternative and papaverine has no bronchoconstrictive effect (contrast PAIR-000924, where adenosine was the sole agent). Low confidence: nothing documents that his angina is refractory or that a heart team has ruled out further revascularization, and his bypass appears recent (post-op ventilation, arterial line, extubation), so symptom outcome is not yet established.</x:v>
+        <x:v>Coronary sinus reducer for no-option refractory angina. His trajectory fits the population, CAD with chronic total occlusion, prior DES PCI and 4+ vessel CABG with IMA graft, intermediate coronary syndrome indicating symptomatic ischaemia; exhausted revascularization is the route into reducer candidacy rather than a bar. Clears all four exclusions: no heart failure coded (argues against EF &lt;35%), creatinine 0–1.0 (eGFR far above 30), asthma rather than GOLD D COPD. Hyperaemic-agent concern is resolvable, regadenoson carries bronchospasm risk in asthma, but the protocol names papaverine as an alternative and papaverine has no bronchoconstrictive effect (contrast PAIR-000924, where adenosine was the sole agent). Low confidence: nothing documents that his angina is refractory or that a heart team has ruled out further revascularization, and his bypass appears recent (post-op ventilation, arterial line, extubation), so symptom outcome is not yet established.</x:v>
       </x:c>
     </x:row>
     <x:row r="877" ht="58" customHeight="1">
@@ -24692,7 +24692,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I877" s="9" t="str">
-        <x:v>Genuine premature CAD phenotype — male aged 52 within the 18–55 window, multivessel disease requiring 4-vessel bypass. Excluded by "prior coronary artery bypass grafting or coronary intervention," hit on both limbs: aortocoronary bypass of 4+ vessels with IMA graft and extracorporeal circulation, plus PTCA with drug-eluting stent insertion and single-vessel procedure. Design enrols "following initial PCI," so treatment-naive anatomy is structural. LDL likely qualifies via the on-statin route (calculated LDL to 124 mg/dL ≈ 3.2 mmol/L vs 1.8 threshold). Clears every other exclusion — no statin/PCSK9 contraindication or prior use, no haemorrhagic stroke, creatinine 0–1.0, normal LFTs (ALT 5–24, AST 3–19, albumin 3.9–4.1), triglycerides 0.8–1.7 mmol/L. Serial OCT would also be technically compromised by existing stent struts and competitive graft flow.</x:v>
+        <x:v>Genuine premature CAD phenotype, male aged 52 within the 18–55 window, multivessel disease requiring 4-vessel bypass. Excluded by "prior coronary artery bypass grafting or coronary intervention," hit on both limbs: aortocoronary bypass of 4+ vessels with IMA graft and extracorporeal circulation, plus PTCA with drug-eluting stent insertion and single-vessel procedure. Design enrols "following initial PCI," so treatment-naive anatomy is structural. LDL likely qualifies via the on-statin route (calculated LDL to 124 mg/dL ≈ 3.2 mmol/L vs 1.8 threshold). Clears every other exclusion, no statin/PCSK9 contraindication or prior use, no haemorrhagic stroke, creatinine 0–1.0, normal LFTs (ALT 5–24, AST 3–19, albumin 3.9–4.1), triglycerides 0.8–1.7 mmol/L. Serial OCT would also be technically compromised by existing stent struts and competitive graft flow.</x:v>
       </x:c>
     </x:row>
     <x:row r="878" ht="58" customHeight="1">
@@ -24719,7 +24719,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I878" s="9" t="str">
-        <x:v>Post-CABG (4+ vessels, IMA graft) AND post-PCI (PTCA, drug-eluting stents) with documented hypertension and long-term antiplatelet therapy; age 52; cognitively intact so smartphone use and consent are unproblematic. Clears ALL exclusions cleanly — no heart failure or arrhythmia (the criterion that disqualified PAIR-000907), no malignancy, normal renal (creatinine 0–1.0) and hepatic (ALT 5–24, AST 3–19, albumin 3.9–4.1) function. Medium rather than High because the conjunctive comorbidity requirement is only partly documented: hypertension coded, but diabetes and dyslipidaemia are not, though glucose to 208 mg/dL with a metabolic_disease tag and LDL 124 with HDL 32 point toward both. "At least one of" criterion likely met via LDL (~3.2 mmol/L). HbA1c and a lipid panel would settle it.</x:v>
+        <x:v>Post-CABG (4+ vessels, IMA graft) AND post-PCI (PTCA, drug-eluting stents) with documented hypertension and long-term antiplatelet therapy; age 52; cognitively intact so smartphone use and consent are unproblematic. Clears ALL exclusions cleanly, no heart failure or arrhythmia (the criterion that disqualified PAIR-000907), no malignancy, normal renal (creatinine 0–1.0) and hepatic (ALT 5–24, AST 3–19, albumin 3.9–4.1) function. Medium rather than High because the conjunctive comorbidity requirement is only partly documented: hypertension coded, but diabetes and dyslipidaemia are not, though glucose to 208 mg/dL with a metabolic_disease tag and LDL 124 with HDL 32 point toward both. "At least one of" criterion likely met via LDL (~3.2 mmol/L). HbA1c and a lipid panel would settle it.</x:v>
       </x:c>
     </x:row>
     <x:row r="879" ht="58" customHeight="1">
@@ -24746,7 +24746,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I879" s="9" t="str">
-        <x:v>Home-based e-health cardiac rehabilitation for CAD after PCI. Meets inclusion — CAD with documented PTCA, drug-eluting stents, and pci clinical tag; age 52; cognitively intact for consent. Clears every clinical exclusion: no aortic stenosis or valvular disease, no arrhythmia, no cognitive impairment, life expectancy unremarkable (normal renal and hepatic function). Appears fully revascularized, having completed both PCI and 4+ vessel CABG. Medium confidence: chronic total occlusion may or may not have been addressed, so confirmation that no further revascularization is pending is the key screening item; and "living at home" plus "otherwise clinically unstable" are transiently unmet during immediate post-bypass recovery, which is a scheduling rather than eligibility matter since CR is normally initiated weeks after discharge. Norwegian national ID and language requirements treated as logistical per review standard, consistent with prior pairs.</x:v>
+        <x:v>Home-based e-health cardiac rehabilitation for CAD after PCI. Meets inclusion, CAD with documented PTCA, drug-eluting stents, and pci clinical tag; age 52; cognitively intact for consent. Clears every clinical exclusion: no aortic stenosis or valvular disease, no arrhythmia, no cognitive impairment, life expectancy unremarkable (normal renal and hepatic function). Appears fully revascularized, having completed both PCI and 4+ vessel CABG. Medium confidence: chronic total occlusion may or may not have been addressed, so confirmation that no further revascularization is pending is the key screening item; and "living at home" plus "otherwise clinically unstable" are transiently unmet during immediate post-bypass recovery, which is a scheduling rather than eligibility matter since CR is normally initiated weeks after discharge. Norwegian national ID and language requirements treated as logistical per review standard, consistent with prior pairs.</x:v>
       </x:c>
     </x:row>
     <x:row r="880" ht="58" customHeight="1">
@@ -24775,7 +24775,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I880" s="9" t="str">
-        <x:v>Trial randomizes conduction system pacing vs right ventricular pacing in patients with atrioventricular block requiring permanent pacemaker. Patient has no AV block, no conduction disorder, no bradycardia, no arrhythmia, and no pacemaker or pacing indication — his cardiac disease is entirely ischaemic (CAD, chronic total occlusion, intermediate coronary syndrome). Not a satisfiable prerequisite: AV block is a diagnosis, not a schedulable procedure. Recent bypass surgery (perioperative course documented) would likely also trigger the PCI/CABG-within-30-days exclusion. Meets age 18–80 and &gt;1 year survival; clears secondary hypertension, orthostatic hypotension, valvular disease, and congenital heart disease.</x:v>
+        <x:v>Trial randomizes conduction system pacing vs right ventricular pacing in patients with atrioventricular block requiring permanent pacemaker. Patient has no AV block, no conduction disorder, no bradycardia, no arrhythmia, and no pacemaker or pacing indication, his cardiac disease is entirely ischaemic (CAD, chronic total occlusion, intermediate coronary syndrome). Not a satisfiable prerequisite: AV block is a diagnosis, not a schedulable procedure. Recent bypass surgery (perioperative course documented) would likely also trigger the PCI/CABG-within-30-days exclusion. Meets age 18–80 and &gt;1 year survival; clears secondary hypertension, orthostatic hypotension, valvular disease, and congenital heart disease.</x:v>
       </x:c>
     </x:row>
     <x:row r="881" ht="58" customHeight="1">
@@ -24833,7 +24833,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I882" s="9" t="str">
-        <x:v>Paediatric study recruiting children aged 7–18 with newly diagnosed primary hypertension from paediatric nephrology clinics, with caregiver consent. Patient is 91 — outside the window by 73 years, and the &gt;18 exclusion is stated explicitly for both cohorts. Also fails the confounding-condition exclusion repeatedly: aortic stenosis, nonrheumatic mitral insufficiency, rheumatic tricuspid insufficiency, first degree AV block, cerebral infarction of the left vertebral artery, and diabetes (HbA1c 6.1–7.0). Cannot complete assessments given disorientation, altered mental status, age-related cognitive decline, hearing loss, and hemiplegia. Hypertension is neither new nor the paediatric primary phenotype. NOTE: registry structured age field reads min 7 / NO MAXIMUM — a matcher filtering on structured age would not exclude a 91-year-old from a paediatric trial.</x:v>
+        <x:v>Paediatric study recruiting children aged 7–18 with newly diagnosed primary hypertension from paediatric nephrology clinics, with caregiver consent. Patient is 91, outside the window by 73 years, and the &gt;18 exclusion is stated explicitly for both cohorts. Also fails the confounding-condition exclusion repeatedly: aortic stenosis, nonrheumatic mitral insufficiency, rheumatic tricuspid insufficiency, first degree AV block, cerebral infarction of the left vertebral artery, and diabetes (HbA1c 6.1–7.0). Cannot complete assessments given disorientation, altered mental status, age-related cognitive decline, hearing loss, and hemiplegia. Hypertension is neither new nor the paediatric primary phenotype. NOTE: registry structured age field reads min 7 / NO MAXIMUM, a matcher filtering on structured age would not exclude a 91-year-old from a paediatric trial.</x:v>
       </x:c>
     </x:row>
     <x:row r="883" ht="58" customHeight="1">
@@ -24862,7 +24862,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I883" s="9" t="str">
-        <x:v>Trial requires type 2 diabetes WITH combined dyslipidaemia — triglycerides 200–499 mg/dL and HDL ≤50 mg/dL for women — for a fibrate intervention targeting that phenotype. Patient's triglycerides are 47–85 mg/dL (n=9), less than half the required floor, and HDL is 65–83 mg/dL (n=9), well above the ceiling; total/HDL ratio 1.9–2.7 and calculated LDL 61–91. Both limbs fail affirmatively and in the favourable direction. Coded "pure hypercholesterolaemia" is inconsistent with her measured lipids and likely historical or treated. Diabetes criterion met (HbA1c 6.1–7.0) and creatinine 0.5–0.9 clears the ≤1.8 requirement. Clears all exclusions except possible clopidogrel use (post-stroke, unverifiable).</x:v>
+        <x:v>Trial requires type 2 diabetes WITH combined dyslipidaemia, triglycerides 200–499 mg/dL and HDL ≤50 mg/dL for women, for a fibrate intervention targeting that phenotype. Patient's triglycerides are 47–85 mg/dL (n=9), less than half the required floor, and HDL is 65–83 mg/dL (n=9), well above the ceiling; total/HDL ratio 1.9–2.7 and calculated LDL 61–91. Both limbs fail affirmatively and in the favourable direction. Coded "pure hypercholesterolaemia" is inconsistent with her measured lipids and likely historical or treated. Diabetes criterion met (HbA1c 6.1–7.0) and creatinine 0.5–0.9 clears the ≤1.8 requirement. Clears all exclusions except possible clopidogrel use (post-stroke, unverifiable).</x:v>
       </x:c>
     </x:row>
     <x:row r="884" ht="58" customHeight="1">
@@ -24891,7 +24891,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I884" s="9" t="str">
-        <x:v>Trial requires ASYMPTOMATIC atherosclerosis — high-priority criterion excluding history of angina, MI, or cerebral infarction. Patient has completed cerebral infarction of the left vertebral artery with residual hemiplegia (left nondominant) plus prior TIA — symptomatic and permanent. Separately fails all three combined-dyslipidaemia limbs: triglycerides 47–85 vs ≥200 required, HDL 65–83 vs ≤50 required, calculated LDL 61–91 vs ≥100 required (n=9 each); total/HDL ratio 1.9–2.7. Meets age ≥20, HbA1c 6.1–7.0 diabetes criterion, and creatinine ≤1.8 (0.5–0.9). Clears renal, hepatic, and hypertension exclusions. Non-statin lipid therapy status unverifiable (medication field empty). Sister trial to PAIR-000936, which lacked the asymptomatic requirement and the LDL limb.</x:v>
+        <x:v>Trial requires ASYMPTOMATIC atherosclerosis, high-priority criterion excluding history of angina, MI, or cerebral infarction. Patient has completed cerebral infarction of the left vertebral artery with residual hemiplegia (left nondominant) plus prior TIA, symptomatic and permanent. Separately fails all three combined-dyslipidaemia limbs: triglycerides 47–85 vs ≥200 required, HDL 65–83 vs ≤50 required, calculated LDL 61–91 vs ≥100 required (n=9 each); total/HDL ratio 1.9–2.7. Meets age ≥20, HbA1c 6.1–7.0 diabetes criterion, and creatinine ≤1.8 (0.5–0.9). Clears renal, hepatic, and hypertension exclusions. Non-statin lipid therapy status unverifiable (medication field empty). Sister trial to PAIR-000936, which lacked the asymptomatic requirement and the LDL limb.</x:v>
       </x:c>
     </x:row>
     <x:row r="885" ht="58" customHeight="1">
@@ -24920,7 +24920,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I885" s="9" t="str">
-        <x:v>Trial requires dyslipidaemia via one of three routes; all fail affirmatively across n=9 measurements each — calculated LDL 61–91 vs ≥160, triglycerides 47–85 vs ≥150, HDL 65–83 vs &lt;50 for women. Total/HDL ratio 1.9–2.7. Coded "pure hypercholesterolaemia" contradicted by measured values. Also explicitly excluded by diabetes (clinical tag, HbA1c 6.1–7.0, glucose 69–196) and by active infectious disease (pneumonia unspecified organism, influenza with pneumonia) — both of which would confound the study's inflammatory marker endpoints. Antibiotic use likely. Clears anticoagulant exclusion (INR 1.1–1.2, PT and PTT normal). Registry age fields both null. Practical feasibility also poor at 91 with hemiplegia, cognitive decline, and recurrent falls.</x:v>
+        <x:v>Trial requires dyslipidaemia via one of three routes; all fail affirmatively across n=9 measurements each, calculated LDL 61–91 vs ≥160, triglycerides 47–85 vs ≥150, HDL 65–83 vs &lt;50 for women. Total/HDL ratio 1.9–2.7. Coded "pure hypercholesterolaemia" contradicted by measured values. Also explicitly excluded by diabetes (clinical tag, HbA1c 6.1–7.0, glucose 69–196) and by active infectious disease (pneumonia unspecified organism, influenza with pneumonia), both of which would confound the study's inflammatory marker endpoints. Antibiotic use likely. Clears anticoagulant exclusion (INR 1.1–1.2, PT and PTT normal). Registry age fields both null. Practical feasibility also poor at 91 with hemiplegia, cognitive decline, and recurrent falls.</x:v>
       </x:c>
     </x:row>
     <x:row r="886" ht="58" customHeight="1">
@@ -24949,7 +24949,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I886" s="9" t="str">
-        <x:v>Excluded by the high-priority "current medical diagnosis of type 1 or type 2 diabetes mellitus" — diabetes clinical tag documented — reinforced by HbA1c reaching 7.0% against a ≥6.5% exclusion; the trial targets pre-diabetes (5.7–6.4%) specifically. Alternative dyslipidaemia route also fails on all four thresholds: total cholesterol 149–182 vs ≥200, LDL 61–91 vs ≥130, HDL 65–83 vs ≤40, triglycerides 47–85 vs ≥150 (n=9 each). Cannot consent or comply — disorientation, altered mental status, age-related cognitive decline, hearing loss, hemiplegia, recurrent falls. Active pneumonia and influenza trigger the infection exclusion (deferrable per protocol). BMI undocumented but likely below the 28–35 band given frailty. Possible GI exclusion via other specified intestinal obstruction (GERD explicitly acceptable). NOTE: registry age_min reads 90 against criteria text of ≥18 — first instance in this review of a structured age field being MORE restrictive than the protocol.</x:v>
+        <x:v>Excluded by the high-priority "current medical diagnosis of type 1 or type 2 diabetes mellitus", diabetes clinical tag documented, reinforced by HbA1c reaching 7.0% against a ≥6.5% exclusion; the trial targets pre-diabetes (5.7–6.4%) specifically. Alternative dyslipidaemia route also fails on all four thresholds: total cholesterol 149–182 vs ≥200, LDL 61–91 vs ≥130, HDL 65–83 vs ≤40, triglycerides 47–85 vs ≥150 (n=9 each). Cannot consent or comply, disorientation, altered mental status, age-related cognitive decline, hearing loss, hemiplegia, recurrent falls. Active pneumonia and influenza trigger the infection exclusion (deferrable per protocol). BMI undocumented but likely below the 28–35 band given frailty. Possible GI exclusion via other specified intestinal obstruction (GERD explicitly acceptable). NOTE: registry age_min reads 90 against criteria text of ≥18, first instance in this review of a structured age field being MORE restrictive than the protocol.</x:v>
       </x:c>
     </x:row>
     <x:row r="887" ht="58" customHeight="1">
@@ -24978,7 +24978,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I887" s="9" t="str">
-        <x:v>Unusually sparse criteria (3 inclusions, 2 exclusions) and she is not clearly barred by any: triglycerides 47–85 well under the 400 ceiling, HbA1c 6.1–7.0 under the ≥10 exclusion, LDL 61–91 straddles the &gt;70 requirement. Lp(a) never measured — the study's central variable, and cohort 1 is already FILLED so only the narrow 20–49 mg/dL band remains. Decided on grounds the criteria do not enumerate: informed consent is not obtainable given disorientation, altered mental status, and age-related cognitive decline, for a 16-week protocol of daily oral drug plus biweekly subcutaneous injections. Cerebral infarction with residual hemiplegia bears on the CV-events-within-3-months exclusion (undated). Active pneumonia and influenza, Hgb nadir 8 requiring transfusion, potassium 2.6–6.1, SIADH. Medium confidence — verdict rests substantially on clinical judgment beyond the stated criteria. Note: unlike the preceding trial, diabetes is NOT disqualifying here.</x:v>
+        <x:v>Unusually sparse criteria (3 inclusions, 2 exclusions) and she is not clearly barred by any: triglycerides 47–85 well under the 400 ceiling, HbA1c 6.1–7.0 under the ≥10 exclusion, LDL 61–91 straddles the &gt;70 requirement. Lp(a) never measured, the study's central variable, and cohort 1 is already FILLED so only the narrow 20–49 mg/dL band remains. Decided on grounds the criteria do not enumerate: informed consent is not obtainable given disorientation, altered mental status, and age-related cognitive decline, for a 16-week protocol of daily oral drug plus biweekly subcutaneous injections. Cerebral infarction with residual hemiplegia bears on the CV-events-within-3-months exclusion (undated). Active pneumonia and influenza, Hgb nadir 8 requiring transfusion, potassium 2.6–6.1, SIADH. Medium confidence, verdict rests substantially on clinical judgment beyond the stated criteria. Note: unlike the preceding trial, diabetes is NOT disqualifying here.</x:v>
       </x:c>
     </x:row>
     <x:row r="888" ht="58" customHeight="1">
@@ -25007,7 +25007,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I888" s="9" t="str">
-        <x:v>Digital tablet-delivered lifestyle intervention with home bio-signal self-monitoring. Excluded by cognitive difficulties (SPMSQ criterion) — disorientation, altered mental status, age-related cognitive decline documented — which also makes the required internet and tablet use unachievable given hemiplegia and hearing loss. Separately excluded by antiepileptic medication: carbamazepine drug levels present in her lab panel, consistent with her documented trigeminal neuralgia; carbamazepine is a CYP3A4 inducer affecting cortisol, the study's stress biomarker. Metabolic entry criterion also fails — hyperlipidaemia component not met (triglycerides 47–85 vs ≥150, HDL 65–83 vs ≤50) and central obesity undocumented; hypertension and diabetes components are met. Chronic pain is organic (osteoarthritis, trigeminal neuralgia, knee effusion, Baker's cyst) rather than psychosomatic as the criterion requires. Hong Kong site and Cantonese requirements treated as logistical.</x:v>
+        <x:v>Digital tablet-delivered lifestyle intervention with home bio-signal self-monitoring. Excluded by cognitive difficulties (SPMSQ criterion), disorientation, altered mental status, age-related cognitive decline documented, which also makes the required internet and tablet use unachievable given hemiplegia and hearing loss. Separately excluded by antiepileptic medication: carbamazepine drug levels present in her lab panel, consistent with her documented trigeminal neuralgia; carbamazepine is a CYP3A4 inducer affecting cortisol, the study's stress biomarker. Metabolic entry criterion also fails, hyperlipidaemia component not met (triglycerides 47–85 vs ≥150, HDL 65–83 vs ≤50) and central obesity undocumented; hypertension and diabetes components are met. Chronic pain is organic (osteoarthritis, trigeminal neuralgia, knee effusion, Baker's cyst) rather than psychosomatic as the criterion requires. Hong Kong site and Cantonese requirements treated as logistical.</x:v>
       </x:c>
     </x:row>
     <x:row r="889" ht="58" customHeight="1">
@@ -25036,7 +25036,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I889" s="9" t="str">
-        <x:v>Cross-sectional chart analysis of hypertensive heart disease at a Congolese tertiary hospital; minimal criteria (2 inclusions, 2 mirrored exclusions) turning entirely on the diagnosis. Hypertensive heart disease is not coded. She has hypertension and cardiac disease separately, with non-hypertensive aetiologies — aortic stenosis (degenerative at 91), nonrheumatic mitral insufficiency, rheumatic tricuspid insufficiency, first degree AV block. No LVH, hypertensive cardiomyopathy, or hypertensive heart failure documented; NTproBNP 483–631 is modest for her age. Medium confidence — the diagnosis is absent rather than excluded, and a clinician might reasonably apply the label to a 91-year-old with long-standing hypertension; an echocardiogram would settle it, and she has had none. Institutional chart-review population noted but treated as logistical per review standard.</x:v>
+        <x:v>Cross-sectional chart analysis of hypertensive heart disease at a Congolese tertiary hospital; minimal criteria (2 inclusions, 2 mirrored exclusions) turning entirely on the diagnosis. Hypertensive heart disease is not coded. She has hypertension and cardiac disease separately, with non-hypertensive aetiologies, aortic stenosis (degenerative at 91), nonrheumatic mitral insufficiency, rheumatic tricuspid insufficiency, first degree AV block. No LVH, hypertensive cardiomyopathy, or hypertensive heart failure documented; NTproBNP 483–631 is modest for her age. Medium confidence, the diagnosis is absent rather than excluded, and a clinician might reasonably apply the label to a 91-year-old with long-standing hypertension; an echocardiogram would settle it, and she has had none. Institutional chart-review population noted but treated as logistical per review standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="890" ht="58" customHeight="1">
@@ -25065,7 +25065,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I890" s="9" t="str">
-        <x:v>Food-insecurity intervention for children with cancer, enrolling within 12 months of completing chemotherapy or radiation, with parent/guardian food insecurity screening. Patient has no malignancy of any kind and no oncologic therapy — her three procedures are total knee replacement, packed cell transfusion, and knee drainage. Age 91 against a paediatric framework, though the criterion does permit over-18 participants under medical guardianship, which her cognitive decline makes nominally conceivable — the cancer requirement is the categorical bar. She would satisfy the impaired glucose metabolism cardiovascular risk factor (HbA1c 6.1–7.0) but fail all four dyslipidaemia sub-thresholds; BMI and BP components use paediatric percentiles.</x:v>
+        <x:v>Food-insecurity intervention for children with cancer, enrolling within 12 months of completing chemotherapy or radiation, with parent/guardian food insecurity screening. Patient has no malignancy of any kind and no oncologic therapy, her three procedures are total knee replacement, packed cell transfusion, and knee drainage. Age 91 against a paediatric framework, though the criterion does permit over-18 participants under medical guardianship, which her cognitive decline makes nominally conceivable, the cancer requirement is the categorical bar. She would satisfy the impaired glucose metabolism cardiovascular risk factor (HbA1c 6.1–7.0) but fail all four dyslipidaemia sub-thresholds; BMI and BP components use paediatric percentiles.</x:v>
       </x:c>
     </x:row>
     <x:row r="891" ht="58" customHeight="1">
@@ -25094,7 +25094,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I891" s="9" t="str">
-        <x:v>Trial specifies 18 &lt; age &lt; 75 as a high-priority criterion; patient is 91, exceeding by 16 years. Registry structured age fields are both null, so the window exists only in criteria text (7th age-field discrepancy in this review). Has the target disease combination — atrial_fibrillation clinical tag with long-term antithrombotics, plus hypertension tag — but no BP values recorded. Also excluded by acute systemic infection (Klebsiella pneumoniae, abnormal urine microbiology, COPD with exacerbation, neutrophils to 80.2%) and by the "not suitable for PVI and RDN" catch-all: DNR status, immediate post-op after open internal fixation of displaced intertrochanteric femoral fracture, Hgb nadir 9.8, rheumatic mitral and tricuspid valve disease with NTproBNP 1155, hyponatraemia (Na 130–132). Skin cancer is remote personal history; alcohol dependence coded in remission. Left atrial size unmeasured but rheumatic mitral disease with AF gives high pretest probability of exceeding the 55 mm bar.</x:v>
+        <x:v>Trial specifies 18 &lt; age &lt; 75 as a high-priority criterion; patient is 91, exceeding by 16 years. Registry structured age fields are both null, so the window exists only in criteria text (7th age-field discrepancy in this review). Has the target disease combination, atrial_fibrillation clinical tag with long-term antithrombotics, plus hypertension tag, but no BP values recorded. Also excluded by acute systemic infection (Klebsiella pneumoniae, abnormal urine microbiology, COPD with exacerbation, neutrophils to 80.2%) and by the "not suitable for PVI and RDN" catch-all: DNR status, immediate post-op after open internal fixation of displaced intertrochanteric femoral fracture, Hgb nadir 9.8, rheumatic mitral and tricuspid valve disease with NTproBNP 1155, hyponatraemia (Na 130–132). Skin cancer is remote personal history; alcohol dependence coded in remission. Left atrial size unmeasured but rheumatic mitral disease with AF gives high pretest probability of exceeding the 55 mm bar.</x:v>
       </x:c>
     </x:row>
     <x:row r="892" ht="58" customHeight="1">
@@ -25123,7 +25123,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I892" s="9" t="str">
-        <x:v>Genuine disease match — COPD documented twice (COPD unspecified, obstructive chronic bronchitis with exacerbation) with tobacco history; no age ceiling in criteria or registry. Excluded by emergency inpatient stay within 4 weeks: displaced intertrochanteric left femoral fracture (initial encounter) after a fall on ice, treated by open reposition with internal fixation, Hgb nadir 9.8. Cannot meet the "physically able to follow instructions" requirement for a full-day protocol including exercise tolerance testing; likely wheelchair bound post-op given pre-existing hip and knee arthroplasties, osteoarthritis, and lumbar spinal stenosis. Active COPD exacerbation and Klebsiella infection (neutrophils 80.2%) would confound respiratory muscle and exercise measurements; rheumatic mitral and tricuspid valve disease with NTproBNP 1155 adds cardiac dyspnoea. Lumbar stenosis is not disc herniation; no epilepsy coded. Time-limited rather than categorical — revisit after recovery.</x:v>
+        <x:v>Genuine disease match, COPD documented twice (COPD unspecified, obstructive chronic bronchitis with exacerbation) with tobacco history; no age ceiling in criteria or registry. Excluded by emergency inpatient stay within 4 weeks: displaced intertrochanteric left femoral fracture (initial encounter) after a fall on ice, treated by open reposition with internal fixation, Hgb nadir 9.8. Cannot meet the "physically able to follow instructions" requirement for a full-day protocol including exercise tolerance testing; likely wheelchair bound post-op given pre-existing hip and knee arthroplasties, osteoarthritis, and lumbar spinal stenosis. Active COPD exacerbation and Klebsiella infection (neutrophils 80.2%) would confound respiratory muscle and exercise measurements; rheumatic mitral and tricuspid valve disease with NTproBNP 1155 adds cardiac dyspnoea. Lumbar stenosis is not disc herniation; no epilepsy coded. Time-limited rather than categorical, revisit after recovery.</x:v>
       </x:c>
     </x:row>
     <x:row r="893" ht="58" customHeight="1">
@@ -25150,7 +25150,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I893" s="9" t="str">
-        <x:v>Observational hypertension registry, data collection only — no drug, procedure, or follow-up burden. Documented primary hypertension with no secondary cause; admitted inpatient status confirmed by displaced intertrochanteric femoral fracture with open internal fixation. Clears the liver/kidney dysfunction exclusion more cleanly than PAIR-000865: creatinine 0.5–0.6 across 4 draws with no renal diagnosis, and no liver disease coded (though LFTs are entirely absent from her panel). Hyponatraemia (Na 130–132) is electrolyte rather than renal dysfunction. Open item is whether alcohol dependence IN REMISSION engages the "mental disorders" exclusion — no dementia, depression, or psychosis coded; transient alteration of awareness is neurological with ready explanations in AF and hyponatraemia. DNR status reflects care goals, not incapacity. Site is a single hospital in Xinjiang, China — treated as logistical per review standard, consistent with PAIR-000865.</x:v>
+        <x:v>Observational hypertension registry, data collection only, no drug, procedure, or follow-up burden. Documented primary hypertension with no secondary cause; admitted inpatient status confirmed by displaced intertrochanteric femoral fracture with open internal fixation. Clears the liver/kidney dysfunction exclusion more cleanly than PAIR-000865: creatinine 0.5–0.6 across 4 draws with no renal diagnosis, and no liver disease coded (though LFTs are entirely absent from her panel). Hyponatraemia (Na 130–132) is electrolyte rather than renal dysfunction. Open item is whether alcohol dependence IN REMISSION engages the "mental disorders" exclusion, no dementia, depression, or psychosis coded; transient alteration of awareness is neurological with ready explanations in AF and hyponatraemia. DNR status reflects care goals, not incapacity. Site is a single hospital in Xinjiang, China, treated as logistical per review standard, consistent with PAIR-000865.</x:v>
       </x:c>
     </x:row>
     <x:row r="894" ht="58" customHeight="1">
@@ -25179,7 +25179,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I894" s="9" t="str">
-        <x:v>Six-month self-guided smartphone app trial with home BP self-monitoring as primary endpoint. Documented primary hypertension; clears the high-priority secondary hypertension exclusion cleanly (no thyroid or kidney disease, creatinine 0.5–0.6). No age limit or cognitive criterion in the protocol. Fails on acute burden and functional capacity: emergency admission with displaced intertrochanteric femoral fracture and open internal fixation, Klebsiella infection, obstructive bronchitis exacerbation, Hgb nadir 9.8, DNR status. Self-guided digital participation doubtful at 91 with unspecified cataract, dizziness and giddiness, and transient alteration of awareness — though notably no dementia is coded. Likely exceeds the &gt;triple antihypertensive cap given hypertension plus AF, rheumatic mitral and tricuspid valve disease, and NTproBNP 1155. No BP values in record; 6-week dose stability implausible post-operatively.</x:v>
+        <x:v>Six-month self-guided smartphone app trial with home BP self-monitoring as primary endpoint. Documented primary hypertension; clears the high-priority secondary hypertension exclusion cleanly (no thyroid or kidney disease, creatinine 0.5–0.6). No age limit or cognitive criterion in the protocol. Fails on acute burden and functional capacity: emergency admission with displaced intertrochanteric femoral fracture and open internal fixation, Klebsiella infection, obstructive bronchitis exacerbation, Hgb nadir 9.8, DNR status. Self-guided digital participation doubtful at 91 with unspecified cataract, dizziness and giddiness, and transient alteration of awareness, though notably no dementia is coded. Likely exceeds the &gt;triple antihypertensive cap given hypertension plus AF, rheumatic mitral and tricuspid valve disease, and NTproBNP 1155. No BP values in record; 6-week dose stability implausible post-operatively.</x:v>
       </x:c>
     </x:row>
     <x:row r="895" ht="58" customHeight="1">
@@ -25208,7 +25208,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I895" s="9" t="str">
-        <x:v>Atrial fibrillation is an explicit named exclusion and she has it documented (clinical tag, long-term antithrombotics, INR 1.3). Methodologically decisive: the study classifies non-dipper status from repeated 24-hour ABPM, and oscillometric ambulatory measurement is unreliable in AF. No ABPM in her record, and the two required studies on a stable regimen are unachievable post-hip-fracture-surgery with active infection. Meets age &gt;18 and hypertension diagnosis; clears dementia (none coded — notable at 91), shift work, limb amputation (arthroplasties are not amputations), and pregnancy. Terminal-malignancy limb unclear — skin cancer is remote personal history, but DNR at 91 with COPD, fracture, and Klebsiella raises the life expectancy question.</x:v>
+        <x:v>Atrial fibrillation is an explicit named exclusion and she has it documented (clinical tag, long-term antithrombotics, INR 1.3). Methodologically decisive: the study classifies non-dipper status from repeated 24-hour ABPM, and oscillometric ambulatory measurement is unreliable in AF. No ABPM in her record, and the two required studies on a stable regimen are unachievable post-hip-fracture-surgery with active infection. Meets age &gt;18 and hypertension diagnosis; clears dementia (none coded, notable at 91), shift work, limb amputation (arthroplasties are not amputations), and pregnancy. Terminal-malignancy limb unclear, skin cancer is remote personal history, but DNR at 91 with COPD, fracture, and Klebsiella raises the life expectancy question.</x:v>
       </x:c>
     </x:row>
     <x:row r="896" ht="58" customHeight="1">
@@ -25237,7 +25237,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I896" s="9" t="str">
-        <x:v>Sleep restriction physiology experiment in healthy normotensive adults aged 18–35 stratified by parental hypertension history. Patient is 91 — 56 years past the ceiling, stated in both inclusion and exclusion lists. Registry age_max is null (8th such discrepancy in this review). Also fails the study's premise in reverse: it requires normotensive participants and she has established hypertension, with an office BP exclusion at ≥130/80. Not "healthy" — AF, COPD with exacerbation, rheumatic mitral and tricuspid valve disease (NTproBNP 1155), acute femoral fracture with ORIF, Klebsiella infection, OSA, hyponatraemia. Regular prescription medication (long-term antithrombotics) is separately exclusionary. Parental hypertension status, the stratification variable, is not realistically obtainable at 91. Hgb 9.8–12.4 straddles the 11.6 g/dL phlebotomy threshold. Clears GFR and likely the nonsmoker criterion (tobacco use is historical).</x:v>
+        <x:v>Sleep restriction physiology experiment in healthy normotensive adults aged 18–35 stratified by parental hypertension history. Patient is 91, 56 years past the ceiling, stated in both inclusion and exclusion lists. Registry age_max is null (8th such discrepancy in this review). Also fails the study's premise in reverse: it requires normotensive participants and she has established hypertension, with an office BP exclusion at ≥130/80. Not "healthy", AF, COPD with exacerbation, rheumatic mitral and tricuspid valve disease (NTproBNP 1155), acute femoral fracture with ORIF, Klebsiella infection, OSA, hyponatraemia. Regular prescription medication (long-term antithrombotics) is separately exclusionary. Parental hypertension status, the stratification variable, is not realistically obtainable at 91. Hgb 9.8–12.4 straddles the 11.6 g/dL phlebotomy threshold. Clears GFR and likely the nonsmoker criterion (tobacco use is historical).</x:v>
       </x:c>
     </x:row>
     <x:row r="897" ht="58" customHeight="1">
@@ -25266,7 +25266,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I897" s="9" t="str">
-        <x:v>Intervention is a 24-week wall squat programme, 3 sessions weekly, with 1-year follow-up. Patient is 91, days post open internal fixation of a displaced intertrochanteric left femoral fracture, with right hip and right knee arthroplasties, osteoarthritis, and lumbar spinal stenosis — cannot perform the intervention. Separately excluded by "diagnosed atrial fibrillation" named as an ABPM contraindication; she has AF documented with long-term antithrombotics, and the primary outcome is daytime systolic ABPM, unreliable in AF. Likely also exceeds the antihypertensive count exclusion. Note the "severe osteoarthritis pending knee replacement" criterion misses her on a literal reading — her knee replacement is already done — though its evident purpose applies squarely. Clears secondary hypertension, active malignancy (skin cancer is remote history), and consent capacity.</x:v>
+        <x:v>Intervention is a 24-week wall squat programme, 3 sessions weekly, with 1-year follow-up. Patient is 91, days post open internal fixation of a displaced intertrochanteric left femoral fracture, with right hip and right knee arthroplasties, osteoarthritis, and lumbar spinal stenosis, cannot perform the intervention. Separately excluded by "diagnosed atrial fibrillation" named as an ABPM contraindication; she has AF documented with long-term antithrombotics, and the primary outcome is daytime systolic ABPM, unreliable in AF. Likely also exceeds the antihypertensive count exclusion. Note the "severe osteoarthritis pending knee replacement" criterion misses her on a literal reading, her knee replacement is already done, though its evident purpose applies squarely. Clears secondary hypertension, active malignancy (skin cancer is remote history), and consent capacity.</x:v>
       </x:c>
     </x:row>
     <x:row r="898" ht="58" customHeight="1">
@@ -25295,7 +25295,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I898" s="9" t="str">
-        <x:v>Meets the entry diagnosis — primary hypertension with no secondary cause, creatinine 0.5–0.6, satisfying the primary_hypertension required signal. Excluded by the high-priority sleep disorder criterion: obstructive sleep apnoea is explicitly coded and is the criterion's own named example, and it would confound the Pittsburgh Sleep Quality Index primary endpoint. Also triggers "other chronic diseases" — COPD with exacerbation, atrial fibrillation with long-term antithrombotics, rheumatic mitral and tricuspid valve disease (NTproBNP 1155), osteoarthritis, lumbar spinal stenosis. Alcohol dependence in remission engages the high-priority "no history of psychiatric disorders" inclusion on a literal reading. Communication difficulties plausible given cataract, dizziness, and transient alteration of awareness against two self-completed written instruments. Tobacco use is historical, not current. Acute picture (femoral fracture with ORIF, Klebsiella, DNR) not captured by criteria but impractical for an outpatient protocol.</x:v>
+        <x:v>Meets the entry diagnosis, primary hypertension with no secondary cause, creatinine 0.5–0.6, satisfying the primary_hypertension required signal. Excluded by the high-priority sleep disorder criterion: obstructive sleep apnoea is explicitly coded and is the criterion's own named example, and it would confound the Pittsburgh Sleep Quality Index primary endpoint. Also triggers "other chronic diseases", COPD with exacerbation, atrial fibrillation with long-term antithrombotics, rheumatic mitral and tricuspid valve disease (NTproBNP 1155), osteoarthritis, lumbar spinal stenosis. Alcohol dependence in remission engages the high-priority "no history of psychiatric disorders" inclusion on a literal reading. Communication difficulties plausible given cataract, dizziness, and transient alteration of awareness against two self-completed written instruments. Tobacco use is historical, not current. Acute picture (femoral fracture with ORIF, Klebsiella, DNR) not captured by criteria but impractical for an outpatient protocol.</x:v>
       </x:c>
     </x:row>
     <x:row r="899" ht="58" customHeight="1">
@@ -25322,7 +25322,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I899" s="9" t="str">
-        <x:v>Device validation study comparing a BP monitor's AF detection against ECG — single cuff measurement plus ECG, no drug, procedure, or follow-up; lowest burden of any trial in this review. Belongs to the AF cohort outright: atrial_fibrillation clinical tag with long-term antithrombotics and INR 1.3 supporting institutional diagnosis. Meets age ≥22; no implanted pacemaker or defibrillator; not pregnant. Cooperation with cuff and ECG plausible — no dementia, delirium, or aphasia coded, and both assessments are passive and likely already routine during her admission. Medium confidence: arm circumference (22–42 cm) unmeasured, and the investigator-discretion catch-all could be invoked on general frailty grounds given DNR status, recent femoral fracture ORIF, Klebsiella infection, and COPD exacerbation — though no safety rationale supports declining.</x:v>
+        <x:v>Device validation study comparing a BP monitor's AF detection against ECG, single cuff measurement plus ECG, no drug, procedure, or follow-up; lowest burden of any trial in this review. Belongs to the AF cohort outright: atrial_fibrillation clinical tag with long-term antithrombotics and INR 1.3 supporting institutional diagnosis. Meets age ≥22; no implanted pacemaker or defibrillator; not pregnant. Cooperation with cuff and ECG plausible, no dementia, delirium, or aphasia coded, and both assessments are passive and likely already routine during her admission. Medium confidence: arm circumference (22–42 cm) unmeasured, and the investigator-discretion catch-all could be invoked on general frailty grounds given DNR status, recent femoral fracture ORIF, Klebsiella infection, and COPD exacerbation, though no safety rationale supports declining.</x:v>
       </x:c>
     </x:row>
     <x:row r="900" ht="58" customHeight="1">
@@ -25351,7 +25351,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I900" s="9" t="str">
-        <x:v>Excluded by active infection — sepsis, septicaemia, pneumonia, aspiration pneumonitis, foot cellulitis and abscess, heel and midfoot ulceration, UTI, E. coli, MSSA, penicillin-resistant organisms, WBC 4.5–15.7, neutrophils to 86% — which the protocol itself names as a major confounder of the inflammatory markers it measures. Also excluded by eGFR &lt;30: creatinine 1.3–3.6 across 39 draws, giving eGFR roughly 16–18 at 83M, with hyperkalaemia (K to 6.2); colchicine accumulates in renal impairment. Cardiogenic shock, acute respiratory failure, intubation with mechanical ventilation, acute posthaemorrhagic anaemia (Hgb nadir 8.1), and melena engage the significant-condition exclusion. Gout raises possible recent colchicine use; AF raises possible diltiazem/verapamil (named CYP3A4 exclusions). Meets the RCRI component requirement several times over (prior MI, heart failure with NTproBNP to 16,559, insulin use, creatinine &gt;2).</x:v>
+        <x:v>Excluded by active infection, sepsis, septicaemia, pneumonia, aspiration pneumonitis, foot cellulitis and abscess, heel and midfoot ulceration, UTI, E. coli, MSSA, penicillin-resistant organisms, WBC 4.5–15.7, neutrophils to 86%, which the protocol itself names as a major confounder of the inflammatory markers it measures. Also excluded by eGFR &lt;30: creatinine 1.3–3.6 across 39 draws, giving eGFR roughly 16–18 at 83M, with hyperkalaemia (K to 6.2); colchicine accumulates in renal impairment. Cardiogenic shock, acute respiratory failure, intubation with mechanical ventilation, acute posthaemorrhagic anaemia (Hgb nadir 8.1), and melena engage the significant-condition exclusion. Gout raises possible recent colchicine use; AF raises possible diltiazem/verapamil (named CYP3A4 exclusions). Meets the RCRI component requirement several times over (prior MI, heart failure with NTproBNP to 16,559, insulin use, creatinine &gt;2).</x:v>
       </x:c>
     </x:row>
     <x:row r="901" ht="58" customHeight="1">
@@ -25378,7 +25378,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I901" s="9" t="str">
-        <x:v>6-week dyadic heart failure education programme beginning within 2 weeks of discharge — no drug or procedure. Heart failure diagnosis unambiguous: clinical tag with NTproBNP 529–16,559, plus aortic stenosis, AF, CAD with chronic total occlusion, and prior subendocardial infarction; chronic substrate supports the ≥3 month requirement. Both exclusions cleanly absent — critically, the renal exclusion bars ESRD relying on HAEMODIALYSIS, and despite creatinine 1.3–3.6 he has no dialysis among 16 procedures, so CKD alone does not disqualify. Low confidence because four inclusion items are undocumented (co-residing primary caregiver, cognition via AMTS &gt;6, smartphone access, NYHA class) and discharge home is uncertain: he is in cardiogenic shock with sepsis, has required intubation and mechanical ventilation, creatinine to 3.6, Hgb nadir 8.1 with melena, and foot ulceration with cellulitis on a background of PVD. Enrolment is inherently prospective at discharge. Hong Kong site treated as logistical.</x:v>
+        <x:v>6-week dyadic heart failure education programme beginning within 2 weeks of discharge, no drug or procedure. Heart failure diagnosis unambiguous: clinical tag with NTproBNP 529–16,559, plus aortic stenosis, AF, CAD with chronic total occlusion, and prior subendocardial infarction; chronic substrate supports the ≥3 month requirement. Both exclusions cleanly absent, critically, the renal exclusion bars ESRD relying on HAEMODIALYSIS, and despite creatinine 1.3–3.6 he has no dialysis among 16 procedures, so CKD alone does not disqualify. Low confidence because four inclusion items are undocumented (co-residing primary caregiver, cognition via AMTS &gt;6, smartphone access, NYHA class) and discharge home is uncertain: he is in cardiogenic shock with sepsis, has required intubation and mechanical ventilation, creatinine to 3.6, Hgb nadir 8.1 with melena, and foot ulceration with cellulitis on a background of PVD. Enrolment is inherently prospective at discharge. Hong Kong site treated as logistical.</x:v>
       </x:c>
     </x:row>
     <x:row r="902" ht="58" customHeight="1">
@@ -25407,7 +25407,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I902" s="9" t="str">
-        <x:v>Screening study using EHR case-finding plus NT-proBNP and AI echo to detect UNDIAGNOSED heart failure. Excluded by the high-priority "previous diagnosis of heart failure — any ejection fraction of any cause": he carries a heart_failure clinical tag with NT-proBNP 529–16,559 pg/mL against the study's own 125 pg/mL action threshold, plus cardiogenic shock. Also engages the investigator-suitability exclusion given sepsis, acute respiratory failure with intubation and ventilation, creatinine to 3.6, Hgb nadir 8.1 with melena, hyperkalaemia to 6.2 — six-month survival uncertain. Notably satisfies the risk-factor inclusion six ways over (CAD with CTO and prior MI, diabetes on insulin, AF, PAD with peripheral revascularization, CKD with eGFR &lt;60, COPD with emphysema and bronchiectasis) when only two are required; only prior stroke is absent. Not on renal replacement therapy.</x:v>
+        <x:v>Screening study using EHR case-finding plus NT-proBNP and AI echo to detect UNDIAGNOSED heart failure. Excluded by the high-priority "previous diagnosis of heart failure, any ejection fraction of any cause": he carries a heart_failure clinical tag with NT-proBNP 529–16,559 pg/mL against the study's own 125 pg/mL action threshold, plus cardiogenic shock. Also engages the investigator-suitability exclusion given sepsis, acute respiratory failure with intubation and ventilation, creatinine to 3.6, Hgb nadir 8.1 with melena, hyperkalaemia to 6.2, six-month survival uncertain. Notably satisfies the risk-factor inclusion six ways over (CAD with CTO and prior MI, diabetes on insulin, AF, PAD with peripheral revascularization, CKD with eGFR &lt;60, COPD with emphysema and bronchiectasis) when only two are required; only prior stroke is absent. Not on renal replacement therapy.</x:v>
       </x:c>
     </x:row>
     <x:row r="903" ht="58" customHeight="1">
@@ -25436,7 +25436,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I903" s="9" t="str">
-        <x:v>Phase 1 CS1 CAR-T for relapsed/refractory multiple myeloma after ≥3 prior lines including proteasome inhibitor, anti-CD38, and anti-BCMA. Patient has no myeloma, no plasma cell disorder, no malignancy at all, and no oncologic therapy; no M-protein, free light chain, or marrow studies in his panel — his anaemia is iron deficiency plus acute posthaemorrhagic with melena. Also fails organ function comprehensively: ECOG 4 (cardiogenic shock, sepsis, intubation and mechanical ventilation) against required ≤1; creatinine 1.3–3.6 giving CrCl in the high teens against a ≥50 mL/min floor, with hyperkalaemia to 6.2; oxygen saturation &gt;91% on room air unmeetable in acute respiratory failure; LVEF ≥45% doubtful given NT-proBNP to 16,559. Active infection exclusion triggered by sepsis, septicaemia, pneumonia, foot cellulitis and abscess, UTI, E. coli, MSSA. Notably passes hepatic function — ALT peak 122 is ~3× ULN, under the 5× ceiling, bilirubin 0.5–0.7 normal.</x:v>
+        <x:v>Phase 1 CS1 CAR-T for relapsed/refractory multiple myeloma after ≥3 prior lines including proteasome inhibitor, anti-CD38, and anti-BCMA. Patient has no myeloma, no plasma cell disorder, no malignancy at all, and no oncologic therapy; no M-protein, free light chain, or marrow studies in his panel, his anaemia is iron deficiency plus acute posthaemorrhagic with melena. Also fails organ function comprehensively: ECOG 4 (cardiogenic shock, sepsis, intubation and mechanical ventilation) against required ≤1; creatinine 1.3–3.6 giving CrCl in the high teens against a ≥50 mL/min floor, with hyperkalaemia to 6.2; oxygen saturation &gt;91% on room air unmeetable in acute respiratory failure; LVEF ≥45% doubtful given NT-proBNP to 16,559. Active infection exclusion triggered by sepsis, septicaemia, pneumonia, foot cellulitis and abscess, UTI, E. coli, MSSA. Notably passes hepatic function, ALT peak 122 is ~3× ULN, under the 5× ceiling, bilirubin 0.5–0.7 normal.</x:v>
       </x:c>
     </x:row>
     <x:row r="904" ht="58" customHeight="1">
@@ -25465,7 +25465,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I904" s="9" t="str">
-        <x:v>Trial has only two inclusion criteria — age ≥18 and heart transplant recipient ≥3 months post-transplant. Patient has never had a transplant: no cardiac transplantation among 16 procedures, no immunosuppression, no endomyocardial biopsy, no calcineurin or mTOR drug levels in an otherwise extensive lab panel. He has the disease transplantation treats (heart failure tag, NT-proBNP to 16,559, cardiogenic shock, aortic stenosis, CAD with CTO) but not the post-transplant stage the trial enrols — and transplant candidacy is unattainable at 83 with sepsis, PVD with foot ulceration, eGFR in the high teens, and COPD. Also excluded independently by eGFR &lt;20 (creatinine 1.3–3.6, hyperkalaemia to 6.2) and active uncontrolled infection (sepsis, septicaemia, pneumonia, foot cellulitis and abscess, UTI, E. coli, MSSA) — the latter doubly relevant since SGLT2 inhibitors raise genitourinary and soft tissue infection risk in a diabetic with existing foot ulcers. Likely type 2 rather than type 1 diabetes.</x:v>
+        <x:v>Trial has only two inclusion criteria, age ≥18 and heart transplant recipient ≥3 months post-transplant. Patient has never had a transplant: no cardiac transplantation among 16 procedures, no immunosuppression, no endomyocardial biopsy, no calcineurin or mTOR drug levels in an otherwise extensive lab panel. He has the disease transplantation treats (heart failure tag, NT-proBNP to 16,559, cardiogenic shock, aortic stenosis, CAD with CTO) but not the post-transplant stage the trial enrols, and transplant candidacy is unattainable at 83 with sepsis, PVD with foot ulceration, eGFR in the high teens, and COPD. Also excluded independently by eGFR &lt;20 (creatinine 1.3–3.6, hyperkalaemia to 6.2) and active uncontrolled infection (sepsis, septicaemia, pneumonia, foot cellulitis and abscess, UTI, E. coli, MSSA), the latter doubly relevant since SGLT2 inhibitors raise genitourinary and soft tissue infection risk in a diabetic with existing foot ulcers. Likely type 2 rather than type 1 diabetes.</x:v>
       </x:c>
     </x:row>
     <x:row r="905" ht="58" customHeight="1">
@@ -25494,7 +25494,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I905" s="9" t="str">
-        <x:v>Trial enrols preoperatively for ELECTIVE major non-cardiac surgery with PCIA planned. Meets age 65–90 (83) and satisfies the risk-factor criterion ten ways over (hypertension, heart failure, CAD, AF, PAD, COPD, diabetes, CKD, anaemia, hypoalbuminaemia) when one suffices. Fails because no elective surgery is scheduled and none is schedulable: cardiogenic shock, sepsis, acute respiratory failure with intubation and mechanical ventilation. Also excluded by acute cardiovascular event within 30 days (cardiogenic shock, subendocardial infarction, troponin to 0.16, NT-proBNP to 16,559) and by inability to communicate preoperatively while ventilated — which also precludes the delirium assessments that are the primary outcome. Clean pass on the high-priority neurological/psychiatric exclusion and on the renal limb, which requires dialysis dependence rather than an eGFR threshold (creatinine 3.6 but no renal replacement therapy).</x:v>
+        <x:v>Trial enrols preoperatively for ELECTIVE major non-cardiac surgery with PCIA planned. Meets age 65–90 (83) and satisfies the risk-factor criterion ten ways over (hypertension, heart failure, CAD, AF, PAD, COPD, diabetes, CKD, anaemia, hypoalbuminaemia) when one suffices. Fails because no elective surgery is scheduled and none is schedulable: cardiogenic shock, sepsis, acute respiratory failure with intubation and mechanical ventilation. Also excluded by acute cardiovascular event within 30 days (cardiogenic shock, subendocardial infarction, troponin to 0.16, NT-proBNP to 16,559) and by inability to communicate preoperatively while ventilated, which also precludes the delirium assessments that are the primary outcome. Clean pass on the high-priority neurological/psychiatric exclusion and on the renal limb, which requires dialysis dependence rather than an eGFR threshold (creatinine 3.6 but no renal replacement therapy).</x:v>
       </x:c>
     </x:row>
     <x:row r="906" ht="58" customHeight="1">
@@ -25523,7 +25523,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I906" s="9" t="str">
-        <x:v>Allogeneic cord blood CAR-T for relapsed/refractory multiple myeloma after ≥3 regimens. No myeloma, no plasma cell disorder, no malignancy, no oncologic therapy; no M-protein, FLC, or marrow studies in his panel. Incidentally satisfies two CRAB features (creatinine to 3.6 exceeding 177 μmol/L; Hgb to 8.1 below 100 g/L) but these are diabetic/hypertensive and iron-deficiency/posthaemorrhagic in origin, not clonal. Age 83 exceeds the 18–75 ceiling (registry age_max null — 9th such discrepancy). Creatinine clearance far below the ≥60 mL/min requirement. Three exclusion blocks hit affirmatively: uncontrolled cardiovascular disease (subendocardial MI, intermediate coronary syndrome, symptomatic CHF with NT-proBNP 16,559, cardiogenic shock, AF), uncontrolled pulmonary disease (COPD, emphysema, bronchiectasis, pneumonia, aspiration pneumonitis, respiratory failure), and active uncontrolled infection (sepsis, septicaemia, foot cellulitis, UTI, E. coli, MSSA). ALT peak 122 marginally above the 3× ULN ceiling; bilirubin normal.</x:v>
+        <x:v>Allogeneic cord blood CAR-T for relapsed/refractory multiple myeloma after ≥3 regimens. No myeloma, no plasma cell disorder, no malignancy, no oncologic therapy; no M-protein, FLC, or marrow studies in his panel. Incidentally satisfies two CRAB features (creatinine to 3.6 exceeding 177 μmol/L; Hgb to 8.1 below 100 g/L) but these are diabetic/hypertensive and iron-deficiency/posthaemorrhagic in origin, not clonal. Age 83 exceeds the 18–75 ceiling (registry age_max null, 9th such discrepancy). Creatinine clearance far below the ≥60 mL/min requirement. Three exclusion blocks hit affirmatively: uncontrolled cardiovascular disease (subendocardial MI, intermediate coronary syndrome, symptomatic CHF with NT-proBNP 16,559, cardiogenic shock, AF), uncontrolled pulmonary disease (COPD, emphysema, bronchiectasis, pneumonia, aspiration pneumonitis, respiratory failure), and active uncontrolled infection (sepsis, septicaemia, foot cellulitis, UTI, E. coli, MSSA). ALT peak 122 marginally above the 3× ULN ceiling; bilirubin normal.</x:v>
       </x:c>
     </x:row>
     <x:row r="907" ht="58" customHeight="1">
@@ -25552,7 +25552,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I907" s="9" t="str">
-        <x:v>Age 83 exceeds the high-priority 18–75 window by 8 years (registry age_max null — 10th such discrepancy). Also fails "stable" chronic heart failure: cardiogenic shock, sepsis, acute respiratory failure with intubation and mechanical ventilation, hyperkalaemia to 6.2, hyponatraemia to 129, mixed acid-base disorder — though the HF diagnosis itself is unambiguous (NT-proBNP to 16,559). Acute kidney injury exclusion triggered by creatinine 1.3–3.6 across 39 draws with shock and sepsis. Active infectious disease exclusion triggered by sepsis, septicaemia, pneumonia, foot cellulitis and abscess, UTI, E. coli, MSSA — substantively decisive since the five study biomarkers (SLPI, Serpin E1, CXCL10, CXCL13, properdin) are inflammatory and complement mediators. Likely nephrotoxic drug exposure. ALT peak 122 borderline against the 3× ULN limb. Clears dialysis/kidney surgery, autoimmune disease (gout is not autoimmune), and malignancy. All three HF subtypes accepted, so missing EF is not a barrier. Contrast PAIR-000898: same trial, age 74, where only acuity failed.</x:v>
+        <x:v>Age 83 exceeds the high-priority 18–75 window by 8 years (registry age_max null, 10th such discrepancy). Also fails "stable" chronic heart failure: cardiogenic shock, sepsis, acute respiratory failure with intubation and mechanical ventilation, hyperkalaemia to 6.2, hyponatraemia to 129, mixed acid-base disorder, though the HF diagnosis itself is unambiguous (NT-proBNP to 16,559). Acute kidney injury exclusion triggered by creatinine 1.3–3.6 across 39 draws with shock and sepsis. Active infectious disease exclusion triggered by sepsis, septicaemia, pneumonia, foot cellulitis and abscess, UTI, E. coli, MSSA, substantively decisive since the five study biomarkers (SLPI, Serpin E1, CXCL10, CXCL13, properdin) are inflammatory and complement mediators. Likely nephrotoxic drug exposure. ALT peak 122 borderline against the 3× ULN limb. Clears dialysis/kidney surgery, autoimmune disease (gout is not autoimmune), and malignancy. All three HF subtypes accepted, so missing EF is not a barrier. Contrast PAIR-000898: same trial, age 74, where only acuity failed.</x:v>
       </x:c>
     </x:row>
     <x:row r="908" ht="58" customHeight="1">
@@ -25581,7 +25581,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I908" s="9" t="str">
-        <x:v>Meets age ≥60 (83), has unstable angina (intermediate coronary syndrome coded), and satisfies the eGFR &lt;90 chronic renal disease entry criterion. Fails three of the trial's five exclusions by exact diagnosis name: cardiogenic shock (coded verbatim — a direct contraindication to a hydration protocol given NT-proBNP to 16,559), severe renal failure with eGFR &lt;30 (creatinine 1.3–3.6 giving eGFR ~16–18 at 83M, with hyperkalaemia to 6.2), and respiratory failure (coded verbatim, with intubation and mechanical ventilation). Recent contrast exposure likely from femoral arteriography and aortography, engaging the within-one-week exclusion. No scheduled coronary PCI — his interventions were peripheral/non-coronary despite the pci clinical tag. Clears malignancy and contrast allergy.</x:v>
+        <x:v>Meets age ≥60 (83), has unstable angina (intermediate coronary syndrome coded), and satisfies the eGFR &lt;90 chronic renal disease entry criterion. Fails three of the trial's five exclusions by exact diagnosis name: cardiogenic shock (coded verbatim, a direct contraindication to a hydration protocol given NT-proBNP to 16,559), severe renal failure with eGFR &lt;30 (creatinine 1.3–3.6 giving eGFR ~16–18 at 83M, with hyperkalaemia to 6.2), and respiratory failure (coded verbatim, with intubation and mechanical ventilation). Recent contrast exposure likely from femoral arteriography and aortography, engaging the within-one-week exclusion. No scheduled coronary PCI, his interventions were peripheral/non-coronary despite the pci clinical tag. Clears malignancy and contrast allergy.</x:v>
       </x:c>
     </x:row>
     <x:row r="909" ht="58" customHeight="1">
@@ -25610,7 +25610,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I909" s="9" t="str">
-        <x:v>Paediatric neurodevelopment study enrolling youth aged 12–17 at Tanner stage II or above, stratified into normal-weight/normoglycaemic, obese/normoglycaemic, and obese/dysglycaemic groups, with MRI and cognitive testing at baseline and 21 months. Patient is 85 — outside by 68 years — and Tanner staging is inapplicable. Registry structured age fields are BOTH null, so no bound exists in machine-readable data (11th age-field discrepancy). Fails "otherwise healthy except for obesity": lung malignancy, DNR status, heart failure, abdominal aortic aneurysm, renal artery atherosclerosis, PVD, celiac artery compression, chronic mesenteric ischaemia, gastric ulcer with haemorrhage, anaemia (Hgb to 9). Fits none of the three study groups — BMI coded 19–24 (normal weight, with abnormal weight loss) and glucose 64–109 (normoglycaemic) despite a diabetes clinical tag. Excluded by prior cerebral infarction (neurologic comorbidity, confounds brain imaging endpoints) and depressive disorder.</x:v>
+        <x:v>Paediatric neurodevelopment study enrolling youth aged 12–17 at Tanner stage II or above, stratified into normal-weight/normoglycaemic, obese/normoglycaemic, and obese/dysglycaemic groups, with MRI and cognitive testing at baseline and 21 months. Patient is 85, outside by 68 years, and Tanner staging is inapplicable. Registry structured age fields are BOTH null, so no bound exists in machine-readable data (11th age-field discrepancy). Fails "otherwise healthy except for obesity": lung malignancy, DNR status, heart failure, abdominal aortic aneurysm, renal artery atherosclerosis, PVD, celiac artery compression, chronic mesenteric ischaemia, gastric ulcer with haemorrhage, anaemia (Hgb to 9). Fits none of the three study groups, BMI coded 19–24 (normal weight, with abnormal weight loss) and glucose 64–109 (normoglycaemic) despite a diabetes clinical tag. Excluded by prior cerebral infarction (neurologic comorbidity, confounds brain imaging endpoints) and depressive disorder.</x:v>
       </x:c>
     </x:row>
     <x:row r="910" ht="58" customHeight="1">
@@ -25639,7 +25639,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I910" s="9" t="str">
-        <x:v>Trial requires newly diagnosed untreated idiopathic intracranial hypertension per modified Dandy criteria — CSF opening pressure &gt;25 cm H2O, papilloedema, normal CSF composition — plus bilateral transverse sinus stenosis with a ≥8 mmHg gradient. Patient has none of this: no IIH, papilloedema, headache disorder, lumbar puncture, or cerebral venous imaging. Her hypertension tag denotes SYSTEMIC arterial hypertension, an unrelated condition. Demographically inverse to the IIH profile (women of childbearing age with obesity) — she is 85 with BMI coded 19–24 and abnormal weight loss. Also engages the major-comorbidity and life-expectancy exclusions: lung malignancy, DNR status, heart failure, AAA, renal artery atherosclerosis, chronic mesenteric ischaemia, gastric ulcer with haemorrhage, Hgb to 9 — against a protocol involving lumbar puncture and venous sinus stenting, with dual antiplatelet therapy hazardous in her bleeding phenotype. Prior TIA/cerebral infarction is arterial, so the venous thrombosis exclusion does not capture her. French social security requirement treated as logistical.</x:v>
+        <x:v>Trial requires newly diagnosed untreated idiopathic intracranial hypertension per modified Dandy criteria, CSF opening pressure &gt;25 cm H2O, papilloedema, normal CSF composition, plus bilateral transverse sinus stenosis with a ≥8 mmHg gradient. Patient has none of this: no IIH, papilloedema, headache disorder, lumbar puncture, or cerebral venous imaging. Her hypertension tag denotes SYSTEMIC arterial hypertension, an unrelated condition. Demographically inverse to the IIH profile (women of childbearing age with obesity), she is 85 with BMI coded 19–24 and abnormal weight loss. Also engages the major-comorbidity and life-expectancy exclusions: lung malignancy, DNR status, heart failure, AAA, renal artery atherosclerosis, chronic mesenteric ischaemia, gastric ulcer with haemorrhage, Hgb to 9, against a protocol involving lumbar puncture and venous sinus stenting, with dual antiplatelet therapy hazardous in her bleeding phenotype. Prior TIA/cerebral infarction is arterial, so the venous thrombosis exclusion does not capture her. French social security requirement treated as logistical.</x:v>
       </x:c>
     </x:row>
     <x:row r="911" ht="58" customHeight="1">
@@ -25668,7 +25668,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I911" s="9" t="str">
-        <x:v>Trial requires coronary artery disease treated with PCI, randomizing 2 hours to 5 days post-procedure. Patient has NO coronary artery disease in 32 diagnoses and no coronary intervention — her procedures are "angioplasty of other non-coronary vessel(s)" and "insertion of non-drug-eluting peripheral (non-coronary) vessel stent(s)". Atherosclerosis is peripheral, aortic, renal, and cerebral: PVD with revascularization, abdominal aneurysm, renal artery atherosclerosis, celiac artery compression, chronic mesenteric ischaemia, prior TIA/cerebral infarction. She satisfies the vascular-history and SMART risk-factor criteria several ways over, but those are additive to the CAD-plus-PCI requirement, not substitutes. Independently excluded by the high-priority cancer criterion: malignant neoplasm of bronchus and lung with solitary pulmonary nodule, within 3 years, no applicable carve-out; DNR status also engages investigator-unsuitability. Peripheral neuropathy raises the neuromuscular-disease exclusion, clinically relevant given colchicine myoneuropathy. Clears renal function (creatinine 0.5–0.6), liver function, IBD, and chronic colchicine use.</x:v>
+        <x:v>Trial requires coronary artery disease treated with PCI, randomizing 2 hours to 5 days post-procedure. Patient has NO coronary artery disease in 32 diagnoses and no coronary intervention, her procedures are "angioplasty of other non-coronary vessel(s)" and "insertion of non-drug-eluting peripheral (non-coronary) vessel stent(s)". Atherosclerosis is peripheral, aortic, renal, and cerebral: PVD with revascularization, abdominal aneurysm, renal artery atherosclerosis, celiac artery compression, chronic mesenteric ischaemia, prior TIA/cerebral infarction. She satisfies the vascular-history and SMART risk-factor criteria several ways over, but those are additive to the CAD-plus-PCI requirement, not substitutes. Independently excluded by the high-priority cancer criterion: malignant neoplasm of bronchus and lung with solitary pulmonary nodule, within 3 years, no applicable carve-out; DNR status also engages investigator-unsuitability. Peripheral neuropathy raises the neuromuscular-disease exclusion, clinically relevant given colchicine myoneuropathy. Clears renal function (creatinine 0.5–0.6), liver function, IBD, and chronic colchicine use.</x:v>
       </x:c>
     </x:row>
     <x:row r="912" ht="58" customHeight="1">
@@ -25697,7 +25697,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I912" s="9" t="str">
-        <x:v>Perinatal outpatient care trial enrolling pregnant individuals in late pregnancy and following mother-infant dyads through the first postpartum year. Patient is an 85-year-old postmenopausal woman — not pregnant and not capable of pregnancy, with no obstetric history and no infant. Notably she DOES satisfy the qualifying comorbidity list three times over (chronic hypertension, diabetes, depressive disorder), which is conjunctive with pregnancy rather than alternative to it. Entire exclusion block concerns neonatal conditions (anencephaly, gastroschisis, hypoplastic left heart, trisomy 13/18), underscoring the population. Clears the maternal seizure disorder exclusion.</x:v>
+        <x:v>Perinatal outpatient care trial enrolling pregnant individuals in late pregnancy and following mother-infant dyads through the first postpartum year. Patient is an 85-year-old postmenopausal woman, not pregnant and not capable of pregnancy, with no obstetric history and no infant. Notably she DOES satisfy the qualifying comorbidity list three times over (chronic hypertension, diabetes, depressive disorder), which is conjunctive with pregnancy rather than alternative to it. Entire exclusion block concerns neonatal conditions (anencephaly, gastroschisis, hypoplastic left heart, trisomy 13/18), underscoring the population. Clears the maternal seizure disorder exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="913" ht="58" customHeight="1">
@@ -25726,7 +25726,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I913" s="9" t="str">
-        <x:v>Trial enrols acute intracerebral haemorrhage — new deficits within 12 hours, clinical stroke signs, CT-confirmed intraparenchymal haematoma &gt;5 cc — for randomized IV antihypertensive management to a 60-minute systolic target. Patient has no ICH; her only cerebrovascular entry is personal history of TIA and cerebral infarction WITHOUT residual deficits, remote and ischaemic rather than haemorrhagic, with no brain imaging among her seven procedures. Two affirmative exclusions: do-not-resuscitate status against the high-priority "living will precludes aggressive ICU management" criterion, and previously known neoplasms (malignant neoplasm of bronchus and lung with solitary pulmonary nodule). Clears bleeding diathesis (INR 1, PT 11.4, PTT 31.3, platelets 245–296 — her gastric ulcer haemorrhage is a structural source, not a coagulopathy), platelet floor, aortic stenosis, and the clevidipine lipid-emulsion allergy exclusions. Age 18–100 met, and unusually the registry age fields match the criteria text.</x:v>
+        <x:v>Trial enrols acute intracerebral haemorrhage, new deficits within 12 hours, clinical stroke signs, CT-confirmed intraparenchymal haematoma &gt;5 cc, for randomized IV antihypertensive management to a 60-minute systolic target. Patient has no ICH; her only cerebrovascular entry is personal history of TIA and cerebral infarction WITHOUT residual deficits, remote and ischaemic rather than haemorrhagic, with no brain imaging among her seven procedures. Two affirmative exclusions: do-not-resuscitate status against the high-priority "living will precludes aggressive ICU management" criterion, and previously known neoplasms (malignant neoplasm of bronchus and lung with solitary pulmonary nodule). Clears bleeding diathesis (INR 1, PT 11.4, PTT 31.3, platelets 245–296, her gastric ulcer haemorrhage is a structural source, not a coagulopathy), platelet floor, aortic stenosis, and the clevidipine lipid-emulsion allergy exclusions. Age 18–100 met, and unusually the registry age fields match the criteria text.</x:v>
       </x:c>
     </x:row>
     <x:row r="914" ht="58" customHeight="1">
@@ -25755,7 +25755,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I914" s="9" t="str">
-        <x:v>Postpartum vascular physiology study recruiting women within 5 years of pregnancy, with or without gestational diabetes, for intradermal microdialysis assessment of endothelin-1 mediated microvascular function. Patient is 85 with no obstetric history — roughly five decades outside the enrolment window. Also triggers three exclusions affirmatively: metabolic disease including diabetes (diabetes and metabolic_disease clinical tags, though glucose 64–109 is normoglycaemic), current hypertension (hypertension tag, with antihypertensive therapy near-certain), and current tobacco use (tobacco use disorder coded as active, not historical) — all three confounding for an endothelial function endpoint. Study specifies "otherwise healthy women"; she has 32 diagnoses including lung malignancy, heart failure, and DNR status. BMI 19–24 clears the &lt;18.5 floor. NOTE: exclusion_criteria array empty in source (8th instance).</x:v>
+        <x:v>Postpartum vascular physiology study recruiting women within 5 years of pregnancy, with or without gestational diabetes, for intradermal microdialysis assessment of endothelin-1 mediated microvascular function. Patient is 85 with no obstetric history, roughly five decades outside the enrolment window. Also triggers three exclusions affirmatively: metabolic disease including diabetes (diabetes and metabolic_disease clinical tags, though glucose 64–109 is normoglycaemic), current hypertension (hypertension tag, with antihypertensive therapy near-certain), and current tobacco use (tobacco use disorder coded as active, not historical), all three confounding for an endothelial function endpoint. Study specifies "otherwise healthy women"; she has 32 diagnoses including lung malignancy, heart failure, and DNR status. BMI 19–24 clears the &lt;18.5 floor. NOTE: exclusion_criteria array empty in source (8th instance).</x:v>
       </x:c>
     </x:row>
     <x:row r="915" ht="58" customHeight="1">
@@ -25784,7 +25784,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I915" s="9" t="str">
-        <x:v>Registry of venous sinus stenting for idiopathic intracranial hypertension, MENA region. Patient has no IIH — no papilloedema, headache, lumbar puncture, raised opening pressure, or venous sinus stenosis, and no brain imaging or venography among her seven procedures. Her hypertension tag denotes SYSTEMIC arterial hypertension; her glaucoma is intraocular, not papilloedema. Independently fails the high-priority 18–60 age window by 25 years (registry age_max null — 12th such discrepancy). Also engages the severe-comorbidity exclusion for endovascular procedures: lung malignancy, DNR status, heart failure, AAA, renal artery atherosclerosis, PVD, chronic mesenteric ischaemia, Hgb 9–11.9. Chronic gastric ulcer with haemorrhage on long-term aspirin raises the antiplatelet contraindication limb, mandatory after sinus stenting — though coagulation itself is normal (INR 1, platelets 245–296). Second IIH trial paired to this patient after PAIR-000965.</x:v>
+        <x:v>Registry of venous sinus stenting for idiopathic intracranial hypertension, MENA region. Patient has no IIH, no papilloedema, headache, lumbar puncture, raised opening pressure, or venous sinus stenosis, and no brain imaging or venography among her seven procedures. Her hypertension tag denotes SYSTEMIC arterial hypertension; her glaucoma is intraocular, not papilloedema. Independently fails the high-priority 18–60 age window by 25 years (registry age_max null, 12th such discrepancy). Also engages the severe-comorbidity exclusion for endovascular procedures: lung malignancy, DNR status, heart failure, AAA, renal artery atherosclerosis, PVD, chronic mesenteric ischaemia, Hgb 9–11.9. Chronic gastric ulcer with haemorrhage on long-term aspirin raises the antiplatelet contraindication limb, mandatory after sinus stenting, though coagulation itself is normal (INR 1, platelets 245–296). Second IIH trial paired to this patient after PAIR-000965.</x:v>
       </x:c>
     </x:row>
     <x:row r="916" ht="58" customHeight="1">
@@ -25813,7 +25813,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I916" s="9" t="str">
-        <x:v>Cross-sectional diet, cardiometabolic marker, and gut microbiota study in Singapore adults aged 21–80. Patient is 85, five years past the ceiling; registry age fields both null (13th age-field discrepancy). Also likely fails the "no drastic change of diet for the past 1 year" criterion — abnormal weight loss coded, with chronic vascular insufficiency of intestine and celiac artery compression syndrome causing postprandial pain and food avoidance, plus gastric ulcer with haemorrhage and active lung malignancy; BMI coded 19–24 at the lower end. Medication-consistency requirement (&gt;5 years of antihypertensive/statin/antidiabetic) unverifiable with an empty medication field. Clears venous access and consent capacity. Beyond the criteria: her mesenteric ischaemia, diverticulosis, gastric ulceration, gastritis, and reflux would make her microbiome unrepresentative of the dietary associations under study. Singapore site treated as logistical.</x:v>
+        <x:v>Cross-sectional diet, cardiometabolic marker, and gut microbiota study in Singapore adults aged 21–80. Patient is 85, five years past the ceiling; registry age fields both null (13th age-field discrepancy). Also likely fails the "no drastic change of diet for the past 1 year" criterion, abnormal weight loss coded, with chronic vascular insufficiency of intestine and celiac artery compression syndrome causing postprandial pain and food avoidance, plus gastric ulcer with haemorrhage and active lung malignancy; BMI coded 19–24 at the lower end. Medication-consistency requirement (&gt;5 years of antihypertensive/statin/antidiabetic) unverifiable with an empty medication field. Clears venous access and consent capacity. Beyond the criteria: her mesenteric ischaemia, diverticulosis, gastric ulceration, gastritis, and reflux would make her microbiome unrepresentative of the dietary associations under study. Singapore site treated as logistical.</x:v>
       </x:c>
     </x:row>
     <x:row r="917" ht="58" customHeight="1">
@@ -25842,7 +25842,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I917" s="9" t="str">
-        <x:v>Trial enrols sedentary pregnant women at 20–24 weeks gestation, aged 18–45, for an 8-week mobile exercise app intervention with FMD, HRV, and PWV outcomes. Patient is 85 and not pregnant — 40 years past the ceiling with no obstetric history. Registry structured age fields read NO MINIMUM with a MAXIMUM OF 90, which would admit her to a pregnancy study (14th age-field discrepancy, and the first where the structured max exceeds the stated ceiling rather than being absent). Also excluded by physician-diagnosed cardiovascular disease (heart failure, hypertension, PVD, AAA, renal artery atherosclerosis, cardiac murmurs, prior TIA/infarction) and metabolic disease (diabetes, metabolic_disease tags, adrenal disorders) — both confounding for vascular function endpoints — plus likely vasoactive medication use and active tobacco use disorder within 3 months. Fails "generally healthy" given lung malignancy and DNR status.</x:v>
+        <x:v>Trial enrols sedentary pregnant women at 20–24 weeks gestation, aged 18–45, for an 8-week mobile exercise app intervention with FMD, HRV, and PWV outcomes. Patient is 85 and not pregnant, 40 years past the ceiling with no obstetric history. Registry structured age fields read NO MINIMUM with a MAXIMUM OF 90, which would admit her to a pregnancy study (14th age-field discrepancy, and the first where the structured max exceeds the stated ceiling rather than being absent). Also excluded by physician-diagnosed cardiovascular disease (heart failure, hypertension, PVD, AAA, renal artery atherosclerosis, cardiac murmurs, prior TIA/infarction) and metabolic disease (diabetes, metabolic_disease tags, adrenal disorders), both confounding for vascular function endpoints, plus likely vasoactive medication use and active tobacco use disorder within 3 months. Fails "generally healthy" given lung malignancy and DNR status.</x:v>
       </x:c>
     </x:row>
     <x:row r="918" ht="58" customHeight="1">
@@ -25871,7 +25871,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I918" s="9" t="str">
-        <x:v>Observational registry with one substantive inclusion criterion — patients who received rotational atherectomy — and required signal rotational_atherectomy. No coronary atherectomy or coronary intervention in her 12 procedures. Coronary work was diagnostic only (arteriography with two catheters, fluoroscopy of multiple coronary arteries, combined right and left heart catheterisation); therapeutic procedures were peripheral (right femoral dilation with intraluminal devices, extirpation of matter percutaneous and open, peripheral thrombolytic) or valvular (percutaneous aortic valve replacement with zooplastic tissue). CAD coded as atherosclerotic heart disease without angina pectoris. Not a plausible future prospect at 93 with DNR status coded twice, myasthenia gravis with exacerbation, PVD with rest pain, and Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia. Sole exclusion — life expectancy &lt;1 year — also likely met. Guardian consent permitted, so her mild cognitive impairment is not the barrier.</x:v>
+        <x:v>Observational registry with one substantive inclusion criterion, patients who received rotational atherectomy, and required signal rotational_atherectomy. No coronary atherectomy or coronary intervention in her 12 procedures. Coronary work was diagnostic only (arteriography with two catheters, fluoroscopy of multiple coronary arteries, combined right and left heart catheterisation); therapeutic procedures were peripheral (right femoral dilation with intraluminal devices, extirpation of matter percutaneous and open, peripheral thrombolytic) or valvular (percutaneous aortic valve replacement with zooplastic tissue). CAD coded as atherosclerotic heart disease without angina pectoris. Not a plausible future prospect at 93 with DNR status coded twice, myasthenia gravis with exacerbation, PVD with rest pain, and Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia. Sole exclusion, life expectancy &lt;1 year, also likely met. Guardian consent permitted, so her mild cognitive impairment is not the barrier.</x:v>
       </x:c>
     </x:row>
     <x:row r="919" ht="58" customHeight="1">
@@ -25900,7 +25900,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I919" s="9" t="str">
-        <x:v>CAD explicitly coded "without angina pectoris," failing the symptomatic angina with objective ischemia requirement affirmatively. No coronary stent or intervention — coronary procedures were diagnostic (arteriography with two catheters, fluoroscopy of multiple coronary arteries, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement; therapeutic arterial procedures were all right femoral. Life expectancy &lt;2 years likely against a 2-year TVF endpoint: age 93, DNR status coded twice, myasthenia gravis with exacerbation, Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia requiring endoscopic control, PVD with rest pain. Antiplatelet contraindication concern from the same bleeding history despite documented long-term aspirin use. Notably clears the CABG exclusion (TAVR is structural, not bypass) and the coronary CTO lesion exclusion — her chronic total occlusion is of an EXTREMITY artery, not coronary. Mirrors PAIR-000853, where the same trial failed a different patient on identical non-anginal coding.</x:v>
+        <x:v>CAD explicitly coded "without angina pectoris," failing the symptomatic angina with objective ischemia requirement affirmatively. No coronary stent or intervention, coronary procedures were diagnostic (arteriography with two catheters, fluoroscopy of multiple coronary arteries, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement; therapeutic arterial procedures were all right femoral. Life expectancy &lt;2 years likely against a 2-year TVF endpoint: age 93, DNR status coded twice, myasthenia gravis with exacerbation, Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia requiring endoscopic control, PVD with rest pain. Antiplatelet contraindication concern from the same bleeding history despite documented long-term aspirin use. Notably clears the CABG exclusion (TAVR is structural, not bypass) and the coronary CTO lesion exclusion, her chronic total occlusion is of an EXTREMITY artery, not coronary. Mirrors PAIR-000853, where the same trial failed a different patient on identical non-anginal coding.</x:v>
       </x:c>
     </x:row>
     <x:row r="920" ht="58" customHeight="1">
@@ -25929,7 +25929,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I920" s="9" t="str">
-        <x:v>Trial randomizes intravascular lithotripsy vs PTA to prepare hostile ilio-femoral access DURING transfemoral TAVI. Patient has already had TAVI — replacement of aortic valve with zooplastic tissue percutaneously, with presence of prosthetic heart valve and presence of other heart-valve replacement coded — so severe aortic stenosis is treated and no valve implantation is upcoming. Also triggers the high-priority index-limb exclusion: right femoral artery dilated with intraluminal devices twice, extirpation of matter percutaneous and open, thrombolytic infusion, with peripheral stent stenosis coded as initial encounter. Active infection exclusion met (pneumonia, acute bronchitis, upper respiratory infection, neutrophils to 90%). Life expectancy &lt;1 year likely (age 93, DNR coded twice, myasthenia gravis with exacerbation, Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia). STS score almost certainly ≥8%. Her peripheral disease and limb_artery_disease required signal are genuine — the substrate is right, the timing is not.</x:v>
+        <x:v>Trial randomizes intravascular lithotripsy vs PTA to prepare hostile ilio-femoral access DURING transfemoral TAVI. Patient has already had TAVI, replacement of aortic valve with zooplastic tissue percutaneously, with presence of prosthetic heart valve and presence of other heart-valve replacement coded, so severe aortic stenosis is treated and no valve implantation is upcoming. Also triggers the high-priority index-limb exclusion: right femoral artery dilated with intraluminal devices twice, extirpation of matter percutaneous and open, thrombolytic infusion, with peripheral stent stenosis coded as initial encounter. Active infection exclusion met (pneumonia, acute bronchitis, upper respiratory infection, neutrophils to 90%). Life expectancy &lt;1 year likely (age 93, DNR coded twice, myasthenia gravis with exacerbation, Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia). STS score almost certainly ≥8%. Her peripheral disease and limb_artery_disease required signal are genuine, the substrate is right, the timing is not.</x:v>
       </x:c>
     </x:row>
     <x:row r="921" ht="58" customHeight="1">
@@ -25958,7 +25958,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I921" s="9" t="str">
-        <x:v>Six-week randomized dietary trial (lean grain-fed beef, grass-fed beef, or plant-based meat) in healthy adults aged 18–45 with metabolic, inflammatory, and gut microbiome outcomes. Patient is 93 — 48 years past the ceiling on a high-priority criterion; registry age fields both null (15th such discrepancy). Also excluded by gastrointestinal disease: GI haemorrhage, angiodysplasia of stomach and duodenum with bleeding, benign gastric neoplasm, diaphragmatic hernia, GERD, pancreatic cyst, abnormal stool findings, with endoscopic control of bleeding and upper GI therapeutic endoscopy — confounding for a microbiome endpoint. Excluded by drug therapy for CAD, PAD, and CHF (all three documented, with long-term aspirin and antithrombotics coded). Recent antibiotics likely given pneumonia, bronchitis, and URI. Diet and weight stability implausible given Hgb nadir 4.8 with acute posthaemorrhagic anaemia. Clean passes: no diabetes (HbA1c 6.2, glucose 71–139, no diabetes tag), no uncontrolled hypertension (hypotension coded instead), non-smoker (tobacco use historical).</x:v>
+        <x:v>Six-week randomized dietary trial (lean grain-fed beef, grass-fed beef, or plant-based meat) in healthy adults aged 18–45 with metabolic, inflammatory, and gut microbiome outcomes. Patient is 93, 48 years past the ceiling on a high-priority criterion; registry age fields both null (15th such discrepancy). Also excluded by gastrointestinal disease: GI haemorrhage, angiodysplasia of stomach and duodenum with bleeding, benign gastric neoplasm, diaphragmatic hernia, GERD, pancreatic cyst, abnormal stool findings, with endoscopic control of bleeding and upper GI therapeutic endoscopy, confounding for a microbiome endpoint. Excluded by drug therapy for CAD, PAD, and CHF (all three documented, with long-term aspirin and antithrombotics coded). Recent antibiotics likely given pneumonia, bronchitis, and URI. Diet and weight stability implausible given Hgb nadir 4.8 with acute posthaemorrhagic anaemia. Clean passes: no diabetes (HbA1c 6.2, glucose 71–139, no diabetes tag), no uncontrolled hypertension (hypotension coded instead), non-smoker (tobacco use historical).</x:v>
       </x:c>
     </x:row>
     <x:row r="922" ht="58" customHeight="1">
@@ -25987,7 +25987,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I922" s="9" t="str">
-        <x:v>Age 93 exceeds the high-priority ≤75 ceiling by 18 years. Registry structured age field reads min 4 / no maximum — third flagging of this same trial's age field (after PAIR-000856 and 000891), 16th age-field discrepancy overall. Blood pressure runs the wrong way: trial requires office SBP ≥150 and DBP ≥90, and hypotension unspecified is affirmatively coded alongside abnormality of gait and history of falling, which also raise the orthostatic hypotension exclusion. Life expectancy &lt;1 year likely and investigator-unsuitability engaged: DNR status coded twice, myasthenia gravis with exacerbation, Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia requiring endoscopic control, pneumonia, PVD with rest pain, mild cognitive impairment. eGFR borderline against the &lt;45 exclusion (creatinine 0.6–1.2 at 93F). Three hypothyroidism entries raise suspected secondary hypertension. Clean passes: no Type 1 diabetes (no diabetes at all, HbA1c 6.2), no contrast allergy, no prior renal denervation.</x:v>
+        <x:v>Age 93 exceeds the high-priority ≤75 ceiling by 18 years. Registry structured age field reads min 4 / no maximum, third flagging of this same trial's age field (after PAIR-000856 and 000891), 16th age-field discrepancy overall. Blood pressure runs the wrong way: trial requires office SBP ≥150 and DBP ≥90, and hypotension unspecified is affirmatively coded alongside abnormality of gait and history of falling, which also raise the orthostatic hypotension exclusion. Life expectancy &lt;1 year likely and investigator-unsuitability engaged: DNR status coded twice, myasthenia gravis with exacerbation, Hgb 4.8–12.6 with GI haemorrhage and angiodysplasia requiring endoscopic control, pneumonia, PVD with rest pain, mild cognitive impairment. eGFR borderline against the &lt;45 exclusion (creatinine 0.6–1.2 at 93F). Three hypothyroidism entries raise suspected secondary hypertension. Clean passes: no Type 1 diabetes (no diabetes at all, HbA1c 6.2), no contrast allergy, no prior renal denervation.</x:v>
       </x:c>
     </x:row>
     <x:row r="923" ht="58" customHeight="1">
@@ -26016,7 +26016,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I923" s="9" t="str">
-        <x:v>Age 93 exceeds the high-priority &lt;80 ceiling by 13 years; registry age fields both null (17th such discrepancy). Trial randomizes intra-procedurally during PCI, requiring DES indication, OCT calcium arc ≥270°, and a failed non-compliant balloon preparation — none has occurred. Her coronary procedures were diagnostic (arteriography with two catheters, coronary fluoroscopy, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement; therapeutic arterial procedures were right femoral. Also excluded by active autoimmune disease: myasthenia gravis WITH EXACERBATION explicitly coded — an autoantibody-mediated disorder in its active phase. DAPT intolerance concern from GI haemorrhage, angiodysplasia with bleeding, and Hgb nadir 4.8 despite documented long-term antiplatelet use. Coronary calcification not specifically coded, unlike the patient at PAIR-000857. Clears contrast allergy, STEMI, and cardiogenic shock.</x:v>
+        <x:v>Age 93 exceeds the high-priority &lt;80 ceiling by 13 years; registry age fields both null (17th such discrepancy). Trial randomizes intra-procedurally during PCI, requiring DES indication, OCT calcium arc ≥270°, and a failed non-compliant balloon preparation, none has occurred. Her coronary procedures were diagnostic (arteriography with two catheters, coronary fluoroscopy, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement; therapeutic arterial procedures were right femoral. Also excluded by active autoimmune disease: myasthenia gravis WITH EXACERBATION explicitly coded, an autoantibody-mediated disorder in its active phase. DAPT intolerance concern from GI haemorrhage, angiodysplasia with bleeding, and Hgb nadir 4.8 despite documented long-term antiplatelet use. Coronary calcification not specifically coded, unlike the patient at PAIR-000857. Clears contrast allergy, STEMI, and cardiogenic shock.</x:v>
       </x:c>
     </x:row>
     <x:row r="924" ht="58" customHeight="1">
@@ -26045,7 +26045,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I924" s="9" t="str">
-        <x:v>Device feasibility study of SoniCracker IVL delivered during elective/planned PCI with at least moderate coronary calcification. Patient is not undergoing PCI — coronary procedures were diagnostic (arteriography with two catheters, coronary fluoroscopy, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement; therapeutic arterial procedures were right femoral. Coronary calcification is not documented, so the calcified_coronary_lesion required signal is unsupported, and no IVUS or OCT exists to assess the 180° arc criterion. Notably clears the age criterion — this protocol has no ceiling, unlike her three preceding pairs. Excluded by significant co-morbidities and investigator unsuitability: DNR coded twice, myasthenia gravis with exacerbation, heart failure with NT-proBNP to 2494, PVD with rest pain, GI haemorrhage with Hgb 4.8 and Hct 15.3, pneumonia. Consent capacity uncertain given mild cognitive impairment, with no guardian provision in this protocol.</x:v>
+        <x:v>Device feasibility study of SoniCracker IVL delivered during elective/planned PCI with at least moderate coronary calcification. Patient is not undergoing PCI, coronary procedures were diagnostic (arteriography with two catheters, coronary fluoroscopy, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement; therapeutic arterial procedures were right femoral. Coronary calcification is not documented, so the calcified_coronary_lesion required signal is unsupported, and no IVUS or OCT exists to assess the 180° arc criterion. Notably clears the age criterion, this protocol has no ceiling, unlike her three preceding pairs. Excluded by significant co-morbidities and investigator unsuitability: DNR coded twice, myasthenia gravis with exacerbation, heart failure with NT-proBNP to 2494, PVD with rest pain, GI haemorrhage with Hgb 4.8 and Hct 15.3, pneumonia. Consent capacity uncertain given mild cognitive impairment, with no guardian provision in this protocol.</x:v>
       </x:c>
     </x:row>
     <x:row r="925" ht="58" customHeight="1">
@@ -26074,7 +26074,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I925" s="9" t="str">
-        <x:v>Trial compares 3DStent angiographic tool against intracoronary IVUS for quantifying coronary calcification; required signals are ivus and calcified_coronary_lesion, and she has neither. No IVUS among her 12 procedures; coronary work was diagnostic (arteriography with two catheters, coronary fluoroscopy, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement. Coronary calcification not documented anywhere — her coronary coding is atherosclerotic heart disease without angina pectoris — so unlike PAIR-000860, where the patient had a coded calcified coronary lesion, here the substrate is absent as well as the procedure. No designated culprit lesion. Mild cognitive impairment with dysarthria raises the EU vulnerable-adult exclusion for adults unable to express consent, though no guardianship is documented and the impairment is characterised as mild. BMI unassessable (undocumented) against the &gt;35 exclusion. Clears STEMI and cardiogenic shock. Age has no ceiling in this protocol. French social security requirement treated as logistical.</x:v>
+        <x:v>Trial compares 3DStent angiographic tool against intracoronary IVUS for quantifying coronary calcification; required signals are ivus and calcified_coronary_lesion, and she has neither. No IVUS among her 12 procedures; coronary work was diagnostic (arteriography with two catheters, coronary fluoroscopy, combined right and left heart catheterisation) and led to percutaneous aortic valve replacement. Coronary calcification not documented anywhere, her coronary coding is atherosclerotic heart disease without angina pectoris, so unlike PAIR-000860, where the patient had a coded calcified coronary lesion, here the substrate is absent as well as the procedure. No designated culprit lesion. Mild cognitive impairment with dysarthria raises the EU vulnerable-adult exclusion for adults unable to express consent, though no guardianship is documented and the impairment is characterised as mild. BMI unassessable (undocumented) against the &gt;35 exclusion. Clears STEMI and cardiogenic shock. Age has no ceiling in this protocol. French social security requirement treated as logistical.</x:v>
       </x:c>
     </x:row>
     <x:row r="926" ht="58" customHeight="1">
@@ -26101,7 +26101,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I926" s="9" t="str">
-        <x:v>Strong cardiorenal fit — heart_failure clinical tag with structural basis (mitral valve disorders with ruptured chordae tendineae, tricuspid valve disease, hypoxemia, s/p mitral valvuloplasty with annuloplasty) plus chronic_kidney_disease tag; both required signals supported on the cardiorenal side. Age 54, cognitively intact, consent unproblematic. eGFR clears the ≥15 floor comfortably (creatinine 1–1.9 at 54M). All stated exclusions absent: normal liver function (ALT 10–36, AST 20–33, bilirubin 1–1.2, albumin 3.8–4.3) so no hepatorenal syndrome, no kidney malformation, not pregnant. Medium confidence pending two items: loop diuretic dose ≥40 mg/day furosemide undocumented but clinically probable (potassium 3.1–4.3 suggestive), and MR conditionality of the mitral annuloplasty ring, possible LAA clip, and discontinued temporary pacing wires — though the imaging target is the kidneys, remote from all hardware. Visit 2 hypokalaemia threshold (K &lt;3.5) is borderline given values to 3.1; does not affect visit 1. Recent post-op course means visit scheduling awaits outpatient recovery. Ontario site treated as logistical.</x:v>
+        <x:v>Strong cardiorenal fit, heart_failure clinical tag with structural basis (mitral valve disorders with ruptured chordae tendineae, tricuspid valve disease, hypoxemia, s/p mitral valvuloplasty with annuloplasty) plus chronic_kidney_disease tag; both required signals supported on the cardiorenal side. Age 54, cognitively intact, consent unproblematic. eGFR clears the ≥15 floor comfortably (creatinine 1–1.9 at 54M). All stated exclusions absent: normal liver function (ALT 10–36, AST 20–33, bilirubin 1–1.2, albumin 3.8–4.3) so no hepatorenal syndrome, no kidney malformation, not pregnant. Medium confidence pending two items: loop diuretic dose ≥40 mg/day furosemide undocumented but clinically probable (potassium 3.1–4.3 suggestive), and MR conditionality of the mitral annuloplasty ring, possible LAA clip, and discontinued temporary pacing wires, though the imaging target is the kidneys, remote from all hardware. Visit 2 hypokalaemia threshold (K &lt;3.5) is borderline given values to 3.1; does not affect visit 1. Recent post-op course means visit scheduling awaits outpatient recovery. Ontario site treated as logistical.</x:v>
       </x:c>
     </x:row>
     <x:row r="927" ht="58" customHeight="1">
@@ -26130,7 +26130,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I927" s="9" t="str">
-        <x:v>Has the chronic substrate — heart_failure tag with mitral valve disorders, ruptured chordae, tricuspid valve disease; chronic_kidney_disease tag with creatinine 1–1.9 (eGFR ~40, CKD 3b) fitting "moderate to advanced." Clears EVERY stated exclusion cleanly: normal LFTs (ALT 10–36, AST 20–33, alk phos 37–43), no diabetes of any type (HbA1c 5.7–5.9, no diabetes tag), no dialysis, no GI disorder, no genitourinary infection (the concern that decided PAIR-000894), male. Protocol explicitly permits acute creatinine rise. Fails on admission state: his hospitalisation is a completed elective mitral valvuloplasty with annuloplasty, LAA exclusion, and ablation on cardiopulmonary bypass, not an ADHF decompensation; hypervolaemia not coded and no natriuretic peptide in his panel. General safety exclusion engaged by perioperative SGLT2 inhibitor initiation (euglycaemic DKA risk post-bypass), with Hgb 9.4–14, platelets 112–290, INR to 2.2. Time-limited rather than categorical — strong candidate if later readmitted decompensated.</x:v>
+        <x:v>Has the chronic substrate, heart_failure tag with mitral valve disorders, ruptured chordae, tricuspid valve disease; chronic_kidney_disease tag with creatinine 1–1.9 (eGFR ~40, CKD 3b) fitting "moderate to advanced." Clears EVERY stated exclusion cleanly: normal LFTs (ALT 10–36, AST 20–33, alk phos 37–43), no diabetes of any type (HbA1c 5.7–5.9, no diabetes tag), no dialysis, no GI disorder, no genitourinary infection (the concern that decided PAIR-000894), male. Protocol explicitly permits acute creatinine rise. Fails on admission state: his hospitalisation is a completed elective mitral valvuloplasty with annuloplasty, LAA exclusion, and ablation on cardiopulmonary bypass, not an ADHF decompensation; hypervolaemia not coded and no natriuretic peptide in his panel. General safety exclusion engaged by perioperative SGLT2 inhibitor initiation (euglycaemic DKA risk post-bypass), with Hgb 9.4–14, platelets 112–290, INR to 2.2. Time-limited rather than categorical, strong candidate if later readmitted decompensated.</x:v>
       </x:c>
     </x:row>
     <x:row r="928" ht="58" customHeight="1">
@@ -26159,7 +26159,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I928" s="9" t="str">
-        <x:v>Phase 2 trial of home self-administered subcutaneous elranatamab in relapsed multiple myeloma with prior proteasome inhibitor, IMiD, and anti-CD38 exposure. Patient has no myeloma, no plasma cell disorder, no malignancy, and no oncologic therapy; no M-protein, free light chain, or marrow studies in his panel. His anaemia (Hgb 9.4–14) and creatinine 1–1.9 are explained by cardiopulmonary bypass and cardiorenal physiology, not CRAB criteria. All 21 procedures are cardiac and perioperative. Clears every stated exclusion — no prior malignancy, no ICANS history, no plasma cell leukaemia or amyloidosis, no viral hepatitis or HIV, male, and no barrier to electronic PRO entry. Recent bypass surgery engages the general significant-medical-condition exclusion.</x:v>
+        <x:v>Phase 2 trial of home self-administered subcutaneous elranatamab in relapsed multiple myeloma with prior proteasome inhibitor, IMiD, and anti-CD38 exposure. Patient has no myeloma, no plasma cell disorder, no malignancy, and no oncologic therapy; no M-protein, free light chain, or marrow studies in his panel. His anaemia (Hgb 9.4–14) and creatinine 1–1.9 are explained by cardiopulmonary bypass and cardiorenal physiology, not CRAB criteria. All 21 procedures are cardiac and perioperative. Clears every stated exclusion, no prior malignancy, no ICANS history, no plasma cell leukaemia or amyloidosis, no viral hepatitis or HIV, male, and no barrier to electronic PRO entry. Recent bypass surgery engages the general significant-medical-condition exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="929" ht="58" customHeight="1">
@@ -26188,7 +26188,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I929" s="9" t="str">
-        <x:v>68Ga-DOTATATE PET/MRI study requiring molecularly confirmed Fabry disease (documented enzyme deficiency in males) plus cardiac MRI within 3 years showing Fabry cardiac involvement. Patient has no Fabry disease, GLA mutation, or enzyme testing, and none of the multisystem features; his heart failure is structural — mitral valve disorders with ruptured chordae tendineae and tricuspid valve disease, surgically repaired by valvuloplasty with annuloplasty. No cardiac MRI among his 21 procedures. Renal limb of the gadolinium exclusion does not apply (creatinine 1–1.9, eGFR ~40, above the 30 threshold), but the MRI limb is a real concern here unlike PAIR-000984: the imaging target is the myocardium and his annuloplasty ring, possible LAA clip, and recently removed pacing wires sit directly in the field of view. AF status post surgical ablation and LAA exclusion is unrecorded; AF would also degrade ECG-gated cardiac PET/MRI. Clears myocarditis, prior gene therapy, and pregnancy exclusions.</x:v>
+        <x:v>68Ga-DOTATATE PET/MRI study requiring molecularly confirmed Fabry disease (documented enzyme deficiency in males) plus cardiac MRI within 3 years showing Fabry cardiac involvement. Patient has no Fabry disease, GLA mutation, or enzyme testing, and none of the multisystem features; his heart failure is structural, mitral valve disorders with ruptured chordae tendineae and tricuspid valve disease, surgically repaired by valvuloplasty with annuloplasty. No cardiac MRI among his 21 procedures. Renal limb of the gadolinium exclusion does not apply (creatinine 1–1.9, eGFR ~40, above the 30 threshold), but the MRI limb is a real concern here unlike PAIR-000984: the imaging target is the myocardium and his annuloplasty ring, possible LAA clip, and recently removed pacing wires sit directly in the field of view. AF status post surgical ablation and LAA exclusion is unrecorded; AF would also degrade ECG-gated cardiac PET/MRI. Clears myocarditis, prior gene therapy, and pregnancy exclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="930" ht="58" customHeight="1">
@@ -26217,7 +26217,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I930" s="9" t="str">
-        <x:v>Trial enrols non-valvular, non-paroxysmal AF with recurrent atrial arrhythmia after a first CATHETER ablation. Patient fails on all three qualifiers: his AF is valvular (mitral valve disorders with ruptured chordae tendineae, tricuspid valve disease); his ablation was a concomitant surgical procedure performed during open heart valve repair on cardiopulmonary bypass, not a standalone catheter ablation; and post-ablation recurrence is undocumented. Triggers the high-priority "previous cardiac surgery" exclusion — open heart mitral valvuloplasty with annuloplasty, LAA exclusion, extracorporeal circulation; the named examples are bypass and valve replacement but the governing phrase is previous cardiac surgery. Left atrial diameter ≥50 mm likely given surgical mitral regurgitation. Clears renal (creatinine 1–1.9, eGFR ~40) and hepatic exclusions, and no cardiomyopathy. Thyroid history unclear and relevant given amiodarone. "Examination of participant in clinical trial" coded, raising the concurrent-trial exclusion.</x:v>
+        <x:v>Trial enrols non-valvular, non-paroxysmal AF with recurrent atrial arrhythmia after a first CATHETER ablation. Patient fails on all three qualifiers: his AF is valvular (mitral valve disorders with ruptured chordae tendineae, tricuspid valve disease); his ablation was a concomitant surgical procedure performed during open heart valve repair on cardiopulmonary bypass, not a standalone catheter ablation; and post-ablation recurrence is undocumented. Triggers the high-priority "previous cardiac surgery" exclusion, open heart mitral valvuloplasty with annuloplasty, LAA exclusion, extracorporeal circulation; the named examples are bypass and valve replacement but the governing phrase is previous cardiac surgery. Left atrial diameter ≥50 mm likely given surgical mitral regurgitation. Clears renal (creatinine 1–1.9, eGFR ~40) and hepatic exclusions, and no cardiomyopathy. Thyroid history unclear and relevant given amiodarone. "Examination of participant in clinical trial" coded, raising the concurrent-trial exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="931" ht="58" customHeight="1">
@@ -26244,7 +26244,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I931" s="9" t="str">
-        <x:v>Non-invasive VExUS ultrasound-guided decongestion vs standard care in ADHF; no drug or procedure, four inclusion criteria and one discretionary exclusion. Clinical picture fits — rupture of chordae tendineae causes acute severe mitral regurgitation presenting as pulmonary congestion, with hypoxemia coded, heart_failure tag, tricuspid valve disease, and creatinine 1–1.9 suggesting cardiorenal involvement. Age 54 and consent capacity clear. Low confidence on two counts: NO NT-proBNP anywhere in his panel, leaving the &gt;800 ng/L entry gate and the elevated_bnp required signal unverifiable (contrast PAIR-000896, where NT-proBNP 3062 cleared it fourfold); and his documented course is operative (mitral valvuloplasty with annuloplasty, LAA exclusion, ablation, CPB), so admission may have been under cardiothoracic surgery rather than the cardiology ward named in the criterion, meaning the at-admission enrolment window may not apply. Sole exclusion is investigator discretion and no safety rationale supports invoking it for a bedside ultrasound; potassium 3.1 worth noting under the study's electrolyte safety focus. Oslo site treated as logistical.</x:v>
+        <x:v>Non-invasive VExUS ultrasound-guided decongestion vs standard care in ADHF; no drug or procedure, four inclusion criteria and one discretionary exclusion. Clinical picture fits, rupture of chordae tendineae causes acute severe mitral regurgitation presenting as pulmonary congestion, with hypoxemia coded, heart_failure tag, tricuspid valve disease, and creatinine 1–1.9 suggesting cardiorenal involvement. Age 54 and consent capacity clear. Low confidence on two counts: NO NT-proBNP anywhere in his panel, leaving the &gt;800 ng/L entry gate and the elevated_bnp required signal unverifiable (contrast PAIR-000896, where NT-proBNP 3062 cleared it fourfold); and his documented course is operative (mitral valvuloplasty with annuloplasty, LAA exclusion, ablation, CPB), so admission may have been under cardiothoracic surgery rather than the cardiology ward named in the criterion, meaning the at-admission enrolment window may not apply. Sole exclusion is investigator discretion and no safety rationale supports invoking it for a bedside ultrasound; potassium 3.1 worth noting under the study's electrolyte safety focus. Oslo site treated as logistical.</x:v>
       </x:c>
     </x:row>
     <x:row r="932" ht="58" customHeight="1">
@@ -26302,7 +26302,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I933" s="9" t="str">
-        <x:v>First patient assessed against this trial to clear the 18–75 age window (54). Has the cardiorenal substrate — heart_failure and chronic_kidney_disease tags supporting the cardiorenal_syndrome required signal — and all three HF subtypes are accepted, so the missing EF is not a barrier. Fails the "stable chronic" requirement: his heart failure is acute valvular, from rupture of chordae tendineae producing severe mitral regurgitation, repaired days ago by open valvuloplasty with annuloplasty on cardiopulmonary bypass, with Hgb 9.4–14, platelets 112–290, INR to 2.2, potassium 3.1. Likely AKI within 3 months (creatinine 1–1.9 near-doubling post-bypass, hyaline casts 2–32/lpf). Clears every high-priority exclusion — no dialysis or kidney surgery, no autoimmune disease, no malignancy — and liver function entirely normal (ALT 10–36, AST 20–33). "Examination of participant in clinical trial" coded, raising the concurrent-trial exclusion. Recent cardiotomy would also confound the inflammatory/complement biomarker panel. Time-limited: at 54 with two decades of age eligibility remaining, he would fit well once recovered.</x:v>
+        <x:v>First patient assessed against this trial to clear the 18–75 age window (54). Has the cardiorenal substrate, heart_failure and chronic_kidney_disease tags supporting the cardiorenal_syndrome required signal, and all three HF subtypes are accepted, so the missing EF is not a barrier. Fails the "stable chronic" requirement: his heart failure is acute valvular, from rupture of chordae tendineae producing severe mitral regurgitation, repaired days ago by open valvuloplasty with annuloplasty on cardiopulmonary bypass, with Hgb 9.4–14, platelets 112–290, INR to 2.2, potassium 3.1. Likely AKI within 3 months (creatinine 1–1.9 near-doubling post-bypass, hyaline casts 2–32/lpf). Clears every high-priority exclusion, no dialysis or kidney surgery, no autoimmune disease, no malignancy, and liver function entirely normal (ALT 10–36, AST 20–33). "Examination of participant in clinical trial" coded, raising the concurrent-trial exclusion. Recent cardiotomy would also confound the inflammatory/complement biomarker panel. Time-limited: at 54 with two decades of age eligibility remaining, he would fit well once recovered.</x:v>
       </x:c>
     </x:row>
     <x:row r="934" ht="58" customHeight="1">
@@ -26331,7 +26331,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I934" s="9" t="str">
-        <x:v>Clears age 18–75 (54) and the renal criterion (eGFR &lt;90 given creatinine 1–1.9 at 54M), and unlike PAIR-000899 has no osteoarticular disease, no mental illness, no severe anaemia (Hgb 9.4–14 is moderate, not severe), and no syncope. Fails the disease-state requirements: not "chronically stable" — acute valvular heart failure from ruptured chordae tendineae with severe mitral regurgitation, repaired days ago by open valvuloplasty with annuloplasty on cardiopulmonary bypass; and not "low risk in exercise risk assessment" given post-sternotomy state with Hgb to 9.4, platelets to 112, INR to 2.2, potassium 3.1, and hypoxemia. HFrEF unconfirmed — no EF documented, and acute mitral regurgitation typically preserves EF by unloading the ventricle, so true function is only apparent post-repair. AF with surgical ablation raises the severe arrhythmia exclusion; rhythm status unrecorded. Stenotic valve exclusion does not apply as written — his lesion is regurgitant. Time-limited: cardiac rehab is standard post-valve surgery and he would plausibly qualify once recovered, if EF proves reduced</x:v>
+        <x:v>Clears age 18–75 (54) and the renal criterion (eGFR &lt;90 given creatinine 1–1.9 at 54M), and unlike PAIR-000899 has no osteoarticular disease, no mental illness, no severe anaemia (Hgb 9.4–14 is moderate, not severe), and no syncope. Fails the disease-state requirements: not "chronically stable", acute valvular heart failure from ruptured chordae tendineae with severe mitral regurgitation, repaired days ago by open valvuloplasty with annuloplasty on cardiopulmonary bypass; and not "low risk in exercise risk assessment" given post-sternotomy state with Hgb to 9.4, platelets to 112, INR to 2.2, potassium 3.1, and hypoxemia. HFrEF unconfirmed, no EF documented, and acute mitral regurgitation typically preserves EF by unloading the ventricle, so true function is only apparent post-repair. AF with surgical ablation raises the severe arrhythmia exclusion; rhythm status unrecorded. Stenotic valve exclusion does not apply as written, his lesion is regurgitant. Time-limited: cardiac rehab is standard post-valve surgery and he would plausibly qualify once recovered, if EF proves reduced</x:v>
       </x:c>
     </x:row>
     <x:row r="935" ht="58" customHeight="1">
@@ -26358,7 +26358,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I935" s="9" t="str">
-        <x:v>Most permissive protocol in the review — AI chatbot plus remote vital-sign monitoring for cardiovascular-kidney-metabolic disease, with one exclusion (unwillingness to consent). All inclusion criteria affirmatively met: age 54 (&gt;18); qualifies via the high-priority CKD stage 2–4 route with chronic_kidney_disease tag and creatinine 1–1.9 giving eGFR ~40–90, spanning stage 3b to stage 2; and the heart-failure hospitalization condition is satisfied rather than violated, since he is currently an inpatient after open mitral valvuloplasty with annuloplasty for ruptured chordae. No coronary stent or CABG (his surgery was valve repair), and HbA1c 5.7–5.9 is prediabetic without a diabetes diagnosis, but only one CKM route is required. Cognitively intact, no consent barrier, and an explicit clinical-trial participation code indicates prior research engagement. Medium rather than High pending confirmation that enrollment falls within one week of this admission, and device/chatbot access.</x:v>
+        <x:v>Most permissive protocol in the review, AI chatbot plus remote vital-sign monitoring for cardiovascular-kidney-metabolic disease, with one exclusion (unwillingness to consent). All inclusion criteria affirmatively met: age 54 (&gt;18); qualifies via the high-priority CKD stage 2–4 route with chronic_kidney_disease tag and creatinine 1–1.9 giving eGFR ~40–90, spanning stage 3b to stage 2; and the heart-failure hospitalization condition is satisfied rather than violated, since he is currently an inpatient after open mitral valvuloplasty with annuloplasty for ruptured chordae. No coronary stent or CABG (his surgery was valve repair), and HbA1c 5.7–5.9 is prediabetic without a diabetes diagnosis, but only one CKM route is required. Cognitively intact, no consent barrier, and an explicit clinical-trial participation code indicates prior research engagement. Medium rather than High pending confirmation that enrollment falls within one week of this admission, and device/chatbot access.</x:v>
       </x:c>
     </x:row>
     <x:row r="936" ht="58" customHeight="1">
@@ -26387,7 +26387,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I936" s="9" t="str">
-        <x:v>Intracortical brain-machine interface for upper limb paralysis from cervical SCI, brainstem stroke, brachial plexus injury, above-elbow amputation, or spinal stroke — none of which he has. His injury is diffuse traumatic brain injury with traumatic and nontraumatic subdural haemorrhage after falls, plus aphasia and toxic encephalopathy: cortical rather than the cortex-sparing pathology this interface requires. Age 84 exceeds the 22–70 window by 14 years. Cardiac pacemaker (coded twice, plus generator battery check) triggers the implantable-generator exclusion and precludes the required screening fMRI. Myocardial infarction history triggers a high-priority exclusion, alongside sudden_cardiac_death and atrial fibrillation tags and postprocedural cardiogenic shock. Injury is acute (initial encounter, s/p subdural evacuation by open craniotomy) rather than &gt;1 year old and stable; the craniotomy also likely engages the prior frontal/parietal neurosurgery exclusion. Aphasia bars English communication, following directions, and normal neuropsychological assessment. Active infection (UTI, Klebsiella, Proteus, WBC to 25.6, vancomycin level). Uncontrolled insulin-dependent diabetes (HbA1c 7.6–9.1, glucose 70–342). Injurious falls documented. Phenytoin level in his panel indicates antiepileptic therapy, engaging the seizure exclusion.</x:v>
+        <x:v>Intracortical brain-machine interface for upper limb paralysis from cervical SCI, brainstem stroke, brachial plexus injury, above-elbow amputation, or spinal stroke, none of which he has. His injury is diffuse traumatic brain injury with traumatic and nontraumatic subdural haemorrhage after falls, plus aphasia and toxic encephalopathy: cortical rather than the cortex-sparing pathology this interface requires. Age 84 exceeds the 22–70 window by 14 years. Cardiac pacemaker (coded twice, plus generator battery check) triggers the implantable-generator exclusion and precludes the required screening fMRI. Myocardial infarction history triggers a high-priority exclusion, alongside sudden_cardiac_death and atrial fibrillation tags and postprocedural cardiogenic shock. Injury is acute (initial encounter, s/p subdural evacuation by open craniotomy) rather than &gt;1 year old and stable; the craniotomy also likely engages the prior frontal/parietal neurosurgery exclusion. Aphasia bars English communication, following directions, and normal neuropsychological assessment. Active infection (UTI, Klebsiella, Proteus, WBC to 25.6, vancomycin level). Uncontrolled insulin-dependent diabetes (HbA1c 7.6–9.1, glucose 70–342). Injurious falls documented. Phenytoin level in his panel indicates antiepileptic therapy, engaging the seizure exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="937" ht="58" customHeight="1">
@@ -26416,7 +26416,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I937" s="9" t="str">
-        <x:v>Target syndrome present and both required signals supported on the cardiorenal side — heart_failure tag with fluid overload, mitral insufficiency, prior CABG and mitral valve repair, postprocedural cardiogenic shock; chronic_kidney_disease tag with creatinine 0.9–2.2 giving eGFR ~28 at worst, above the ≥15 floor. Loop diuretic use probable (fluid overload, hypokalaemia coded, K 2.9–6.6, digoxin level in panel). Excluded by two categorical barriers: cardiac pacemaker (coded twice plus generator battery check) as a direct MR scanning contraindication — materially different from the annuloplasty ring at PAIR-000984, which was a passive device remote from the kidneys; and inability to consent given aphasia and toxic encephalopathy after diffuse TBI and subdural haemorrhage with open craniotomy, with no surrogate consent route in this protocol. Visit 2 hypokalaemia threshold also breached (K to 2.9 vs &lt;3.5). Clears hepatorenal syndrome, kidney malformation, and pregnancy exclusions.</x:v>
+        <x:v>Target syndrome present and both required signals supported on the cardiorenal side, heart_failure tag with fluid overload, mitral insufficiency, prior CABG and mitral valve repair, postprocedural cardiogenic shock; chronic_kidney_disease tag with creatinine 0.9–2.2 giving eGFR ~28 at worst, above the ≥15 floor. Loop diuretic use probable (fluid overload, hypokalaemia coded, K 2.9–6.6, digoxin level in panel). Excluded by two categorical barriers: cardiac pacemaker (coded twice plus generator battery check) as a direct MR scanning contraindication, materially different from the annuloplasty ring at PAIR-000984, which was a passive device remote from the kidneys; and inability to consent given aphasia and toxic encephalopathy after diffuse TBI and subdural haemorrhage with open craniotomy, with no surrogate consent route in this protocol. Visit 2 hypokalaemia threshold also breached (K to 2.9 vs &lt;3.5). Clears hepatorenal syndrome, kidney malformation, and pregnancy exclusions.</x:v>
       </x:c>
     </x:row>
     <x:row r="938" ht="58" customHeight="1">
@@ -26445,7 +26445,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I938" s="9" t="str">
-        <x:v>Best population fit of the three patients assessed against this trial — "Fluid overload, unspecified" affirmatively coded (vs dehydration at PAIR-000894 and no volume status at PAIR-000985), with heart_failure tag, postprocedural cardiogenic shock, and CKD stage 4 at worst (creatinine 0.9–2.2, eGFR ~28 at 84M). Excluded by recurrent/severe urinary tract infection: UTI with both Proteus and Klebsiella, abnormal urinary findings, WBC to 25.6, neutrophils to 81.6%, vancomycin level — mechanistically critical since SGLT2 inhibitors induce glycosuria and he has HbA1c 7.6–9.1 with glucose to 342. General safety exclusion engaged by traumatic and nontraumatic subdural haemorrhage with open craniotomy, diffuse TBI, toxic encephalopathy, aphasia, Hgb 7.1, platelets 79, INR 2.8, PTT 89.4, 4-factor PCC transfusion, sodium 126–151. Enteral tube feeding with oral-phase dysphagia raises the absorption exclusion. Consent not obtainable (aphasia, encephalopathy). Clears liver disease, type 1 diabetes, DKA, and dialysis exclusions; protocol explicitly permits acute creatinine rise. NOTE: inclusion_criteria array entirely EMPTY in source.</x:v>
+        <x:v>Best population fit of the three patients assessed against this trial, "Fluid overload, unspecified" affirmatively coded (vs dehydration at PAIR-000894 and no volume status at PAIR-000985), with heart_failure tag, postprocedural cardiogenic shock, and CKD stage 4 at worst (creatinine 0.9–2.2, eGFR ~28 at 84M). Excluded by recurrent/severe urinary tract infection: UTI with both Proteus and Klebsiella, abnormal urinary findings, WBC to 25.6, neutrophils to 81.6%, vancomycin level, mechanistically critical since SGLT2 inhibitors induce glycosuria and he has HbA1c 7.6–9.1 with glucose to 342. General safety exclusion engaged by traumatic and nontraumatic subdural haemorrhage with open craniotomy, diffuse TBI, toxic encephalopathy, aphasia, Hgb 7.1, platelets 79, INR 2.8, PTT 89.4, 4-factor PCC transfusion, sodium 126–151. Enteral tube feeding with oral-phase dysphagia raises the absorption exclusion. Consent not obtainable (aphasia, encephalopathy). Clears liver disease, type 1 diabetes, DKA, and dialysis exclusions; protocol explicitly permits acute creatinine rise. NOTE: inclusion_criteria array entirely EMPTY in source.</x:v>
       </x:c>
     </x:row>
     <x:row r="939" ht="58" customHeight="1">
@@ -26474,7 +26474,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I939" s="9" t="str">
-        <x:v>Trial targets sepsis-induced myocardial dysfunction dx within 24h. No sepsis/SIMD documented; cardiac dysfunction is chronic ischemic/structural — ischemic CM, chronic systolic HF, old MI, prior CABG, mitral repair for nonrheumatic MR, chronic AF/PAF, VT, pacemaker. Explicit exclusions present: HF from structural disease + arrhythmia, cardiomyopathy-related HF, ACS (NSTEMI w/ postprocedural cardiogenic shock), cardiorenal syndrome. Age 84 meets 50–85. Soft items (SOFA, surrogate consent, NG dosing, med rec) moot. Enrollment would confound the BNP/NT-proBNP endpoint.</x:v>
+        <x:v>Trial targets sepsis-induced myocardial dysfunction dx within 24h. No sepsis/SIMD documented; cardiac dysfunction is chronic ischemic/structural, ischemic CM, chronic systolic HF, old MI, prior CABG, mitral repair for nonrheumatic MR, chronic AF/PAF, VT, pacemaker. Explicit exclusions present: HF from structural disease + arrhythmia, cardiomyopathy-related HF, ACS (NSTEMI w/ postprocedural cardiogenic shock), cardiorenal syndrome. Age 84 meets 50–85. Soft items (SOFA, surrogate consent, NG dosing, med rec) moot. Enrollment would confound the BNP/NT-proBNP endpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="940" ht="58" customHeight="1">
@@ -26501,7 +26501,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I940" s="9" t="str">
-        <x:v>Permissive ADHF decongestion study — only criteria are age ≥18, clinical ADHF, proBNP &gt;800, consent, plus one investigator-discretion exclusion. 84M with chronic systolic HF from ischemic CM, documented fluid overload, hyponatremia, hypoxemia, and CKD w/ diabetic nephropathy = the cardiorenal phenotype targeted. No hard exclusion tripped; pacemaker, chronic AF, VT, prior CABG, anticoagulation all unrestricted. Open questions are screening-level: proBNP not measured (very likely &gt;800), congestion may be post-cardiotomy rather than de novo ADHF, and consent capacity uncertain given aphasia/toxic encephalopathy/TBI — no surrogate provision stated. Single-center Oslo. Worth screening.</x:v>
+        <x:v>Permissive ADHF decongestion study, only criteria are age ≥18, clinical ADHF, proBNP &gt;800, consent, plus one investigator-discretion exclusion. 84M with chronic systolic HF from ischemic CM, documented fluid overload, hyponatremia, hypoxemia, and CKD w/ diabetic nephropathy = the cardiorenal phenotype targeted. No hard exclusion tripped; pacemaker, chronic AF, VT, prior CABG, anticoagulation all unrestricted. Open questions are screening-level: proBNP not measured (very likely &gt;800), congestion may be post-cardiotomy rather than de novo ADHF, and consent capacity uncertain given aphasia/toxic encephalopathy/TBI, no surrogate provision stated. Single-center Oslo. Worth screening.</x:v>
       </x:c>
     </x:row>
     <x:row r="941" ht="58" customHeight="1">
@@ -26530,7 +26530,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I941" s="9" t="str">
-        <x:v>R/R multiple myeloma CAR-T trial; patient has no plasma cell disorder — no myeloma, plasmacytoma, M protein, FLC studies, or lytic lesions. Only neoplasms are benign colonic polyps. Anemia and CKD fully explained by posthemorrhagic anemia and diabetic/hypertensive nephropathy, not CRAB. Also age 84 vs hard cap 75; no prior anti-MM therapy so R/R criterion unmeetable; no measurable disease; CrCl &lt;60. Independently excluded by uncontrolled CV disease (VT, chronic/PAF AF, NSTEMI, cardiogenic shock, symptomatic HF, prior TIA, likely LVEF &lt;45%), major surgery within 3 mo (CABG + mitral repair, craniotomy), and active CNS abnormality (SDH s/p evacuation, TBI, toxic encephalopathy). Likely a tag-noise retrieval artifact.</x:v>
+        <x:v>R/R multiple myeloma CAR-T trial; patient has no plasma cell disorder, no myeloma, plasmacytoma, M protein, FLC studies, or lytic lesions. Only neoplasms are benign colonic polyps. Anemia and CKD fully explained by posthemorrhagic anemia and diabetic/hypertensive nephropathy, not CRAB. Also age 84 vs hard cap 75; no prior anti-MM therapy so R/R criterion unmeetable; no measurable disease; CrCl &lt;60. Independently excluded by uncontrolled CV disease (VT, chronic/PAF AF, NSTEMI, cardiogenic shock, symptomatic HF, prior TIA, likely LVEF &lt;45%), major surgery within 3 mo (CABG + mitral repair, craniotomy), and active CNS abnormality (SDH s/p evacuation, TBI, toxic encephalopathy). Likely a tag-noise retrieval artifact.</x:v>
       </x:c>
     </x:row>
     <x:row r="942" ht="58" customHeight="1">
@@ -26559,7 +26559,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I942" s="9" t="str">
-        <x:v>Disease match is good — CRS biomarker cohort and patient has chronic systolic HF w/ CKD and diabetic nephropathy. Fails on population: hard age window 18–75, patient is 84 (9 yrs over, high-priority criterion). Also requires STABLE chronic HF followed 12 mo; patient is critically ill with postprocedural cardiogenic shock, fluid overload, VT, recent CABG + mitral repair and craniotomy. Active infection exclusion tripped (UTI w/ Proteus + Klebsiella, WBC 19.6). Recent post-cardiotomy AKI likely present (Cr 1.4, BUN 26) though not explicitly coded. LVEF undocumented but likely HFrEF — moot given age. Near-miss on phenotype, hard fail on eligibility.</x:v>
+        <x:v>Disease match is good, CRS biomarker cohort and patient has chronic systolic HF w/ CKD and diabetic nephropathy. Fails on population: hard age window 18–75, patient is 84 (9 yrs over, high-priority criterion). Also requires STABLE chronic HF followed 12 mo; patient is critically ill with postprocedural cardiogenic shock, fluid overload, VT, recent CABG + mitral repair and craniotomy. Active infection exclusion tripped (UTI w/ Proteus + Klebsiella, WBC 19.6). Recent post-cardiotomy AKI likely present (Cr 1.4, BUN 26) though not explicitly coded. LVEF undocumented but likely HFrEF, moot given age. Near-miss on phenotype, hard fail on eligibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="943" ht="58" customHeight="1">
@@ -26588,7 +26588,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I943" s="9" t="str">
-        <x:v>Home-based exercise rehab in CRS + HFrEF. Phenotype fits (chronic systolic HF from ischemic CM, CKD w/ diabetic nephropathy, eGFR almost certainly &lt;90), but hard age window 18–75 and patient is 84. Also fails "chronically stable" (postprocedural cardiogenic shock, fluid overload, invasive ventilation, PA catheter) and "low risk on exercise risk assessment." Severe-arrhythmia exclusion clearly present: ventricular tachycardia plus chronic/paroxysmal AF, pacemaker, s/p EP study and ablation. Likely syncope history — two falls incl. down stairs causing TBI/SDH in a patient w/ VT. Bilateral hip arthroplasties, bronchiectasis, hypoxemia, and toxic encephalopathy/aphasia further impede unsupervised home training. Safety exclusion, not just administrative.</x:v>
+        <x:v>Home-based exercise rehab in CRS + HFrEF. Phenotype fits (chronic systolic HF from ischemic CM, CKD w/ diabetic nephropathy, eGFR almost certainly &lt;90), but hard age window 18–75 and patient is 84. Also fails "chronically stable" (postprocedural cardiogenic shock, fluid overload, invasive ventilation, PA catheter) and "low risk on exercise risk assessment." Severe-arrhythmia exclusion clearly present: ventricular tachycardia plus chronic/paroxysmal AF, pacemaker, s/p EP study and ablation. Likely syncope history, two falls incl. down stairs causing TBI/SDH in a patient w/ VT. Bilateral hip arthroplasties, bronchiectasis, hypoxemia, and toxic encephalopathy/aphasia further impede unsupervised home training. Safety exclusion, not just administrative.</x:v>
       </x:c>
     </x:row>
     <x:row r="944" ht="58" customHeight="1">
@@ -26615,7 +26615,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I944" s="9" t="str">
-        <x:v>Pragmatic CKM care-coordination trial — needs only age &gt;18 plus ONE CKM component; sole exclusion is refusal of consent. Patient satisfies three components: insulin-treated T2DM w/ hyperglycemia and diabetic nephropathy; 3-vessel CABG this encounter (well within 12 mo); CKD stage 3 range (Cr 1.4, diabetic + hypertensive CKD coded). HF sub-requirement of hospitalization within 1 week is met — currently admitted. No upper age limit, no EF/eGFR cutoffs, no arrhythmia, device, or comorbidity exclusions, so VT, AF, pacemaker, prior MI, SDH, and anticoagulation are all non-issues. Work-up items only: A1c not documented (CABG + CKD qualify independently), eGFR staging, consent capacity given aphasia/toxic encephalopathy, and caregiver support for the chatbot/remote-monitoring arm.</x:v>
+        <x:v>Pragmatic CKM care-coordination trial, needs only age &gt;18 plus ONE CKM component; sole exclusion is refusal of consent. Patient satisfies three components: insulin-treated T2DM w/ hyperglycemia and diabetic nephropathy; 3-vessel CABG this encounter (well within 12 mo); CKD stage 3 range (Cr 1.4, diabetic + hypertensive CKD coded). HF sub-requirement of hospitalization within 1 week is met, currently admitted. No upper age limit, no EF/eGFR cutoffs, no arrhythmia, device, or comorbidity exclusions, so VT, AF, pacemaker, prior MI, SDH, and anticoagulation are all non-issues. Work-up items only: A1c not documented (CABG + CKD qualify independently), eGFR staging, consent capacity given aphasia/toxic encephalopathy, and caregiver support for the chatbot/remote-monitoring arm.</x:v>
       </x:c>
     </x:row>
     <x:row r="945" ht="58" customHeight="1">
@@ -26644,7 +26644,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I945" s="9" t="str">
-        <x:v>HF early-screening trial in at-risk but UNDIAGNOSED patients. Explicit high-priority exclusion: any previous HF diagnosis, any EF, any cause. Patient has congestive heart failure coded — hard stop. Over-qualifies on inclusion side (age 88 &gt;40; four+ risk factors: CAD w/ PCI and CABG, AF, extensive PAD w/ peripheral stenting, bypass grafts and BKA, and CKD), which makes this a useful test case — every inclusion criterion hit, single exclusion disqualifies. Supporting cardiac disease: secondary pulmonary HTN, mitral valve disorder, pericardial disease. AKI w/ ATN documented but no RRT (Cr recovered to 0.9–1.3). Canadian primary-care catchment is logistical and moot.</x:v>
+        <x:v>HF early-screening trial in at-risk but UNDIAGNOSED patients. Explicit high-priority exclusion: any previous HF diagnosis, any EF, any cause. Patient has congestive heart failure coded, hard stop. Over-qualifies on inclusion side (age 88 &gt;40; four+ risk factors: CAD w/ PCI and CABG, AF, extensive PAD w/ peripheral stenting, bypass grafts and BKA, and CKD), which makes this a useful test case, every inclusion criterion hit, single exclusion disqualifies. Supporting cardiac disease: secondary pulmonary HTN, mitral valve disorder, pericardial disease. AKI w/ ATN documented but no RRT (Cr recovered to 0.9–1.3). Canadian primary-care catchment is logistical and moot.</x:v>
       </x:c>
     </x:row>
     <x:row r="946" ht="58" customHeight="1">
@@ -26673,7 +26673,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I946" s="9" t="str">
-        <x:v>Post-acute-PE cohort screening for CTEPH. Patient has no PE, no DVT, no VTE anywhere in record — vascular disease is entirely arterial (coronary and peripheral atherosclerosis, bypass graft disease, rest pain, BKA); the thrombolytic infusion was arterial for limb ischemia, not pulmonary. Index event absent, so PESI/sPESI criterion is inapplicable, not just undocumented. Secondary pulmonary HTN is coded and is an explicit exclusion — hers is Group 2 (left-heart) from mitral valve disorder + CHF, the opposite of the Group 4 thromboembolic PH under study. Age 88 vs 18–80 window. AKI w/ ATN resolved (Cr 0.9–1.3), anticoagulation tolerated long-term. Likely a PH-keyword retrieval artifact; good distractor case.</x:v>
+        <x:v>Post-acute-PE cohort screening for CTEPH. Patient has no PE, no DVT, no VTE anywhere in record, vascular disease is entirely arterial (coronary and peripheral atherosclerosis, bypass graft disease, rest pain, BKA); the thrombolytic infusion was arterial for limb ischemia, not pulmonary. Index event absent, so PESI/sPESI criterion is inapplicable, not just undocumented. Secondary pulmonary HTN is coded and is an explicit exclusion, hers is Group 2 (left-heart) from mitral valve disorder + CHF, the opposite of the Group 4 thromboembolic PH under study. Age 88 vs 18–80 window. AKI w/ ATN resolved (Cr 0.9–1.3), anticoagulation tolerated long-term. Likely a PH-keyword retrieval artifact; good distractor case.</x:v>
       </x:c>
     </x:row>
     <x:row r="947" ht="58" customHeight="1">
@@ -26702,7 +26702,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I947" s="9" t="str">
-        <x:v>Right disease, wrong clinical moment. CRAFT-WHF enrolls within 48h of an admission for worsening HF requiring urgent IV diuretics for volume overload. Patient has chronic CHF but this admission is for critical limb ischemia — peripheral angioplasty/stenting, arterial thrombolysis, bypass, femoral arteriography, BKA — complicated by AKI/ATN and Klebsiella. No volume overload, no IV diuretic, no BNP documented. Index event is an occurrence, not a workup item, and her non-HF acute trigger independently trips that exclusion. Body weight &lt;70 kg exclusion very likely met (88F post-BKA) though undocumented. Soft items: BNP, loop diuretic confirmation, weight, echo to characterize mitral lesion, CABG/PCI dates. Confidence Medium — if she decompensated later in this admission and got IV diuretics she should be re-reviewed.</x:v>
+        <x:v>Right disease, wrong clinical moment. CRAFT-WHF enrolls within 48h of an admission for worsening HF requiring urgent IV diuretics for volume overload. Patient has chronic CHF but this admission is for critical limb ischemia, peripheral angioplasty/stenting, arterial thrombolysis, bypass, femoral arteriography, BKA, complicated by AKI/ATN and Klebsiella. No volume overload, no IV diuretic, no BNP documented. Index event is an occurrence, not a workup item, and her non-HF acute trigger independently trips that exclusion. Body weight &lt;70 kg exclusion very likely met (88F post-BKA) though undocumented. Soft items: BNP, loop diuretic confirmation, weight, echo to characterize mitral lesion, CABG/PCI dates. Confidence Medium, if she decompensated later in this admission and got IV diuretics she should be re-reviewed.</x:v>
       </x:c>
     </x:row>
     <x:row r="948" ht="58" customHeight="1">
@@ -26731,7 +26731,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I948" s="9" t="str">
-        <x:v>Esketamine POD-prevention trial in ELECTIVE major NON-CARDIAC surgery, with vascular surgery explicitly excluded. Patient meets age window (88, within 65–&lt;90) and hits 8+ delirium risk factors (HTN, CHF, CAD, AF, PAD, CKD, chronic pain, anemia) — inclusion side is emphatic. Fails on surgical category: her operative course is entirely vascular (peripheral bypass/shunt, non-coronary angioplasty, peripheral stenting, femoral arteriography, aortography, arterial thrombolysis, BKA). Also not elective — limb salvage for rest pain is urgent — and acute limb ischemia requiring thrombolysis likely trips the 30-day acute CV event exclusion. Right patient, wrong operation; would qualify if scheduled for elective abdominal/ortho surgery. Alt mechanism label: Prior procedure conflict.</x:v>
+        <x:v>Esketamine POD-prevention trial in ELECTIVE major NON-CARDIAC surgery, with vascular surgery explicitly excluded. Patient meets age window (88, within 65–&lt;90) and hits 8+ delirium risk factors (HTN, CHF, CAD, AF, PAD, CKD, chronic pain, anemia), inclusion side is emphatic. Fails on surgical category: her operative course is entirely vascular (peripheral bypass/shunt, non-coronary angioplasty, peripheral stenting, femoral arteriography, aortography, arterial thrombolysis, BKA). Also not elective, limb salvage for rest pain is urgent, and acute limb ischemia requiring thrombolysis likely trips the 30-day acute CV event exclusion. Right patient, wrong operation; would qualify if scheduled for elective abdominal/ortho surgery. Alt mechanism label: Prior procedure conflict.</x:v>
       </x:c>
     </x:row>
     <x:row r="949" ht="58" customHeight="1">
@@ -26760,7 +26760,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I949" s="9" t="str">
-        <x:v>Large-bore femoral closure device trial for elective TAVR/TEVAR/PEVAR-type procedures. Five independent disqualifiers: (1) below-knee amputation — excluded by name; (2) Rutherford 5–6 PAD (rest pain progressing to tissue loss/amputation) — excluded by name; (3) prior vascular surgery, bypass graft, and peripheral stent in the access region, with graft atherosclerosis documented; (4) thrombolytic administration; (5) no qualifying elective large-bore catheterization anywhere in record — her interventions were urgent limb salvage, not structural. Also likely unable to ambulate at baseline and has active Klebsiella/UTI. Labs actually clear the anemia, platelet, and renal thresholds (Hgb 11.6–13.9, plt 209–295, Cr 0.9–1.3). Retrieval likely keyed on femoral arteriography; trial wants clean femoral anatomy, she is the opposite.</x:v>
+        <x:v>Large-bore femoral closure device trial for elective TAVR/TEVAR/PEVAR-type procedures. Five independent disqualifiers: (1) below-knee amputation, excluded by name; (2) Rutherford 5–6 PAD (rest pain progressing to tissue loss/amputation), excluded by name; (3) prior vascular surgery, bypass graft, and peripheral stent in the access region, with graft atherosclerosis documented; (4) thrombolytic administration; (5) no qualifying elective large-bore catheterization anywhere in record, her interventions were urgent limb salvage, not structural. Also likely unable to ambulate at baseline and has active Klebsiella/UTI. Labs actually clear the anemia, platelet, and renal thresholds (Hgb 11.6–13.9, plt 209–295, Cr 0.9–1.3). Retrieval likely keyed on femoral arteriography; trial wants clean femoral anatomy, she is the opposite.</x:v>
       </x:c>
     </x:row>
     <x:row r="950" ht="58" customHeight="1">
@@ -26789,7 +26789,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I950" s="9" t="str">
-        <x:v>Same CRS biomarker cohort as PAIR-001001, different patient, same age wall — 88 vs hard 18–75 window (13 yrs over). Unlike that pair, exclusions here are documented not inferred: acute kidney failure with tubular necrosis coded this encounter trips the AKI-within-3-months exclusion (recovery to Cr 0.9–1.3 doesn't clear a history-based criterion), and UTI with Klebsiella trips acute infection. Fails "stable CHF" — encounter includes arterial thrombolysis, peripheral bypass/stenting, BKA, acute postop pain, secondary pulmonary HTN, mitral valve disorder. Nephrotoxic exposure likely (aortography, femoral arteriography, multiple contrast studies, antibiotics). LVEF undocumented but echo was performed. Second consecutive patient failing this protocol on age — retrieval appears to weight cardiorenal phenotype without the age constraint.</x:v>
+        <x:v>Same CRS biomarker cohort as PAIR-001001, different patient, same age wall, 88 vs hard 18–75 window (13 yrs over). Unlike that pair, exclusions here are documented not inferred: acute kidney failure with tubular necrosis coded this encounter trips the AKI-within-3-months exclusion (recovery to Cr 0.9–1.3 doesn't clear a history-based criterion), and UTI with Klebsiella trips acute infection. Fails "stable CHF", encounter includes arterial thrombolysis, peripheral bypass/stenting, BKA, acute postop pain, secondary pulmonary HTN, mitral valve disorder. Nephrotoxic exposure likely (aortography, femoral arteriography, multiple contrast studies, antibiotics). LVEF undocumented but echo was performed. Second consecutive patient failing this protocol on age, retrieval appears to weight cardiorenal phenotype without the age constraint.</x:v>
       </x:c>
     </x:row>
     <x:row r="951" ht="58" customHeight="1">
@@ -26818,7 +26818,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I951" s="9" t="str">
-        <x:v>68Ga-FAPI PET/CT fibrosis pilot enrolling only non-ischemic dilated cardiomyopathy (LVEF ≤40%) or sarcomeric-mutation hypertrophic cardiomyopathy (LVEF ≥50%). Patient has neither — no DCM, no HCM, no genetic testing, CHF coded unspecified. Her HF is ischemic/valvular/hypertensive: coronary atherosclerosis of native coronary artery with PCI and CABG history, which directly trips the "significant atherosclerotic CAD" exclusion and makes the required normal coronary angiogram within 6 months unobtainable. Mitral valve disorders likely trip the significant primary valvular disease exclusion, supported by secondary pulmonary HTN. Echo performed (LVEF not in record); no CMR. Retrieval keyed on "heart failure"/"fibrosis" without the non-ischemic constraint that defines the cohort.</x:v>
+        <x:v>68Ga-FAPI PET/CT fibrosis pilot enrolling only non-ischemic dilated cardiomyopathy (LVEF ≤40%) or sarcomeric-mutation hypertrophic cardiomyopathy (LVEF ≥50%). Patient has neither, no DCM, no HCM, no genetic testing, CHF coded unspecified. Her HF is ischemic/valvular/hypertensive: coronary atherosclerosis of native coronary artery with PCI and CABG history, which directly trips the "significant atherosclerotic CAD" exclusion and makes the required normal coronary angiogram within 6 months unobtainable. Mitral valve disorders likely trip the significant primary valvular disease exclusion, supported by secondary pulmonary HTN. Echo performed (LVEF not in record); no CMR. Retrieval keyed on "heart failure"/"fibrosis" without the non-ischemic constraint that defines the cohort.</x:v>
       </x:c>
     </x:row>
     <x:row r="952" ht="58" customHeight="1">
@@ -26847,7 +26847,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I952" s="9" t="str">
-        <x:v>IV iron trial in PH with 6MWT-based exercise capacity as the primary endpoint. Patient has secondary (likely Group 2) PH, which is an eligible category, but cannot meaningfully perform a 6MWT — recent below-knee amputation plus contralateral native-artery atherosclerosis with rest pain and limb pain. That trips the investigator-judgment exclusion and makes her unassessable on the primary outcome; barrier is anatomic, not temporary. Active Klebsiella/UTI also excluded (treatable). Group 2 arm requires LVEF &gt;50%; echo was performed but LVEF undocumented — if HFrEF she is categorically out. Iron studies (TSAT, ferritin) never drawn; Hgb 11.6–13.9 normocytic, within the 8–15 window. Mitral valve disorder severity unknown — severe MR would exclude. Revisit only if she rehabs to prosthetic ambulation AND is HFpEF AND TSAT &lt;21%.</x:v>
+        <x:v>IV iron trial in PH with 6MWT-based exercise capacity as the primary endpoint. Patient has secondary (likely Group 2) PH, which is an eligible category, but cannot meaningfully perform a 6MWT, recent below-knee amputation plus contralateral native-artery atherosclerosis with rest pain and limb pain. That trips the investigator-judgment exclusion and makes her unassessable on the primary outcome; barrier is anatomic, not temporary. Active Klebsiella/UTI also excluded (treatable). Group 2 arm requires LVEF &gt;50%; echo was performed but LVEF undocumented, if HFrEF she is categorically out. Iron studies (TSAT, ferritin) never drawn; Hgb 11.6–13.9 normocytic, within the 8–15 window. Mitral valve disorder severity unknown, severe MR would exclude. Revisit only if she rehabs to prosthetic ambulation AND is HFpEF AND TSAT &lt;21%.</x:v>
       </x:c>
     </x:row>
     <x:row r="953" ht="58" customHeight="1">
@@ -26874,7 +26874,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I953" s="9" t="str">
-        <x:v>Same permissive CKM trial as PAIR-001003 — age &gt;18 plus ONE CKM component, sole exclusion is refusal of consent. Qualifies on CKD stage 3 (Cr 0.9–1.3 in an 88F ≈ eGFR high-30s to low-50s) and on heart disease with stenting (coronary atherosclerosis of native coronary artery, PCI and CABG in tags; stents documented this encounter are peripheral). HF sub-requirement of hospitalization within 1 week is met — currently inpatient with CHF. Not diabetic (glucose 101–120), but diabetes is only one of several qualifying routes. No upper age limit, no eGFR/EF/arrhythmia/comorbidity exclusions, so BKA, PAD, AF, secondary pulm HTN, mitral valve disorder, resolved ATN, and Klebsiella are all non-issues. Capacity appears intact — no cognitive dx coded. Work-up: eGFR staging, coronary vs peripheral stent documentation, CABG date, and caregiver support for the remote-monitoring/chatbot arm.</x:v>
+        <x:v>Same permissive CKM trial as PAIR-001003, age &gt;18 plus ONE CKM component, sole exclusion is refusal of consent. Qualifies on CKD stage 3 (Cr 0.9–1.3 in an 88F ≈ eGFR high-30s to low-50s) and on heart disease with stenting (coronary atherosclerosis of native coronary artery, PCI and CABG in tags; stents documented this encounter are peripheral). HF sub-requirement of hospitalization within 1 week is met, currently inpatient with CHF. Not diabetic (glucose 101–120), but diabetes is only one of several qualifying routes. No upper age limit, no eGFR/EF/arrhythmia/comorbidity exclusions, so BKA, PAD, AF, secondary pulm HTN, mitral valve disorder, resolved ATN, and Klebsiella are all non-issues. Capacity appears intact, no cognitive dx coded. Work-up: eGFR staging, coronary vs peripheral stent documentation, CABG date, and caregiver support for the remote-monitoring/chatbot arm.</x:v>
       </x:c>
     </x:row>
     <x:row r="954" ht="58" customHeight="1">
@@ -26903,7 +26903,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I954" s="9" t="str">
-        <x:v>Exercise + liraglutide physiology study in NON-diabetic metabolic syndrome. Patient has T2DM with hyperglycemia and diabetic polyneuropathy — explicit high-priority exclusion ("any type of diabetes"). Also trips the "significant cardiac/pulmonary/hematologic/endocrine disease" exclusion across five systems: dilated cardiomyopathy, acute systolic HF, cardiogenic shock, Takotsubo, coronary atherosclerosis, acute hypoxic respiratory failure with pneumonia, thrombocytopenia, anemia, hypothyroidism. Recent cardiogenic + septic shock is a contraindication to the 24-week exercise arm. Age 63 vs ≤60 cap. Note HDL 42 is actually above the &lt;40 male threshold so that ATP III component is NOT met; TC 242 stays under the 260 exclusion. Medication noncompliance coded, arguing against 3-month dose stability. Retrieval keyed on metabolic-syndrome/diabetes tags — diabetes is the very thing this trial excludes.</x:v>
+        <x:v>Exercise + liraglutide physiology study in NON-diabetic metabolic syndrome. Patient has T2DM with hyperglycemia and diabetic polyneuropathy, explicit high-priority exclusion ("any type of diabetes"). Also trips the "significant cardiac/pulmonary/hematologic/endocrine disease" exclusion across five systems: dilated cardiomyopathy, acute systolic HF, cardiogenic shock, Takotsubo, coronary atherosclerosis, acute hypoxic respiratory failure with pneumonia, thrombocytopenia, anemia, hypothyroidism. Recent cardiogenic + septic shock is a contraindication to the 24-week exercise arm. Age 63 vs ≤60 cap. Note HDL 42 is actually above the &lt;40 male threshold so that ATP III component is NOT met; TC 242 stays under the 260 exclusion. Medication noncompliance coded, arguing against 3-month dose stability. Retrieval keyed on metabolic-syndrome/diabetes tags, diabetes is the very thing this trial excludes.</x:v>
       </x:c>
     </x:row>
     <x:row r="955" ht="58" customHeight="1">
@@ -26932,7 +26932,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I955" s="9" t="str">
-        <x:v>Pediatric cohort study, ages 7–18, newly diagnosed primary hypertension recruited from pediatric hypertension/nephrology clinics. Patient is a 63-year-old man — 45 years past the ceiling, with the age bound stated at high priority as BOTH an inclusion and an exclusion criterion. Also fails: hypertension is established, not newly diagnosed; multiple confounding conditions excluded by name (T2DM w/ polyneuropathy, dilated cardiomyopathy, acute systolic HF, cardiogenic shock, Takotsubo, coronary atherosclerosis — far beyond the permitted "hypertension-associated echo changes or albuminuria"); critical illness precludes study assessments; caregiver-consent structure is inapplicable to an adult. Pure retrieval artifact on the hypertension tag. Useful sanity-check pair for whether the model respects registered age bounds.</x:v>
+        <x:v>Pediatric cohort study, ages 7–18, newly diagnosed primary hypertension recruited from pediatric hypertension/nephrology clinics. Patient is a 63-year-old man, 45 years past the ceiling, with the age bound stated at high priority as BOTH an inclusion and an exclusion criterion. Also fails: hypertension is established, not newly diagnosed; multiple confounding conditions excluded by name (T2DM w/ polyneuropathy, dilated cardiomyopathy, acute systolic HF, cardiogenic shock, Takotsubo, coronary atherosclerosis, far beyond the permitted "hypertension-associated echo changes or albuminuria"); critical illness precludes study assessments; caregiver-consent structure is inapplicable to an adult. Pure retrieval artifact on the hypertension tag. Useful sanity-check pair for whether the model respects registered age bounds.</x:v>
       </x:c>
     </x:row>
     <x:row r="956" ht="58" customHeight="1">
@@ -26961,7 +26961,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I956" s="9" t="str">
-        <x:v>Mechanistic microvascular physiology study recruiting uncomplicated T2DM. Patient clears entry — T2DM at 63, within 18–80 — but trips multiple flat exclusions: heart failure (acute systolic HF + dilated cardiomyopathy, cardiogenic shock, PA catheter), hyperlipidemia AND hypercholesterolemia (both named separately; TC 242, LDL 124, TC/HDL 5.8), likely anticoagulant use (PTT 48.3–53.9 with INR 1.3), and diabetic polyneuropathy as a documented neuromuscular disorder. CAD is coded WITHOUT angina so the "symptomatic CAD" exclusion may not strictly apply, though Takotsubo and cardiogenic shock are overt cardiac events. Renal function is actually clean (Cr 0.8, ACR 16). Retinopathy undocumented but plausible given polyneuropathy — high-priority exclusion worth an eye exam. Recent shock also makes the 2-day physiology protocol + 14-day trehalose course unworkable. Design wants diabetes as the isolated variable; he brings four confounders.</x:v>
+        <x:v>Mechanistic microvascular physiology study recruiting uncomplicated T2DM. Patient clears entry, T2DM at 63, within 18–80, but trips multiple flat exclusions: heart failure (acute systolic HF + dilated cardiomyopathy, cardiogenic shock, PA catheter), hyperlipidemia AND hypercholesterolemia (both named separately; TC 242, LDL 124, TC/HDL 5.8), likely anticoagulant use (PTT 48.3–53.9 with INR 1.3), and diabetic polyneuropathy as a documented neuromuscular disorder. CAD is coded WITHOUT angina so the "symptomatic CAD" exclusion may not strictly apply, though Takotsubo and cardiogenic shock are overt cardiac events. Renal function is actually clean (Cr 0.8, ACR 16). Retinopathy undocumented but plausible given polyneuropathy, high-priority exclusion worth an eye exam. Recent shock also makes the 2-day physiology protocol + 14-day trehalose course unworkable. Design wants diabetes as the isolated variable; he brings four confounders.</x:v>
       </x:c>
     </x:row>
     <x:row r="957" ht="58" customHeight="1">
@@ -26988,7 +26988,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I957" s="9" t="str">
-        <x:v>Broad observational MASLD/MASH screening pathway — entry needs T2DM, metabolic syndrome, obesity, or hypertension. Patient qualifies twice: established T2DM w/ hyperglycemia and polyneuropathy (glucose 157, 225), and treated essential hypertension. Exclusions target competing liver etiologies, not comorbidity, so his cardiac/infectious illness doesn't affect eligibility. Key open item: alcohol dependence IN REMISSION — exclusion is phrased as current excessive intake, which remission argues against, but lifetime intake must be quantified since alcohol is the main competing fibrosis etiology. No hepatitis B/C, HIV, or other liver disease; ALT 25, albumin 3.5, platelets 163 all reassuring. HDL 42 fails the &lt;40 male metabolic-syndrome component but T2DM qualifies independently. Not enrollable while in ICU with cardiogenic/septic shock — timing, not eligibility. Opioid dependence and coded medication noncompliance bear on 5-yr follow-up adherence.</x:v>
+        <x:v>Broad observational MASLD/MASH screening pathway, entry needs T2DM, metabolic syndrome, obesity, or hypertension. Patient qualifies twice: established T2DM w/ hyperglycemia and polyneuropathy (glucose 157, 225), and treated essential hypertension. Exclusions target competing liver etiologies, not comorbidity, so his cardiac/infectious illness doesn't affect eligibility. Key open item: alcohol dependence IN REMISSION, exclusion is phrased as current excessive intake, which remission argues against, but lifetime intake must be quantified since alcohol is the main competing fibrosis etiology. No hepatitis B/C, HIV, or other liver disease; ALT 25, albumin 3.5, platelets 163 all reassuring. HDL 42 fails the &lt;40 male metabolic-syndrome component but T2DM qualifies independently. Not enrollable while in ICU with cardiogenic/septic shock, timing, not eligibility. Opioid dependence and coded medication noncompliance bear on 5-yr follow-up adherence.</x:v>
       </x:c>
     </x:row>
     <x:row r="958" ht="58" customHeight="1">
@@ -27017,7 +27017,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I958" s="9" t="str">
-        <x:v>Phenotype is a direct hit (T2DM + systolic HF), age 63 and Cr 0.8 clear the age and eGFR criteria — fails on timing/stability. Trial needs HF established BEFORE screening with imaging in prior 6 mo, stable GDMT dosing, and no cardiovascular event within 3 months. Patient is mid-event: cardiogenic shock, acute systolic HF, Takotsubo, severe sepsis w/ septic shock this admission, plus coded medication noncompliance — GDMT cannot be stable. HF appears newly diagnosed, and the Takotsubo component may be reversible, so persistence of reduced EF is the pivotal unknown. Active opioid dependence is a discretionary adherence barrier against a 4-MRI protocol with 8 draws in one visit and daily dosing. SGLT2i use unverified and would exclude — worth checking, possibly washout-resolvable. FLAG FOR RE-SCREEN at 3–6 months if EF stays reduced on stable GDMT.</x:v>
+        <x:v>Phenotype is a direct hit (T2DM + systolic HF), age 63 and Cr 0.8 clear the age and eGFR criteria, fails on timing/stability. Trial needs HF established BEFORE screening with imaging in prior 6 mo, stable GDMT dosing, and no cardiovascular event within 3 months. Patient is mid-event: cardiogenic shock, acute systolic HF, Takotsubo, severe sepsis w/ septic shock this admission, plus coded medication noncompliance, GDMT cannot be stable. HF appears newly diagnosed, and the Takotsubo component may be reversible, so persistence of reduced EF is the pivotal unknown. Active opioid dependence is a discretionary adherence barrier against a 4-MRI protocol with 8 draws in one visit and daily dosing. SGLT2i use unverified and would exclude, worth checking, possibly washout-resolvable. FLAG FOR RE-SCREEN at 3–6 months if EF stays reduced on stable GDMT.</x:v>
       </x:c>
     </x:row>
     <x:row r="959" ht="58" customHeight="1">
@@ -27046,7 +27046,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I959" s="9" t="str">
-        <x:v>Hong Kong community digital lifestyle-education RCT for ambulatory adults 50+ with metabolic syndrome plus psychosomatic distress. Metabolic components are met (treated hypertension, previously diagnosed T2DM w/ glucose 157–225, coded hyperlipidemia; note HDL 42 fails the &lt;40 male sub-threshold but the treatment route holds), but the ANCHORING inclusion is central obesity by waist circumference and there is no waist, height, weight, or BMI in the record. The ≥2 distressing psychosomatic/stress symptoms requirement is also entirely undocumented — chronic pain is coded and opioid dependence suggests a pain history, but psychosomatic attribution and 6-month duration are not established. Cohort is Cantonese-language, Hong Kong-resident, requires independent tablet/internet use — definitional to the study, not incidental. Patient is meanwhile an ICU patient in cardiogenic and septic shock with dilated cardiomyopathy, not a community-dwelling participant. Another metabolic-tag match masking a different target population.</x:v>
+        <x:v>Hong Kong community digital lifestyle-education RCT for ambulatory adults 50+ with metabolic syndrome plus psychosomatic distress. Metabolic components are met (treated hypertension, previously diagnosed T2DM w/ glucose 157–225, coded hyperlipidemia; note HDL 42 fails the &lt;40 male sub-threshold but the treatment route holds), but the ANCHORING inclusion is central obesity by waist circumference and there is no waist, height, weight, or BMI in the record. The ≥2 distressing psychosomatic/stress symptoms requirement is also entirely undocumented, chronic pain is coded and opioid dependence suggests a pain history, but psychosomatic attribution and 6-month duration are not established. Cohort is Cantonese-language, Hong Kong-resident, requires independent tablet/internet use, definitional to the study, not incidental. Patient is meanwhile an ICU patient in cardiogenic and septic shock with dilated cardiomyopathy, not a community-dwelling participant. Another metabolic-tag match masking a different target population.</x:v>
       </x:c>
     </x:row>
     <x:row r="960" ht="58" customHeight="1">
@@ -27075,7 +27075,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I960" s="9" t="str">
-        <x:v>Minimal criteria: age ≥18 plus a diagnosis of hypertensive heart disease, with exclusions being the negation of each. Age clears; the diagnosis does not appear in the record. Patient has essential hypertension and extensive cardiac disease, but his HF is attributed to dilated cardiomyopathy, Takotsubo syndrome, and coronary atherosclerosis — not hypertensive heart disease. Absence looks meaningful rather than a documentation gap, since the coding system captures "hypertensive heart disease with heart failure" explicitly for another patient in this same package. Takotsubo is stress-mediated and typically reversible, a distinct entity from hypertensive remodeling. Study is a cross-sectional record review at a single Congolese tertiary hospital. RESOLVABLE BY ECHO — a hypertensive LVH phenotype would reclassify him. FLAG AS REVIEWER-DEPENDENT: with criteria this thin a lenient reading could reach MATCH; not a clear model error either way.</x:v>
+        <x:v>Minimal criteria: age ≥18 plus a diagnosis of hypertensive heart disease, with exclusions being the negation of each. Age clears; the diagnosis does not appear in the record. Patient has essential hypertension and extensive cardiac disease, but his HF is attributed to dilated cardiomyopathy, Takotsubo syndrome, and coronary atherosclerosis, not hypertensive heart disease. Absence looks meaningful rather than a documentation gap, since the coding system captures "hypertensive heart disease with heart failure" explicitly for another patient in this same package. Takotsubo is stress-mediated and typically reversible, a distinct entity from hypertensive remodeling. Study is a cross-sectional record review at a single Congolese tertiary hospital. RESOLVABLE BY ECHO, a hypertensive LVH phenotype would reclassify him. FLAG AS REVIEWER-DEPENDENT: with criteria this thin a lenient reading could reach MATCH; not a clear model error either way.</x:v>
       </x:c>
     </x:row>
     <x:row r="961" ht="58" customHeight="1">
@@ -27104,7 +27104,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I961" s="9" t="str">
-        <x:v>Dietary crossover trial (3 six-week arms, 15 visits) in metabolically stable adults, with exclusions designed to protect a clean microbiome/inflammation readout. Patient fails five ways: (1) heart failure within 1 year — acute systolic HF, dilated cardiomyopathy, cardiogenic shock, Takotsubo, high-priority exclusion; (2) thyroid disorder — hypothyroidism, flatly excluded despite TSH 1.3 meeting the inclusion threshold; (3) antibiotics within 6 months — certain given severe sepsis, septic shock, pneumonia, blood/urine cultures — directly confounds the microbiome endpoint; (4) inclusion requires CRP &lt;5 mg/L, impossible with septic shock and WBC 26.3; (5) no medication stable ≥14 days while on active ICU therapy. Waist circumference and BMI undocumented (waist is the gating inclusion). HDL 42 mg/dL ≈ 1.09 mmol/L is ABOVE the ≤1.0 male threshold so that component fails. Hgb 12.0 g/dL sits exactly at the 120 g/L floor. Dysphagia also relevant to a high-fiber food protocol. Heart failure excludes ≥1 yr; hypothyroidism excludes permanently as written.</x:v>
+        <x:v>Dietary crossover trial (3 six-week arms, 15 visits) in metabolically stable adults, with exclusions designed to protect a clean microbiome/inflammation readout. Patient fails five ways: (1) heart failure within 1 year, acute systolic HF, dilated cardiomyopathy, cardiogenic shock, Takotsubo, high-priority exclusion; (2) thyroid disorder, hypothyroidism, flatly excluded despite TSH 1.3 meeting the inclusion threshold; (3) antibiotics within 6 months, certain given severe sepsis, septic shock, pneumonia, blood/urine cultures, directly confounds the microbiome endpoint; (4) inclusion requires CRP &lt;5 mg/L, impossible with septic shock and WBC 26.3; (5) no medication stable ≥14 days while on active ICU therapy. Waist circumference and BMI undocumented (waist is the gating inclusion). HDL 42 mg/dL ≈ 1.09 mmol/L is ABOVE the ≤1.0 male threshold so that component fails. Hgb 12.0 g/dL sits exactly at the 120 g/L floor. Dysphagia also relevant to a high-fiber food protocol. Heart failure excludes ≥1 yr; hypothyroidism excludes permanently as written.</x:v>
       </x:c>
     </x:row>
     <x:row r="962" ht="58" customHeight="1">
@@ -27133,7 +27133,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I962" s="9" t="str">
-        <x:v>ED-based POCUS screening for PRE-SYMPTOMATIC Stage B heart failure. Patient meets both inclusion criteria (age 63 ≥45; treated hypertension AND T2DM w/ hyperglycemia and polyneuropathy) but trips two exclusions: history of heart failure — acute systolic HF and dilated cardiomyopathy coded, with cardiogenic shock and PA catheter — and symptoms of acute HF, with acute hypoxic respiratory failure (pO2 38, sat 69% on one gas). He is Stage C/D, the exact endpoint the study is trying to prevent people from reaching undetected. Exclusion is written on history, so recovery would not clear it. Currently also unable to tolerate the exam and adherence questionable for 3-month phone follow-up (opioid dependence, coded medication noncompliance). PAIR WITH 001004 — both early-detection trials where all inclusion criteria are met and a single prior-diagnosis exclusion decides it; good test of whether the model over-weights inclusion overlap.</x:v>
+        <x:v>ED-based POCUS screening for PRE-SYMPTOMATIC Stage B heart failure. Patient meets both inclusion criteria (age 63 ≥45; treated hypertension AND T2DM w/ hyperglycemia and polyneuropathy) but trips two exclusions: history of heart failure, acute systolic HF and dilated cardiomyopathy coded, with cardiogenic shock and PA catheter, and symptoms of acute HF, with acute hypoxic respiratory failure (pO2 38, sat 69% on one gas). He is Stage C/D, the exact endpoint the study is trying to prevent people from reaching undetected. Exclusion is written on history, so recovery would not clear it. Currently also unable to tolerate the exam and adherence questionable for 3-month phone follow-up (opioid dependence, coded medication noncompliance). PAIR WITH 001004, both early-detection trials where all inclusion criteria are met and a single prior-diagnosis exclusion decides it; good test of whether the model over-weights inclusion overlap.</x:v>
       </x:c>
     </x:row>
     <x:row r="963" ht="58" customHeight="1">
@@ -27162,7 +27162,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I963" s="9" t="str">
-        <x:v>Crossover time-restricted-eating trial (two 5-week hypocaloric phases, 10–12 wk washout) in ambulatory overweight adults with normal, impaired, or NON-INSULIN-TREATED T2DM. Diabetes qualifies him on entry (T2DM w/ hyperglycemia and polyneuropathy, glucose 157–225) but the severe-chronic-illness exclusion naming "recent cardiovascular event" applies directly: cardiogenic shock, acute systolic HF, dilated cardiomyopathy, Takotsubo, plus severe sepsis w/ septic shock, acute hypoxic respiratory failure, pneumonia. Anticoagulation likely unpausable (PTT 48.3–53.9, INR 1.3). Insulin status undocumented and would independently exclude — plausible given polyneuropathy and glucose 225. Weight stability improbable after septic-shock resuscitation. BMI, HbA1c, and eating-window all undocumented. Dysphagia coded, directly relevant to a structured feeding protocol. Caloric restriction here would be unsafe, not just ineligible.</x:v>
+        <x:v>Crossover time-restricted-eating trial (two 5-week hypocaloric phases, 10–12 wk washout) in ambulatory overweight adults with normal, impaired, or NON-INSULIN-TREATED T2DM. Diabetes qualifies him on entry (T2DM w/ hyperglycemia and polyneuropathy, glucose 157–225) but the severe-chronic-illness exclusion naming "recent cardiovascular event" applies directly: cardiogenic shock, acute systolic HF, dilated cardiomyopathy, Takotsubo, plus severe sepsis w/ septic shock, acute hypoxic respiratory failure, pneumonia. Anticoagulation likely unpausable (PTT 48.3–53.9, INR 1.3). Insulin status undocumented and would independently exclude, plausible given polyneuropathy and glucose 225. Weight stability improbable after septic-shock resuscitation. BMI, HbA1c, and eating-window all undocumented. Dysphagia coded, directly relevant to a structured feeding protocol. Caloric restriction here would be unsafe, not just ineligible.</x:v>
       </x:c>
     </x:row>
     <x:row r="964" ht="58" customHeight="1">
@@ -27191,7 +27191,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I964" s="9" t="str">
-        <x:v>Pragmatic primary-care trial of intensive BP targets vs cognitive decline, requiring age ≥70. Patient is 54 — 16 years under, criterion stated at high priority on BOTH inclusion and exclusion sides. Independently trips "major and unstable heart disease," which names acute systolic HF, ACS, and cardiac arrest: he has acute systolic HF, cardiogenic shock, and a resuscitated cardiac arrest with CPR and invasive mechanical ventilation (lactate 14.8, pH 7.13, base excess −12, sat 76%). Also congestive HF, coronary atherosclerosis, prior PCI, old MI, tricuspid and aortic valve disease, secondary pulmonary HTN. Not an ambulatory primary-care patient. Notably hypertension is NOT among his coded diagnoses, so even the BP inclusion is unsupported — weak pairing on every axis. Registry age_max field reads 70, conflicting with protocol text ("70 or older"); he falls outside either way.</x:v>
+        <x:v>Pragmatic primary-care trial of intensive BP targets vs cognitive decline, requiring age ≥70. Patient is 54, 16 years under, criterion stated at high priority on BOTH inclusion and exclusion sides. Independently trips "major and unstable heart disease," which names acute systolic HF, ACS, and cardiac arrest: he has acute systolic HF, cardiogenic shock, and a resuscitated cardiac arrest with CPR and invasive mechanical ventilation (lactate 14.8, pH 7.13, base excess −12, sat 76%). Also congestive HF, coronary atherosclerosis, prior PCI, old MI, tricuspid and aortic valve disease, secondary pulmonary HTN. Not an ambulatory primary-care patient. Notably hypertension is NOT among his coded diagnoses, so even the BP inclusion is unsupported, weak pairing on every axis. Registry age_max field reads 70, conflicting with protocol text ("70 or older"); he falls outside either way.</x:v>
       </x:c>
     </x:row>
     <x:row r="965" ht="58" customHeight="1">
@@ -27218,7 +27218,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I965" s="9" t="str">
-        <x:v>Strongest phenotype fit in the series. Trial enrolls comatose post-cardiac-arrest patients in vasopressor-dependent shock; patient presents with cardiac arrest + CPR, cardiogenic shock, invasive mechanical ventilation, central line, and severe shock physiology (lactate 14.8, pH 7.13, base excess −12, sat 76%). Presumed cardiac origin well supported — coronary atherosclerosis, old MI, PTCA status, acute systolic HF, dysrhythmias, sudden_cardiac_death tag — with no trauma, bleeding, or poisoning coded. Age 54 clears the ≥30 floor. No documented vitamin C contraindication (no urolithiasis, oxalate nephropathy, hemochromatosis, G6PD), no ECMO. TWO PIVOTAL UNKNOWNS: (1) out-of-hospital vs in-hospital arrest — trial requires OHCA; (2) vasopressor dose, since ≥2 µg/kg/h within 4h excludes the most refractory shock, plausible given his lactate. Also verify baseline eGFR — CKD tag and acute kidney failure coded, but exclusion targets PRE-EXISTING GFR &lt;30. Both key checks are answerable at the bedside in minutes. Practical constraint is the 6-hour randomization window, not eligibility.</x:v>
+        <x:v>Strongest phenotype fit in the series. Trial enrolls comatose post-cardiac-arrest patients in vasopressor-dependent shock; patient presents with cardiac arrest + CPR, cardiogenic shock, invasive mechanical ventilation, central line, and severe shock physiology (lactate 14.8, pH 7.13, base excess −12, sat 76%). Presumed cardiac origin well supported, coronary atherosclerosis, old MI, PTCA status, acute systolic HF, dysrhythmias, sudden_cardiac_death tag, with no trauma, bleeding, or poisoning coded. Age 54 clears the ≥30 floor. No documented vitamin C contraindication (no urolithiasis, oxalate nephropathy, hemochromatosis, G6PD), no ECMO. TWO PIVOTAL UNKNOWNS: (1) out-of-hospital vs in-hospital arrest, trial requires OHCA; (2) vasopressor dose, since ≥2 µg/kg/h within 4h excludes the most refractory shock, plausible given his lactate. Also verify baseline eGFR, CKD tag and acute kidney failure coded, but exclusion targets PRE-EXISTING GFR &lt;30. Both key checks are answerable at the bedside in minutes. Practical constraint is the 6-hour randomization window, not eligibility.</x:v>
       </x:c>
     </x:row>
     <x:row r="966" ht="58" customHeight="1">
@@ -27247,7 +27247,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I966" s="9" t="str">
-        <x:v>Home air-cleaner RCT in ambulatory adults with mild systolic hypertension (SBP 130–159) plus metabolic syndrome, Qatar-resident. High-priority exclusion for ANY cardiovascular disease — because the design requires tolerating home BP &gt;130/80 for 10 weeks — and patient has coronary atherosclerosis, old MI, PTCA status, acute systolic HF, congestive HF, cardiogenic shock, and resuscitated cardiac arrest, plus tricuspid/aortic valve disorders, secondary pulmonary HTN, transplanted valve, and CKD tag with acute kidney failure. Also fails the non-smoker inclusion: tobacco use disorder coded (active), against a 1-year abstinence requirement with cotinine verification. Acute illness within 4 weeks (post-arrest, lactate 14.8, pH 7.13, ventilated). No medication regimen stable. Chronic airway obstruction + OSA + mechanical ventilation likely trips the oxygen-requiring lung disease exclusion. Notably HYPERTENSION IS NOT CODED for this patient, so the qualifying condition itself is absent. Age 54 does clear the &lt;60 cap.</x:v>
+        <x:v>Home air-cleaner RCT in ambulatory adults with mild systolic hypertension (SBP 130–159) plus metabolic syndrome, Qatar-resident. High-priority exclusion for ANY cardiovascular disease, because the design requires tolerating home BP &gt;130/80 for 10 weeks, and patient has coronary atherosclerosis, old MI, PTCA status, acute systolic HF, congestive HF, cardiogenic shock, and resuscitated cardiac arrest, plus tricuspid/aortic valve disorders, secondary pulmonary HTN, transplanted valve, and CKD tag with acute kidney failure. Also fails the non-smoker inclusion: tobacco use disorder coded (active), against a 1-year abstinence requirement with cotinine verification. Acute illness within 4 weeks (post-arrest, lactate 14.8, pH 7.13, ventilated). No medication regimen stable. Chronic airway obstruction + OSA + mechanical ventilation likely trips the oxygen-requiring lung disease exclusion. Notably HYPERTENSION IS NOT CODED for this patient, so the qualifying condition itself is absent. Age 54 does clear the &lt;60 cap.</x:v>
       </x:c>
     </x:row>
     <x:row r="967" ht="58" customHeight="1">
@@ -27276,7 +27276,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I967" s="9" t="str">
-        <x:v>Renal denervation pivotal trial requiring documented hypertension plus willingness to stop all antihypertensives for 4-wk washout and 2 mo post-procedure. Hypertension is NOT coded for this patient — qualifying diagnosis absent. Trips high-priority exclusion for severe CV event within 12 months: acute systolic HF requiring hospitalization, cardiogenic shock, resuscitated cardiac arrest, plus old MI and PTCA status. Antihypertensive washout would be unsafe given ischemic cardiomyopathy and HF — protocol has a separate exclusion for exactly this. Also excluded by continuous invasive mechanical ventilation (permitted only as nocturnal sleep-apnea support) and likely by severe valvular disease (tricuspid valve disease, aortic valve disorders, heart valve replaced by transplant, with secondary pulmonary HTN). Note his pulmonary HTN is SECONDARY so that specific exclusion does not fire. Age 54 clears 22–75. THIRD CONSECUTIVE PAIR matching him to an ambulatory hypertension study despite no hypertension diagnosis — systematic retrieval pattern, not three independent errors.</x:v>
+        <x:v>Renal denervation pivotal trial requiring documented hypertension plus willingness to stop all antihypertensives for 4-wk washout and 2 mo post-procedure. Hypertension is NOT coded for this patient, qualifying diagnosis absent. Trips high-priority exclusion for severe CV event within 12 months: acute systolic HF requiring hospitalization, cardiogenic shock, resuscitated cardiac arrest, plus old MI and PTCA status. Antihypertensive washout would be unsafe given ischemic cardiomyopathy and HF, protocol has a separate exclusion for exactly this. Also excluded by continuous invasive mechanical ventilation (permitted only as nocturnal sleep-apnea support) and likely by severe valvular disease (tricuspid valve disease, aortic valve disorders, heart valve replaced by transplant, with secondary pulmonary HTN). Note his pulmonary HTN is SECONDARY so that specific exclusion does not fire. Age 54 clears 22–75. THIRD CONSECUTIVE PAIR matching him to an ambulatory hypertension study despite no hypertension diagnosis, systematic retrieval pattern, not three independent errors.</x:v>
       </x:c>
     </x:row>
     <x:row r="968" ht="58" customHeight="1">
@@ -27305,7 +27305,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I968" s="9" t="str">
-        <x:v>Swan-Ganz hemodynamic study in cardiogenic shock DUE TO ACUTE MI. Patient has cardiogenic shock with clear end-organ hypoperfusion (lactate 14.8, pH 7.13, base excess −12, acute kidney failure) and would meet the shock criteria, but is excluded by "cardiac arrest prior to Swan-Ganz catheterization" — arrest with CPR affirmatively documented, plus invasive mechanical ventilation. Also fails the required etiology: MI is coded as OLD, with coronary atherosclerosis and PTCA status but no acute infarct this encounter; the trial's early-revascularization pathway doesn't apply. Valve findings (transplanted valve, tricuspid disease, aortic valve disorders) are acquired, not congenital, so that exclusion likely doesn't fire. INR/platelets unavailable for the coagulopathy check. Single-site Bach Mai Hospital. CONTRAST PAIR WITH 001026 — same patient, same clinical picture, opposite verdicts, because one trial requires post-arrest shock and this one excludes it. Strong probe for criteria-direction sensitivity.</x:v>
+        <x:v>Swan-Ganz hemodynamic study in cardiogenic shock DUE TO ACUTE MI. Patient has cardiogenic shock with clear end-organ hypoperfusion (lactate 14.8, pH 7.13, base excess −12, acute kidney failure) and would meet the shock criteria, but is excluded by "cardiac arrest prior to Swan-Ganz catheterization", arrest with CPR affirmatively documented, plus invasive mechanical ventilation. Also fails the required etiology: MI is coded as OLD, with coronary atherosclerosis and PTCA status but no acute infarct this encounter; the trial's early-revascularization pathway doesn't apply. Valve findings (transplanted valve, tricuspid disease, aortic valve disorders) are acquired, not congenital, so that exclusion likely doesn't fire. INR/platelets unavailable for the coagulopathy check. Single-site Bach Mai Hospital. CONTRAST PAIR WITH 001026, same patient, same clinical picture, opposite verdicts, because one trial requires post-arrest shock and this one excludes it. Strong probe for criteria-direction sensitivity.</x:v>
       </x:c>
     </x:row>
     <x:row r="969" ht="58" customHeight="1">
@@ -27334,7 +27334,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I969" s="9" t="str">
-        <x:v>Biomarker cohort sampling patients in the post-primary-PCI window after acute MI who develop protocol-defined ischemia-reperfusion injury. Patient's infarct is coded OLD and his PCI appears as PTCA STATUS — both historical. No acute infarct, no coronary angiography, no PCI in this encounter; documented procedures are CPR, central line, mechanical ventilation, PICC. Without the index revascularization there is no reperfusion injury to characterize — an event, not a workup item. Independently excluded by advanced heart failure NYHA III–IV: acute systolic HF, congestive HF, cardiogenic shock on mechanical ventilation. Refractory VT/VF exclusion likely also fires — cardiac arrest with CPR, other specified cardiac dysrhythmias, sudden_cardiac_death tag — though arrest rhythm isn't specified. No active infection (WBC 9.3), no malignancy, no cerebrovascular event. eGFR unavailable for the renal check. Alt mechanism label: Procedure/imaging unmet. Recurring theme for this patient — several trials hinge on acute vs historical MI/PCI, and the coding is clearly historical.</x:v>
+        <x:v>Biomarker cohort sampling patients in the post-primary-PCI window after acute MI who develop protocol-defined ischemia-reperfusion injury. Patient's infarct is coded OLD and his PCI appears as PTCA STATUS, both historical. No acute infarct, no coronary angiography, no PCI in this encounter; documented procedures are CPR, central line, mechanical ventilation, PICC. Without the index revascularization there is no reperfusion injury to characterize, an event, not a workup item. Independently excluded by advanced heart failure NYHA III–IV: acute systolic HF, congestive HF, cardiogenic shock on mechanical ventilation. Refractory VT/VF exclusion likely also fires, cardiac arrest with CPR, other specified cardiac dysrhythmias, sudden_cardiac_death tag, though arrest rhythm isn't specified. No active infection (WBC 9.3), no malignancy, no cerebrovascular event. eGFR unavailable for the renal check. Alt mechanism label: Procedure/imaging unmet. Recurring theme for this patient, several trials hinge on acute vs historical MI/PCI, and the coding is clearly historical.</x:v>
       </x:c>
     </x:row>
     <x:row r="970" ht="58" customHeight="1">
@@ -27363,7 +27363,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I970" s="9" t="str">
-        <x:v>Third pairing to this CRS biomarker cohort, and the first patient who CLEARS the 18–75 age gate (54). Fails instead on state and lookback: cohort requires STABLE chronic HF followed 12 months, and he is in acute systolic HF with cardiogenic shock, resuscitated cardiac arrest, CPR, and invasive mechanical ventilation (lactate 14.8, pH 7.13, base excess −12). Acute kidney failure coded this encounter trips the explicit AKI-within-3-months exclusion, which is history-based and holds even after renal recovery. Nephrotoxic exposure likely (vasopressors, probable contrast) but unverifiable. No dialysis, no autoimmune disease, no malignancy, no liver disease; WBC 9.3 so no active infection. LVEF undocumented — acute systolic HF suggests HFrEF. BOTH FAILURES ARE TIME-ANCHORED, NOT PERMANENT — flag for re-screen if he recovers, regains renal function, and is &gt;3 months out on stable GDMT; phenotype fits the panel well. Three pairings to this protocol now, three different failure mechanisms across three patients.</x:v>
+        <x:v>Third pairing to this CRS biomarker cohort, and the first patient who CLEARS the 18–75 age gate (54). Fails instead on state and lookback: cohort requires STABLE chronic HF followed 12 months, and he is in acute systolic HF with cardiogenic shock, resuscitated cardiac arrest, CPR, and invasive mechanical ventilation (lactate 14.8, pH 7.13, base excess −12). Acute kidney failure coded this encounter trips the explicit AKI-within-3-months exclusion, which is history-based and holds even after renal recovery. Nephrotoxic exposure likely (vasopressors, probable contrast) but unverifiable. No dialysis, no autoimmune disease, no malignancy, no liver disease; WBC 9.3 so no active infection. LVEF undocumented, acute systolic HF suggests HFrEF. BOTH FAILURES ARE TIME-ANCHORED, NOT PERMANENT, flag for re-screen if he recovers, regains renal function, and is &gt;3 months out on stable GDMT; phenotype fits the panel well. Three pairings to this protocol now, three different failure mechanisms across three patients.</x:v>
       </x:c>
     </x:row>
     <x:row r="971" ht="58" customHeight="1">
@@ -27392,7 +27392,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I971" s="9" t="str">
-        <x:v>Serial CMR perfusion cohort in obstructive HCM followed in an outpatient HCM clinic. Patient has no hypertrophic cardiomyopathy of any kind — no LVOT obstruction, no septal hypertrophy; his disease is ischemic and valvular (coronary atherosclerosis, old MI, PTCA status, acute systolic HF, tricuspid and aortic valve disorders). HOCM features preserved/hyperdynamic systolic function, the opposite of his acute systolic failure with cardiogenic shock. Trips two named exclusions: significant CAD and/or prior stent/CABG — the exact confounder the criterion screens out — and sudden cardiac arrest or sustained VA within 12 months, documented with CPR this admission plus sudden_cardiac_death tag. Also no baseline clinical CMR perfusion scan, which the enrollment design presupposes, and 6MWT is unperformable on invasive mechanical ventilation. eGFR unavailable, relevant to contrast administration. PAIR WITH 001010 — same error pattern inverted: ischemic HF patient matched to a study requiring non-ischemic cardiomyopathy and excluding coronary disease.</x:v>
+        <x:v>Serial CMR perfusion cohort in obstructive HCM followed in an outpatient HCM clinic. Patient has no hypertrophic cardiomyopathy of any kind, no LVOT obstruction, no septal hypertrophy; his disease is ischemic and valvular (coronary atherosclerosis, old MI, PTCA status, acute systolic HF, tricuspid and aortic valve disorders). HOCM features preserved/hyperdynamic systolic function, the opposite of his acute systolic failure with cardiogenic shock. Trips two named exclusions: significant CAD and/or prior stent/CABG, the exact confounder the criterion screens out, and sudden cardiac arrest or sustained VA within 12 months, documented with CPR this admission plus sudden_cardiac_death tag. Also no baseline clinical CMR perfusion scan, which the enrollment design presupposes, and 6MWT is unperformable on invasive mechanical ventilation. eGFR unavailable, relevant to contrast administration. PAIR WITH 001010, same error pattern inverted: ischemic HF patient matched to a study requiring non-ischemic cardiomyopathy and excluding coronary disease.</x:v>
       </x:c>
     </x:row>
     <x:row r="972" ht="58" customHeight="1">
@@ -27421,7 +27421,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I972" s="9" t="str">
-        <x:v>Observational SGLT2i cohort in HFpEF + CKD stage 3–4, with endothelial function (FMD), pulse wave velocity, and IMT as core measures. High-priority exclusion for coronary artery disease — including prior ACS or angiography showing significant lesions — fires directly: coronary atherosclerosis of native coronary artery, old MI, PTCA status. Prior angioplasty also likely means a coronary stent, separately excluded. Phenotype fails too: trial requires EF &gt;40% (HFpEF) and he has acute systolic HF with cardiogenic shock after resuscitated arrest; LVEF undocumented but reduced EF is the likely picture given old MI and ischemic substrate. CKD staging can't be established — CKD tag and acute kidney failure coded but no creatinine values; eGFR &lt;15/dialysis not documented so that exclusion doesn't fire. No active infection (WBC 9.3); valvular findings are acquired not congenital. FMD/PWV/IMT are outpatient measures, unperformable on a ventilated post-arrest patient.</x:v>
+        <x:v>Observational SGLT2i cohort in HFpEF + CKD stage 3–4, with endothelial function (FMD), pulse wave velocity, and IMT as core measures. High-priority exclusion for coronary artery disease, including prior ACS or angiography showing significant lesions, fires directly: coronary atherosclerosis of native coronary artery, old MI, PTCA status. Prior angioplasty also likely means a coronary stent, separately excluded. Phenotype fails too: trial requires EF &gt;40% (HFpEF) and he has acute systolic HF with cardiogenic shock after resuscitated arrest; LVEF undocumented but reduced EF is the likely picture given old MI and ischemic substrate. CKD staging can't be established, CKD tag and acute kidney failure coded but no creatinine values; eGFR &lt;15/dialysis not documented so that exclusion doesn't fire. No active infection (WBC 9.3); valvular findings are acquired not congenital. FMD/PWV/IMT are outpatient measures, unperformable on a ventilated post-arrest patient.</x:v>
       </x:c>
     </x:row>
     <x:row r="973" ht="58" customHeight="1">
@@ -27450,7 +27450,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I973" s="9" t="str">
-        <x:v>Testosterone undecanoate RCT for hepatic fat in hypogonadal men with T2DM/prediabetes. Metabolic entry fits — 47M, T2DM with nephropathy/polyneuropathy/retinopathy/foot ulcer, glucose 150–154, obesity coded, hyperlipidemia — and untested testosterone would be a routine screening lab, not a disqualifier. EPILEPSY is a named flat exclusion and is coded twice plus "other convulsions"; non-intractable status gives no carve-out. Also active osteomyelitis of ankle/foot with cellulitis, chronic foot ulcers, infected amputation stump, MRSA history — safety/stability barrier to a 160-week protocol. Long-term antiplatelet/antithrombotic and aspirin use conflicts with the deep IM depot injection route, compounded by thrombocytopenia (plt 150–171). Cr 1.3 is under the &gt;1.5 cutoff but marginal with CKD III plus AKI. Hct 34% clears the &gt;50% exclusion. Bipolar I with documented mood instability and CP with contractures bear on adherence and MRI feasibility. Good test of whether a model catches one named exclusion buried in a long comorbidity list.</x:v>
+        <x:v>Testosterone undecanoate RCT for hepatic fat in hypogonadal men with T2DM/prediabetes. Metabolic entry fits, 47M, T2DM with nephropathy/polyneuropathy/retinopathy/foot ulcer, glucose 150–154, obesity coded, hyperlipidemia, and untested testosterone would be a routine screening lab, not a disqualifier. EPILEPSY is a named flat exclusion and is coded twice plus "other convulsions"; non-intractable status gives no carve-out. Also active osteomyelitis of ankle/foot with cellulitis, chronic foot ulcers, infected amputation stump, MRSA history, safety/stability barrier to a 160-week protocol. Long-term antiplatelet/antithrombotic and aspirin use conflicts with the deep IM depot injection route, compounded by thrombocytopenia (plt 150–171). Cr 1.3 is under the &gt;1.5 cutoff but marginal with CKD III plus AKI. Hct 34% clears the &gt;50% exclusion. Bipolar I with documented mood instability and CP with contractures bear on adherence and MRI feasibility. Good test of whether a model catches one named exclusion buried in a long comorbidity list.</x:v>
       </x:c>
     </x:row>
     <x:row r="974" ht="58" customHeight="1">
@@ -27479,7 +27479,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I974" s="9" t="str">
-        <x:v>PEMF device trial for ischemic burden in CAD, anchored on cardiopulmonary exercise testing. Two clean failures. (1) SEIZURES is a named exclusion and epilepsy is coded twice plus "other convulsions" — mechanistically relevant to an electromagnetic field device. (2) Both the inclusion ("able to complete CPET without significant non-cardiac limitations, primarily orthopedic") and the matching exclusion fire: spastic diplegic cerebral palsy, left ankle and right lower leg contractures, bilateral tendon divisions, acquired absence of right great toe, bilateral chronic foot ulcers, active osteomyelitis of ankle/foot. Limitation is severe and permanent. Also no documented ischemia — coronary atherosclerosis is coded but no stress test, perfusion imaging, or ischemic ECG within 6 months, and no LVEF. Labs clear the other thresholds: Hgb 11.5, K 4.9, Cr 1.3. No arrhythmia coded. Second consecutive pair for this patient where a documented seizure disorder is a named exclusion.</x:v>
+        <x:v>PEMF device trial for ischemic burden in CAD, anchored on cardiopulmonary exercise testing. Two clean failures. (1) SEIZURES is a named exclusion and epilepsy is coded twice plus "other convulsions", mechanistically relevant to an electromagnetic field device. (2) Both the inclusion ("able to complete CPET without significant non-cardiac limitations, primarily orthopedic") and the matching exclusion fire: spastic diplegic cerebral palsy, left ankle and right lower leg contractures, bilateral tendon divisions, acquired absence of right great toe, bilateral chronic foot ulcers, active osteomyelitis of ankle/foot. Limitation is severe and permanent. Also no documented ischemia, coronary atherosclerosis is coded but no stress test, perfusion imaging, or ischemic ECG within 6 months, and no LVEF. Labs clear the other thresholds: Hgb 11.5, K 4.9, Cr 1.3. No arrhythmia coded. Second consecutive pair for this patient where a documented seizure disorder is a named exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="975" ht="58" customHeight="1">
@@ -27508,7 +27508,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I975" s="9" t="str">
-        <x:v>Device RCT (contractility modulation vs CRT) in serologically confirmed Chagas cardiomyopathy with NYHA II–III and LVEF &lt;35%. Patient has no Chagas disease, no T. cruzi serology, no exposure history — and NO heart failure diagnosis of any kind, no systolic dysfunction, no LVEF documented. Every core inclusion fails; his cardiac record is coronary atherosclerosis plus unspecified mitral valve disorders. Also trips named exclusions: peripheral polyneuropathy (diabetic polyneuropathy coded three ways) and other concomitant cardiovascular disease including uncontrolled diabetes (NIDDM neuro/renal/other manifestations all coded UNCONTROLLED, plus uncontrolled ophthalmic manifestations, background retinopathy, glucose 150–154). Renal exclusion likely does NOT fire — Cr 1.3 under the &gt;1.5 cutoff, CKD III implies eGFR 30–59. Bipolar I coded; psychotic features unspecified so the psychosis exclusion is interpretation-dependent. CLEAN NEGATIVE CONTROL — anything other than NO MATCH here is a meaningful model failure.</x:v>
+        <x:v>Device RCT (contractility modulation vs CRT) in serologically confirmed Chagas cardiomyopathy with NYHA II–III and LVEF &lt;35%. Patient has no Chagas disease, no T. cruzi serology, no exposure history, and NO heart failure diagnosis of any kind, no systolic dysfunction, no LVEF documented. Every core inclusion fails; his cardiac record is coronary atherosclerosis plus unspecified mitral valve disorders. Also trips named exclusions: peripheral polyneuropathy (diabetic polyneuropathy coded three ways) and other concomitant cardiovascular disease including uncontrolled diabetes (NIDDM neuro/renal/other manifestations all coded UNCONTROLLED, plus uncontrolled ophthalmic manifestations, background retinopathy, glucose 150–154). Renal exclusion likely does NOT fire, Cr 1.3 under the &gt;1.5 cutoff, CKD III implies eGFR 30–59. Bipolar I coded; psychotic features unspecified so the psychosis exclusion is interpretation-dependent. CLEAN NEGATIVE CONTROL, anything other than NO MATCH here is a meaningful model failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="976" ht="58" customHeight="1">
@@ -27537,7 +27537,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I976" s="9" t="str">
-        <x:v>ED cardioversion RCT whose entry event is paroxysmal AF documented by 12-lead ECG. Patient has NO atrial fibrillation — no AF, no flutter, no arrhythmia of any kind coded. He has only the coronary context (coronary atherosclerosis of native coronary artery), which is the qualifying background, not the enrollment presentation. Also fails "CAD without residual ischemia": no PCI, no CABG, no stress testing, so his CAD is unrevascularized and unassessed — the safety precondition for flecainide is unmet and the mirrored exclusion for known stenosis without revascularization may apply. Severe-systemic-disease exclusion likely fires: osteomyelitis of ankle/foot, cellulitis of limb, toe and foot, infected amputation stump, chronic bilateral foot ulcers, MRSA history, long-term antibiotics. CKD is stage III so the stage ≥4 exclusion does NOT fire (Cr 1.3). LVEF never measured. Registry age field 30–48 conflicts with protocol text 18–85; he satisfies both. STRUCTURAL TWIN OF PAIR-001006 — right comorbidity background, absent index event.</x:v>
+        <x:v>ED cardioversion RCT whose entry event is paroxysmal AF documented by 12-lead ECG. Patient has NO atrial fibrillation, no AF, no flutter, no arrhythmia of any kind coded. He has only the coronary context (coronary atherosclerosis of native coronary artery), which is the qualifying background, not the enrollment presentation. Also fails "CAD without residual ischemia": no PCI, no CABG, no stress testing, so his CAD is unrevascularized and unassessed, the safety precondition for flecainide is unmet and the mirrored exclusion for known stenosis without revascularization may apply. Severe-systemic-disease exclusion likely fires: osteomyelitis of ankle/foot, cellulitis of limb, toe and foot, infected amputation stump, chronic bilateral foot ulcers, MRSA history, long-term antibiotics. CKD is stage III so the stage ≥4 exclusion does NOT fire (Cr 1.3). LVEF never measured. Registry age field 30–48 conflicts with protocol text 18–85; he satisfies both. STRUCTURAL TWIN OF PAIR-001006, right comorbidity background, absent index event.</x:v>
       </x:c>
     </x:row>
     <x:row r="977" ht="58" customHeight="1">
@@ -27566,7 +27566,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I977" s="9" t="str">
-        <x:v>Aspiration thrombectomy device trial for acute PE with CTA-confirmed main/lobar filling defect and RV/LV ratio &gt;0.9. Patient has no pulmonary embolism, no DVT, no VTE of any kind — no CTA, no echo, no RV strain, no dyspnea/chest pain/hypoxemia. Admission is for diabetic foot infection with osteomyelitis, cellulitis, toe amputation, and debridement. Vascular pathology is arterial and microvascular (coronary atherosclerosis, diabetic complications), not venous. No thrombus to aspirate. Notable that his labs CLEAR nearly every exclusion threshold — platelets 150–171 (&gt;100k despite coded thrombocytopenia), Hct 34% (&gt;28%), Cr 1.3 (&lt;1.8) — so the failure is entirely on the inclusion side, which makes this a clean single-axis negative. PAIRS WITH 001005: second PE-related trial matched to a patient with purely arterial disease, suggesting the retrieval may conflate arterial and venous vascular tags.</x:v>
+        <x:v>Aspiration thrombectomy device trial for acute PE with CTA-confirmed main/lobar filling defect and RV/LV ratio &gt;0.9. Patient has no pulmonary embolism, no DVT, no VTE of any kind, no CTA, no echo, no RV strain, no dyspnea/chest pain/hypoxemia. Admission is for diabetic foot infection with osteomyelitis, cellulitis, toe amputation, and debridement. Vascular pathology is arterial and microvascular (coronary atherosclerosis, diabetic complications), not venous. No thrombus to aspirate. Notable that his labs CLEAR nearly every exclusion threshold, platelets 150–171 (&gt;100k despite coded thrombocytopenia), Hct 34% (&gt;28%), Cr 1.3 (&lt;1.8), so the failure is entirely on the inclusion side, which makes this a clean single-axis negative. PAIRS WITH 001005: second PE-related trial matched to a patient with purely arterial disease, suggesting the retrieval may conflate arterial and venous vascular tags.</x:v>
       </x:c>
     </x:row>
     <x:row r="978" ht="58" customHeight="1">
@@ -27595,7 +27595,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I978" s="9" t="str">
-        <x:v>HD-tDCS plus Chlorella supplement trial in long COVID patients with cardiovascular risk. Patient has the CV risk (coronary atherosclerosis, hypertensive CKD, hyperlipidemia, T2DM with multiple complications, obesity, mitral valve disorders) but NO COVID-19 infection and no post-COVID syndrome anywhere in the record — defining population absent. Study design specifies participants whose index hospitalization was for COVID; his is for diabetic foot infection with osteomyelitis and amputation. Independently trips the high-priority exclusion for neuromuscular or cognitive instability and neurostimulation contraindications: spastic diplegic cerebral palsy with bilateral contractures and tendon divisions, EPILEPSY with convulsions (standard contraindication to tDCS over primary motor cortex — safety, not technicality), bipolar I disorder with impulsiveness and psychotropic adverse effects, Asperger's/pervasive developmental disorder. THIRD OF SIX PAIRS for this patient where the seizure disorder is decisive, second where cerebral palsy is — a model reasoning only from cardiometabolic tags would miss both.</x:v>
+        <x:v>HD-tDCS plus Chlorella supplement trial in long COVID patients with cardiovascular risk. Patient has the CV risk (coronary atherosclerosis, hypertensive CKD, hyperlipidemia, T2DM with multiple complications, obesity, mitral valve disorders) but NO COVID-19 infection and no post-COVID syndrome anywhere in the record, defining population absent. Study design specifies participants whose index hospitalization was for COVID; his is for diabetic foot infection with osteomyelitis and amputation. Independently trips the high-priority exclusion for neuromuscular or cognitive instability and neurostimulation contraindications: spastic diplegic cerebral palsy with bilateral contractures and tendon divisions, EPILEPSY with convulsions (standard contraindication to tDCS over primary motor cortex, safety, not technicality), bipolar I disorder with impulsiveness and psychotropic adverse effects, Asperger's/pervasive developmental disorder. THIRD OF SIX PAIRS for this patient where the seizure disorder is decisive, second where cerebral palsy is, a model reasoning only from cardiometabolic tags would miss both.</x:v>
       </x:c>
     </x:row>
     <x:row r="979" ht="58" customHeight="1">
@@ -27624,7 +27624,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I979" s="9" t="str">
-        <x:v>Phase IIa plaque-regression study in coronary atherosclerosis with serial coronary CTA endpoints. Closest fit in this patient's series — target diagnosis present (coronary atherosclerosis of native coronary artery) and age 47 within 18–75. Defeated by a flat "presence of renal insufficiency" exclusion with no numeric carve-out: CKD stage III, hypertensive CKD, diabetic CKD with nephropathy, plus coded acute kidney failure (Cr 1.3, BUN 23, Na 132). Second exclusion also fires — major disease not recovered within 2 weeks: osteomyelitis of ankle/foot, cellulitis of limb/toe/foot, infected amputation stump, bilateral chronic foot ulcers with fat layer exposed, recent toe amputation and debridements, with further foot surgery foreseeable. Renal status likely contraindicates the two contrast CTAs the primary endpoint requires. HbA1c not measured but diabetes coded UNCONTROLLED with renal/neuro/ophthalmic manifestations — &gt;9% plausible, would independently exclude. No CCTA on record to establish the required stenosis. Australia site is logistical, not verdict-carrying. Failure here is comorbidity-threshold driven rather than diagnosis driven — different mechanism from his other pairs.</x:v>
+        <x:v>Phase IIa plaque-regression study in coronary atherosclerosis with serial coronary CTA endpoints. Closest fit in this patient's series, target diagnosis present (coronary atherosclerosis of native coronary artery) and age 47 within 18–75. Defeated by a flat "presence of renal insufficiency" exclusion with no numeric carve-out: CKD stage III, hypertensive CKD, diabetic CKD with nephropathy, plus coded acute kidney failure (Cr 1.3, BUN 23, Na 132). Second exclusion also fires, major disease not recovered within 2 weeks: osteomyelitis of ankle/foot, cellulitis of limb/toe/foot, infected amputation stump, bilateral chronic foot ulcers with fat layer exposed, recent toe amputation and debridements, with further foot surgery foreseeable. Renal status likely contraindicates the two contrast CTAs the primary endpoint requires. HbA1c not measured but diabetes coded UNCONTROLLED with renal/neuro/ophthalmic manifestations, &gt;9% plausible, would independently exclude. No CCTA on record to establish the required stenosis. Australia site is logistical, not verdict-carrying. Failure here is comorbidity-threshold driven rather than diagnosis driven, different mechanism from his other pairs.</x:v>
       </x:c>
     </x:row>
     <x:row r="980" ht="58" customHeight="1">
@@ -27653,7 +27653,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I980" s="9" t="str">
-        <x:v>Trial enrolls patients ≥1 year AFTER drug-coated balloon angioplasty who completed 1–3 mo DAPT and stayed event-free on single antiplatelet, then randomizes to discontinue. Patient has never had DCB angioplasty, PCI, or any coronary revascularization — coronary atherosclerosis is unrevascularized and not angiographically characterized; documented procedures are foot debridement, toe amputation, bilateral tendon divisions. The index procedure that anchors enrollment does not exist, so the DAPT course and the year of event-free maintenance are all unmeetable. His long-term aspirin/antiplatelet use is prevention, not post-DCB maintenance. High bleeding risk also NOT established: age 47 (&lt;75), Hgb 11.5 (just above the &lt;11 threshold), platelets 150–171 (above &lt;100k despite coded thrombocytopenia), CrCl likely &gt;40 with CKD III and Cr 1.3, no intracranial bleed, no bleeding admission, no cancer, no liver disease — only criterion K (expected non-compliance) is arguable via bipolar I and conduct disturbance. High-priority stroke/MI exclusion does NOT fire. PAOD not coded but plausible given diabetic foot ulcers and toe amputation. Procedure-anchored failure, distinct from the diagnosis-anchored ones elsewhere in his series.</x:v>
+        <x:v>Trial enrolls patients ≥1 year AFTER drug-coated balloon angioplasty who completed 1–3 mo DAPT and stayed event-free on single antiplatelet, then randomizes to discontinue. Patient has never had DCB angioplasty, PCI, or any coronary revascularization, coronary atherosclerosis is unrevascularized and not angiographically characterized; documented procedures are foot debridement, toe amputation, bilateral tendon divisions. The index procedure that anchors enrollment does not exist, so the DAPT course and the year of event-free maintenance are all unmeetable. His long-term aspirin/antiplatelet use is prevention, not post-DCB maintenance. High bleeding risk also NOT established: age 47 (&lt;75), Hgb 11.5 (just above the &lt;11 threshold), platelets 150–171 (above &lt;100k despite coded thrombocytopenia), CrCl likely &gt;40 with CKD III and Cr 1.3, no intracranial bleed, no bleeding admission, no cancer, no liver disease, only criterion K (expected non-compliance) is arguable via bipolar I and conduct disturbance. High-priority stroke/MI exclusion does NOT fire. PAOD not coded but plausible given diabetic foot ulcers and toe amputation. Procedure-anchored failure, distinct from the diagnosis-anchored ones elsewhere in his series.</x:v>
       </x:c>
     </x:row>
     <x:row r="981" ht="58" customHeight="1">
@@ -27682,7 +27682,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I981" s="9" t="str">
-        <x:v>Phase 1b MAD study in symptomatic HFmrEF/HFpEF (NYHA II–III, LVEF &gt;40%, stable GDMT, plus NT-proBNP/echo or invasive filling-pressure criteria). Patient has NO heart failure diagnosis of any kind — no LVEF, no echo, no natriuretic peptides, no diuretic therapy, no HF hospitalization, no catheterization. Every route to satisfying the biomarker/echo criterion is unavailable; cardiac findings are only coronary atherosclerosis and unspecified mitral valve disorders. Age 47 does clear the 40–75 window. Independently trips a flat exclusion for insulin-treated diabetes — long-term use of insulin coded twice — and the "probable alternative diagnoses accounting for HF symptoms" exclusion names both anaemia (coded, Hgb 11.5) and obesity (coded). HbA1c unmeasured but diabetes is coded uncontrolled with neuro/renal/ophthalmic manifestations, so the HbA1c ceiling may also fire. eGFR clears (Cr 1.3, CKD III, well above the &lt;20 cutoff). CLOSES PATIENT 14721873's RUN OF NINE PAIRS — across all of them the operative disqualifiers were epilepsy, cerebral palsy, active foot osteomyelitis, and insulin-treated uncontrolled diabetes, not his cardiac diagnoses.</x:v>
+        <x:v>Phase 1b MAD study in symptomatic HFmrEF/HFpEF (NYHA II–III, LVEF &gt;40%, stable GDMT, plus NT-proBNP/echo or invasive filling-pressure criteria). Patient has NO heart failure diagnosis of any kind, no LVEF, no echo, no natriuretic peptides, no diuretic therapy, no HF hospitalization, no catheterization. Every route to satisfying the biomarker/echo criterion is unavailable; cardiac findings are only coronary atherosclerosis and unspecified mitral valve disorders. Age 47 does clear the 40–75 window. Independently trips a flat exclusion for insulin-treated diabetes, long-term use of insulin coded twice, and the "probable alternative diagnoses accounting for HF symptoms" exclusion names both anaemia (coded, Hgb 11.5) and obesity (coded). HbA1c unmeasured but diabetes is coded uncontrolled with neuro/renal/ophthalmic manifestations, so the HbA1c ceiling may also fire. eGFR clears (Cr 1.3, CKD III, well above the &lt;20 cutoff). CLOSES PATIENT 14721873's RUN OF NINE PAIRS, across all of them the operative disqualifiers were epilepsy, cerebral palsy, active foot osteomyelitis, and insulin-treated uncontrolled diabetes, not his cardiac diagnoses.</x:v>
       </x:c>
     </x:row>
     <x:row r="982" ht="58" customHeight="1">
@@ -27711,7 +27711,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I982" s="9" t="str">
-        <x:v>STEMI reperfusion trial (ischemic postconditioning + IVUS-guided primary PCI) with entry defined by specific ST-elevation ECG thresholds. Patient's infarct is coded SUBENDOCARDIAL INFARCTION — the ICD designation for NSTEMI — which directly contradicts the required presentation. Not a documentation gap: STEMI and NSTEMI are separately coded and hers is explicitly non-ST-elevation, supported by an enzymatic diagnosis (CK 304, CK-MB 37, CK-MB index 12.2%). Both trial arms depend on acute total occlusion with transmural ischemia, which subendocardial infarction is by definition not. Also likely trips the "culprit in bypass graft" exclusion shared by both arms — coronary atherosclerosis of autologous vein bypass graft coded, CABG in tags — though the culprit vessel isn't specified. Age 83 clears (≥18, no upper limit); capacity appears intact. SUBTLE-BUT-DECISIVE CASE: MI present, PCI present, drug-eluting stent placed — only the infarct SUBTYPE separates match from no match. Good discrimination probe.</x:v>
+        <x:v>STEMI reperfusion trial (ischemic postconditioning + IVUS-guided primary PCI) with entry defined by specific ST-elevation ECG thresholds. Patient's infarct is coded SUBENDOCARDIAL INFARCTION, the ICD designation for NSTEMI, which directly contradicts the required presentation. Not a documentation gap: STEMI and NSTEMI are separately coded and hers is explicitly non-ST-elevation, supported by an enzymatic diagnosis (CK 304, CK-MB 37, CK-MB index 12.2%). Both trial arms depend on acute total occlusion with transmural ischemia, which subendocardial infarction is by definition not. Also likely trips the "culprit in bypass graft" exclusion shared by both arms, coronary atherosclerosis of autologous vein bypass graft coded, CABG in tags, though the culprit vessel isn't specified. Age 83 clears (≥18, no upper limit); capacity appears intact. SUBTLE-BUT-DECISIVE CASE: MI present, PCI present, drug-eluting stent placed, only the infarct SUBTYPE separates match from no match. Good discrimination probe.</x:v>
       </x:c>
     </x:row>
     <x:row r="983" ht="58" customHeight="1">
@@ -27740,7 +27740,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I983" s="9" t="str">
-        <x:v>ULTRA-CTO enrolls patients after PCI of a CHRONIC TOTAL OCCLUSION, then performs intracoronary physiology (RFR/FFR/CFR/IMR) and OCT on the treated vessel. Patient did have PCI — single-vessel PTCA, one drug-eluting stent, coronary arteriography, left heart cath — but the indication was acute subendocardial infarction, not a CTO. No CTO coded anywhere; CTO PCI is elective for a ≥3-month occlusion, a different entity from an acute NSTEMI intervention. No OCT and no physiologic measurements performed, and the protocol states patients in whom these can't be done are not included. Coronary atherosclerosis of autologous vein bypass graft also bears on the "no remaining lesion ≥30% proximal to stent" requirement. Sole exclusion — adenosine contraindication — likely fires: chronic airway obstruction, supplemental oxygen dependence, postinflammatory pulmonary fibrosis; adenosine is contraindicated in bronchospastic disease and is required for the hyperemic measurements. Age 83 clears. SECOND CONSECUTIVE PAIR for her where PCI is documented but lesion/infarct subtype decides the verdict.</x:v>
+        <x:v>ULTRA-CTO enrolls patients after PCI of a CHRONIC TOTAL OCCLUSION, then performs intracoronary physiology (RFR/FFR/CFR/IMR) and OCT on the treated vessel. Patient did have PCI, single-vessel PTCA, one drug-eluting stent, coronary arteriography, left heart cath, but the indication was acute subendocardial infarction, not a CTO. No CTO coded anywhere; CTO PCI is elective for a ≥3-month occlusion, a different entity from an acute NSTEMI intervention. No OCT and no physiologic measurements performed, and the protocol states patients in whom these can't be done are not included. Coronary atherosclerosis of autologous vein bypass graft also bears on the "no remaining lesion ≥30% proximal to stent" requirement. Sole exclusion, adenosine contraindication, likely fires: chronic airway obstruction, supplemental oxygen dependence, postinflammatory pulmonary fibrosis; adenosine is contraindicated in bronchospastic disease and is required for the hyperemic measurements. Age 83 clears. SECOND CONSECUTIVE PAIR for her where PCI is documented but lesion/infarct subtype decides the verdict.</x:v>
       </x:c>
     </x:row>
     <x:row r="984" ht="58" customHeight="1">
@@ -27769,7 +27769,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I984" s="9" t="str">
-        <x:v>IVUS/angiography machine-learning registry for stent optimization. Explicit unqualified exclusion for patients who underwent CABG — she has CABG in clinical tags with coronary atherosclerosis of autologous vein bypass graft coded. Rationale is sound: prior surgical revascularization alters coronary physiology, collaterals, and vessel morphology, confounding FFR-prediction and stent-expansion algorithms. Inclusion side actually fits well — age 83 (≥19), objective ischemia with enzymatically confirmed subendocardial infarction (CK 304, CK-MB 37, index 12.2%), and a major epicardial vessel stented (single-vessel PTCA with DES, coronary arteriography, left heart cath). Her NSTEMI coding works IN HER FAVOR here, since the STEMI-at-admission exclusion doesn't fire. No shock, no antiplatelet contraindication (plt 186–191, Hct 35.9–37.9). LVEF undocumented; 2-year follow-up endpoint is a legitimate concern at 83 with oxygen-dependent COPD and pulmonary fibrosis. A culprit within the vein graft would compound the exclusion. Korean multicenter; enrollment window originally Jan 2020–Jun 2025 though still listed recruiting — worth confirming still open. SINGLE-EXCLUSION CASE like 001004 and 001023.</x:v>
+        <x:v>IVUS/angiography machine-learning registry for stent optimization. Explicit unqualified exclusion for patients who underwent CABG, she has CABG in clinical tags with coronary atherosclerosis of autologous vein bypass graft coded. Rationale is sound: prior surgical revascularization alters coronary physiology, collaterals, and vessel morphology, confounding FFR-prediction and stent-expansion algorithms. Inclusion side actually fits well, age 83 (≥19), objective ischemia with enzymatically confirmed subendocardial infarction (CK 304, CK-MB 37, index 12.2%), and a major epicardial vessel stented (single-vessel PTCA with DES, coronary arteriography, left heart cath). Her NSTEMI coding works IN HER FAVOR here, since the STEMI-at-admission exclusion doesn't fire. No shock, no antiplatelet contraindication (plt 186–191, Hct 35.9–37.9). LVEF undocumented; 2-year follow-up endpoint is a legitimate concern at 83 with oxygen-dependent COPD and pulmonary fibrosis. A culprit within the vein graft would compound the exclusion. Korean multicenter; enrollment window originally Jan 2020–Jun 2025 though still listed recruiting, worth confirming still open. SINGLE-EXCLUSION CASE like 001004 and 001023.</x:v>
       </x:c>
     </x:row>
     <x:row r="985" ht="58" customHeight="1">
@@ -27798,7 +27798,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I985" s="9" t="str">
-        <x:v>PRIMARY prevention trial in ASYMPTOMATIC patients with subclinical coronary calcification (Agatston ≥100) and no established CVD. Patient is the inverse on both axes. High-priority exclusion "history of coronary or peripheral arterial revascularization" is met twice: prior CABG with coronary atherosclerosis of autologous vein bypass graft, and PCI this encounter (PTCA, single-vessel, drug-eluting stent, coronary arteriography, left heart cath). Also not asymptomatic — subendocardial infarction with enzymatic confirmation (CK 304, CK-MB 37, index 12.2%) — and she had objective ischemia that actually required and received revascularization, tripping that exclusion too. No CAC score obtained, and CAC scanning has no clinical role in a patient with prior CABG and a fresh stent. Cerebrovascular exclusion does NOT fire (no stroke/TIA coded); no liver disease, no statin intolerance. Age 83 clears ≥40; life-expectancy consideration reasonable given oxygen-dependent COPD and pulmonary fibrosis but not clearly &lt;1 yr. NO EQUIPOISE — she'd already be on high-intensity statin as standard secondary prevention. Clean primary-vs-secondary prevention mismatch.</x:v>
+        <x:v>PRIMARY prevention trial in ASYMPTOMATIC patients with subclinical coronary calcification (Agatston ≥100) and no established CVD. Patient is the inverse on both axes. High-priority exclusion "history of coronary or peripheral arterial revascularization" is met twice: prior CABG with coronary atherosclerosis of autologous vein bypass graft, and PCI this encounter (PTCA, single-vessel, drug-eluting stent, coronary arteriography, left heart cath). Also not asymptomatic, subendocardial infarction with enzymatic confirmation (CK 304, CK-MB 37, index 12.2%), and she had objective ischemia that actually required and received revascularization, tripping that exclusion too. No CAC score obtained, and CAC scanning has no clinical role in a patient with prior CABG and a fresh stent. Cerebrovascular exclusion does NOT fire (no stroke/TIA coded); no liver disease, no statin intolerance. Age 83 clears ≥40; life-expectancy consideration reasonable given oxygen-dependent COPD and pulmonary fibrosis but not clearly &lt;1 yr. NO EQUIPOISE, she'd already be on high-intensity statin as standard secondary prevention. Clean primary-vs-secondary prevention mismatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="986" ht="58" customHeight="1">
@@ -27827,7 +27827,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I986" s="9" t="str">
-        <x:v>Cangrelor vs clopidogrel for microvascular protection during ELECTIVE PCI in CHRONIC coronary syndrome, with acute coronary syndromes an explicit exclusion. Patient's subendocardial infarction is an NSTEMI — by definition an ACS — and her PCI was performed for that acute event, not electively. This is the study's whole premise: cangrelor's proposed benefit is in stable patients inadequately P2Y12-loaded at a planned procedure; in ACS potent antiplatelet loading is already standard, so no equipoise. Also no FFR measured, so the required functionally significant (FFR ≤0.80) de-novo intermediate stenosis was never established, and coronary atherosclerosis of autologous vein bypass graft raises whether the target was de-novo in a native major vessel. NSTEMI culprits are often &gt;90% stenosed, which would independently trip the subtotal-occlusion exclusion. P2Y12-naive status undocumented pre-procedure and plausible she was already on therapy given prior CABG. No HF coded so the LVEF &lt;30% exclusion doesn't fire. FOURTH PAIR in her series decided by acute-vs-chronic or STEMI-vs-NSTEMI rather than by presence of CAD — tests whether the model reads presentation context, not just diagnosis tags.</x:v>
+        <x:v>Cangrelor vs clopidogrel for microvascular protection during ELECTIVE PCI in CHRONIC coronary syndrome, with acute coronary syndromes an explicit exclusion. Patient's subendocardial infarction is an NSTEMI, by definition an ACS, and her PCI was performed for that acute event, not electively. This is the study's whole premise: cangrelor's proposed benefit is in stable patients inadequately P2Y12-loaded at a planned procedure; in ACS potent antiplatelet loading is already standard, so no equipoise. Also no FFR measured, so the required functionally significant (FFR ≤0.80) de-novo intermediate stenosis was never established, and coronary atherosclerosis of autologous vein bypass graft raises whether the target was de-novo in a native major vessel. NSTEMI culprits are often &gt;90% stenosed, which would independently trip the subtotal-occlusion exclusion. P2Y12-naive status undocumented pre-procedure and plausible she was already on therapy given prior CABG. No HF coded so the LVEF &lt;30% exclusion doesn't fire. FOURTH PAIR in her series decided by acute-vs-chronic or STEMI-vs-NSTEMI rather than by presence of CAD, tests whether the model reads presentation context, not just diagnosis tags.</x:v>
       </x:c>
     </x:row>
     <x:row r="987" ht="58" customHeight="1">
@@ -27854,7 +27854,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I987" s="9" t="str">
-        <x:v>Nurse-led web-based physical activity pilot with NO exclusion criteria at all. Inclusions fit her directly: age 83 (≥65, high-priority), ~3 months post-hospitalization for PCI or CABG — she has both, with PTCA, single-vessel procedure, and drug-eluting stent this encounter after a subendocardial infarction, plus prior CABG evidenced by coronary atherosclerosis of autologous vein bypass graft. No cognitive impairment coded; depressive disorder and anxiety state are documented but do not meet the protocol's cognitive definition (complex attention, executive function, learning, memory, social skills). Remaining criteria — French fluency, greater Montreal residence, internet access, interest in increasing activity, no concurrent cardiac rehab — are screening/logistical and shouldn't carry a rejection. MOST LIKELY PRACTICAL CONFLICT: post-PCI patients are routinely referred to cardiac rehab, which the protocol excludes concurrently — check directly. CLINICAL CAVEAT: oxygen-dependent chronic airway obstruction and postinflammatory pulmonary fibrosis, plus prior hip replacement, will shape a safe activity prescription — assessment, not disqualifier. First match after six consecutive no-match pairs, and it comes from the one trial with no exclusion list.</x:v>
+        <x:v>Nurse-led web-based physical activity pilot with NO exclusion criteria at all. Inclusions fit her directly: age 83 (≥65, high-priority), ~3 months post-hospitalization for PCI or CABG, she has both, with PTCA, single-vessel procedure, and drug-eluting stent this encounter after a subendocardial infarction, plus prior CABG evidenced by coronary atherosclerosis of autologous vein bypass graft. No cognitive impairment coded; depressive disorder and anxiety state are documented but do not meet the protocol's cognitive definition (complex attention, executive function, learning, memory, social skills). Remaining criteria, French fluency, greater Montreal residence, internet access, interest in increasing activity, no concurrent cardiac rehab, are screening/logistical and shouldn't carry a rejection. MOST LIKELY PRACTICAL CONFLICT: post-PCI patients are routinely referred to cardiac rehab, which the protocol excludes concurrently, check directly. CLINICAL CAVEAT: oxygen-dependent chronic airway obstruction and postinflammatory pulmonary fibrosis, plus prior hip replacement, will shape a safe activity prescription, assessment, not disqualifier. First match after six consecutive no-match pairs, and it comes from the one trial with no exclusion list.</x:v>
       </x:c>
     </x:row>
     <x:row r="988" ht="58" customHeight="1">
@@ -27881,7 +27881,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I988" s="9" t="str">
-        <x:v>Unlike INNOVATE-PCI (PAIR-001047), this protocol does NOT exclude prior CABG patients — only lesions LOCATED IN a bypass graft. That distinction keeps her in play. She is a stentable ischemic heart disease patient: subendocardial infarction with enzymatic confirmation, old MI, PTCA status, single-vessel PCI with drug-eluting stent after coronary arteriography and left heart cath. NSTEMI coding again works in her favor — the STEMI-culprit exclusion doesn't fire. High-priority bleeding-diathesis exclusion also clear (plt 186–191, Hct 35.9–37.9, tolerated DAPT). PIVOTAL UNKNOWN: coronary atherosclerosis of autologous vein bypass graft is coded, and the procedure record says only "procedure on single vessel" — if the graft was the target she is excluded outright; if native, she is not. One line in the cath report decides it. Secondary unknowns: stenosis not quantified (an NSTEMI culprit &gt;90% would fall outside the 50–90% window), vessel diameter, left main status, and angiographic image quality for QFR suitability. Life expectancy &lt;2 yr exclusion is arguable at 83 with oxygen dependence, chronic airway obstruction, and pulmonary fibrosis against a 24-month endpoint. NO exclusion is affirmatively documented — all are unverified, unlike her earlier pairs. LOW CONFIDENCE BY DESIGN: a reviewer assuming graft involvement would reasonably score NO MATCH.</x:v>
+        <x:v>Unlike INNOVATE-PCI (PAIR-001047), this protocol does NOT exclude prior CABG patients, only lesions LOCATED IN a bypass graft. That distinction keeps her in play. She is a stentable ischemic heart disease patient: subendocardial infarction with enzymatic confirmation, old MI, PTCA status, single-vessel PCI with drug-eluting stent after coronary arteriography and left heart cath. NSTEMI coding again works in her favor, the STEMI-culprit exclusion doesn't fire. High-priority bleeding-diathesis exclusion also clear (plt 186–191, Hct 35.9–37.9, tolerated DAPT). PIVOTAL UNKNOWN: coronary atherosclerosis of autologous vein bypass graft is coded, and the procedure record says only "procedure on single vessel", if the graft was the target she is excluded outright; if native, she is not. One line in the cath report decides it. Secondary unknowns: stenosis not quantified (an NSTEMI culprit &gt;90% would fall outside the 50–90% window), vessel diameter, left main status, and angiographic image quality for QFR suitability. Life expectancy &lt;2 yr exclusion is arguable at 83 with oxygen dependence, chronic airway obstruction, and pulmonary fibrosis against a 24-month endpoint. NO exclusion is affirmatively documented, all are unverified, unlike her earlier pairs. LOW CONFIDENCE BY DESIGN: a reviewer assuming graft involvement would reasonably score NO MATCH.</x:v>
       </x:c>
     </x:row>
     <x:row r="989" ht="58" customHeight="1">
@@ -27910,7 +27910,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I989" s="9" t="str">
-        <x:v>SAPT vs DAPT after drug-coated BALLOON PCI in elderly/HBR patients. Two-sided failure: the required index intervention (Essential Pro DCB) never occurred, and the explicit exclusion "stent implantation during index or recent &lt;6 months procedure" fires — she received insertion of drug-eluting coronary artery stent(s) this admission. The protocol's premise is that DCB leaves no metal behind, permitting shortened single antiplatelet therapy; a fresh DES mandates conventional DAPT and removes equipoise. Demographically she is ideal: age 83 satisfies the ≥75 route outright (HBR status not needed), and her subendocardial infarction is an unstable coronary syndrome, which is explicitly permitted. NSTEMI again avoids the STEMI exclusion. Other exclusions clear: Cr 1.0 (eGFR well above 30), platelets 186–191, no bleeding diathesis, no GI ulceration/perforation/bleeding, no HF coded, no methotrexate, no thyrotoxicosis. Vein graft atherosclerosis coded but target vessel unidentified — moot given the stent exclusion. DEVICE-STRATEGY MISMATCH, not a patient mismatch. Pairs instructively with PAIR-001042, the other DCB trial, where the same fit failed for the opposite reason (no DCB ever performed).</x:v>
+        <x:v>SAPT vs DAPT after drug-coated BALLOON PCI in elderly/HBR patients. Two-sided failure: the required index intervention (Essential Pro DCB) never occurred, and the explicit exclusion "stent implantation during index or recent &lt;6 months procedure" fires, she received insertion of drug-eluting coronary artery stent(s) this admission. The protocol's premise is that DCB leaves no metal behind, permitting shortened single antiplatelet therapy; a fresh DES mandates conventional DAPT and removes equipoise. Demographically she is ideal: age 83 satisfies the ≥75 route outright (HBR status not needed), and her subendocardial infarction is an unstable coronary syndrome, which is explicitly permitted. NSTEMI again avoids the STEMI exclusion. Other exclusions clear: Cr 1.0 (eGFR well above 30), platelets 186–191, no bleeding diathesis, no GI ulceration/perforation/bleeding, no HF coded, no methotrexate, no thyrotoxicosis. Vein graft atherosclerosis coded but target vessel unidentified, moot given the stent exclusion. DEVICE-STRATEGY MISMATCH, not a patient mismatch. Pairs instructively with PAIR-001042, the other DCB trial, where the same fit failed for the opposite reason (no DCB ever performed).</x:v>
       </x:c>
     </x:row>
     <x:row r="990" ht="58" customHeight="1">
@@ -27939,7 +27939,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I990" s="9" t="str">
-        <x:v>Retrospective CTO-PCI vs OMT cohort. High-priority exclusion for history of CABG fires — coronary atherosclerosis of autologous vein bypass graft coded, CABG in clinical tags — and the study's own detailed description states patients were excluded from the cohort for CABG surgery, so intent is unambiguous (prior bypass alters collateral supply and revascularization decisions in CTO territories). Independently, no chronic total occlusion appears anywhere in her record; her PCI treated an acute subendocardial infarct, and CTO is a specific angiographic entity (≥3 months, TIMI 0 flow) that is nowhere established. Second CTO-based trial she fails for that reason after PAIR-001045. STEMI exclusion does not fire (NSTEMI); no cardiogenic shock (Cr 1.0, bicarb 25–28, anion gap 13–14); no malignancy. Also a closed retrospective enrollment window, Jan 2011–Dec 2017, single center in Nanjing. PRIOR CABG IS NOW THE OPERATIVE EXCLUSION IN FOUR OF HER NINE PAIRS (001047, 001048, 001052, 001053) — if retrieval keys on CAD/PCI tags without weighting bypass history, that's a specific correctable failure mode.</x:v>
+        <x:v>Retrospective CTO-PCI vs OMT cohort. High-priority exclusion for history of CABG fires, coronary atherosclerosis of autologous vein bypass graft coded, CABG in clinical tags, and the study's own detailed description states patients were excluded from the cohort for CABG surgery, so intent is unambiguous (prior bypass alters collateral supply and revascularization decisions in CTO territories). Independently, no chronic total occlusion appears anywhere in her record; her PCI treated an acute subendocardial infarct, and CTO is a specific angiographic entity (≥3 months, TIMI 0 flow) that is nowhere established. Second CTO-based trial she fails for that reason after PAIR-001045. STEMI exclusion does not fire (NSTEMI); no cardiogenic shock (Cr 1.0, bicarb 25–28, anion gap 13–14); no malignancy. Also a closed retrospective enrollment window, Jan 2011–Dec 2017, single center in Nanjing. PRIOR CABG IS NOW THE OPERATIVE EXCLUSION IN FOUR OF HER NINE PAIRS (001047, 001048, 001052, 001053), if retrieval keys on CAD/PCI tags without weighting bypass history, that's a specific correctable failure mode.</x:v>
       </x:c>
     </x:row>
     <x:row r="991" ht="58" customHeight="1">
@@ -27968,7 +27968,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I991" s="9" t="str">
-        <x:v>Ultrasound renal denervation RCT for primary hypertension. She has the qualifying diagnosis (unspecified essential hypertension) but fails three ways. (1) Age 83 vs a high-priority hard ceiling of ≤75, missed by 8 years. (2) Long-term supplemental oxygen support is excluded by name outside nocturnal sleep-apnea use — "other dependence on machines, supplemental oxygen" coded with chronic airway obstruction and postinflammatory pulmonary fibrosis, so the carve-out doesn't apply. (3) Acute MI within 3 months — subendocardial infarction this admission (CK 304, CK-MB 37, index 12.2%). Protocol also requires swapping her regimen to valsartan/amlodipine ± HCTZ for a 4-week run-in, which would be clinically inadvisable days after an infarct; no BP values exist to assess the 150–179/≥90 and ABPM 135–169 windows. eGFR borderline — Cr 1.0 in an 83F ≈ mid-50s, likely above the &lt;45 cutoff but worth calculating. High-priority exclusions for T1DM and contrast allergy do NOT fire (no diabetes, glucose 104; she tolerated coronary arteriography and left heart cath). CLOSES PATIENT 14855185's TEN PAIRS — recurring disqualifiers were prior CABG, NSTEMI-vs-STEMI, and absence of a CTO; her one match came from the single trial with no exclusion criteria.</x:v>
+        <x:v>Ultrasound renal denervation RCT for primary hypertension. She has the qualifying diagnosis (unspecified essential hypertension) but fails three ways. (1) Age 83 vs a high-priority hard ceiling of ≤75, missed by 8 years. (2) Long-term supplemental oxygen support is excluded by name outside nocturnal sleep-apnea use, "other dependence on machines, supplemental oxygen" coded with chronic airway obstruction and postinflammatory pulmonary fibrosis, so the carve-out doesn't apply. (3) Acute MI within 3 months, subendocardial infarction this admission (CK 304, CK-MB 37, index 12.2%). Protocol also requires swapping her regimen to valsartan/amlodipine ± HCTZ for a 4-week run-in, which would be clinically inadvisable days after an infarct; no BP values exist to assess the 150–179/≥90 and ABPM 135–169 windows. eGFR borderline, Cr 1.0 in an 83F ≈ mid-50s, likely above the &lt;45 cutoff but worth calculating. High-priority exclusions for T1DM and contrast allergy do NOT fire (no diabetes, glucose 104; she tolerated coronary arteriography and left heart cath). CLOSES PATIENT 14855185's TEN PAIRS, recurring disqualifiers were prior CABG, NSTEMI-vs-STEMI, and absence of a CTO; her one match came from the single trial with no exclusion criteria.</x:v>
       </x:c>
     </x:row>
     <x:row r="992" ht="58" customHeight="1">
@@ -27997,7 +27997,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I992" s="9" t="str">
-        <x:v>Observational CMR perfusion study in hypertrophic cardiomyopathy phenotypes (sarcomeric HCM, Anderson-Fabry, cardiac amyloidosis), plus first-degree relatives and mutation carriers. Patient has none — no hypertrophic phenotype, no LVH, no AFD, no amyloidosis, no genetic testing, no family history; all three routes into the cohort fail. The trial's SOLE exclusion, flagged high priority, reads like her chart: previous MI or revascularization (CABG or PCI) and/or coronary stenosis ≥50%. She satisfies every clause — old myocardial infarction AND subendocardial infarction this admission; coronary atherosclerosis of autologous vein bypass graft with CABG in tags; PTCA status plus PTCA with drug-eluting stent this admission; ≥50% stenosis implicit in a stented lesion. Exclusion exists to keep ischemic microvascular disease out of the perfusion signature. Also no CMR performed or indicated, and CMR feasibility would be limited anyway by supplemental oxygen dependence, chronic airway obstruction, and pulmonary fibrosis. Age 83 clears ≥18. CLEANEST NEGATIVE IN THE PACKAGE — one exclusion criterion, met four ways, plus a failed defining inclusion. THIRD INSTANCE of the ischemic-patient-to-non-ischemic-cardiomyopathy-study pattern (with 001010, 001032) across three different patients.</x:v>
+        <x:v>Observational CMR perfusion study in hypertrophic cardiomyopathy phenotypes (sarcomeric HCM, Anderson-Fabry, cardiac amyloidosis), plus first-degree relatives and mutation carriers. Patient has none, no hypertrophic phenotype, no LVH, no AFD, no amyloidosis, no genetic testing, no family history; all three routes into the cohort fail. The trial's SOLE exclusion, flagged high priority, reads like her chart: previous MI or revascularization (CABG or PCI) and/or coronary stenosis ≥50%. She satisfies every clause, old myocardial infarction AND subendocardial infarction this admission; coronary atherosclerosis of autologous vein bypass graft with CABG in tags; PTCA status plus PTCA with drug-eluting stent this admission; ≥50% stenosis implicit in a stented lesion. Exclusion exists to keep ischemic microvascular disease out of the perfusion signature. Also no CMR performed or indicated, and CMR feasibility would be limited anyway by supplemental oxygen dependence, chronic airway obstruction, and pulmonary fibrosis. Age 83 clears ≥18. CLEANEST NEGATIVE IN THE PACKAGE, one exclusion criterion, met four ways, plus a failed defining inclusion. THIRD INSTANCE of the ischemic-patient-to-non-ischemic-cardiomyopathy-study pattern (with 001010, 001032) across three different patients.</x:v>
       </x:c>
     </x:row>
     <x:row r="993" ht="58" customHeight="1">
@@ -28026,7 +28026,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I993" s="9" t="str">
-        <x:v>RCT of extended-release vs immediate-release tacrolimus in LIVER transplant recipients, with basiliximab induction at POD 0 and 4 and day-3 bilirubin monitoring — the design presupposes an active liver transplant admission. Patient is a KIDNEY transplant recipient: kidney replaced by transplant, complications of transplanted kidney, renal dialysis status. No liver transplant, no cirrhosis, no hepatic failure, no liver disease of any kind. Wrong organ, wrong enrollment window. Two exclusions also fire squarely: CKD with eGFR &lt;45 — she has end stage renal disease, hypertensive CKD stage V/ESRD, and dialysis status, the most severe renal picture in the package — and acute kidney injury, with acute kidney failure plus lesion of tubular necrosis, transplant complications, hydronephrosis, ureteral calculus, UTI, nephrostomy tube removal, acidosis, and dehydration. No HCC (prior malignancy is skin), no re-transplant, no multi-visceral transplant, no long QT. DISTINCT ERROR TYPE from others in this package — not a subtype or timing confusion but a transplanted-ORGAN mismatch, trivially separable if the matcher reads the organ in the trial title.</x:v>
+        <x:v>RCT of extended-release vs immediate-release tacrolimus in LIVER transplant recipients, with basiliximab induction at POD 0 and 4 and day-3 bilirubin monitoring, the design presupposes an active liver transplant admission. Patient is a KIDNEY transplant recipient: kidney replaced by transplant, complications of transplanted kidney, renal dialysis status. No liver transplant, no cirrhosis, no hepatic failure, no liver disease of any kind. Wrong organ, wrong enrollment window. Two exclusions also fire squarely: CKD with eGFR &lt;45, she has end stage renal disease, hypertensive CKD stage V/ESRD, and dialysis status, the most severe renal picture in the package, and acute kidney injury, with acute kidney failure plus lesion of tubular necrosis, transplant complications, hydronephrosis, ureteral calculus, UTI, nephrostomy tube removal, acidosis, and dehydration. No HCC (prior malignancy is skin), no re-transplant, no multi-visceral transplant, no long QT. DISTINCT ERROR TYPE from others in this package, not a subtype or timing confusion but a transplanted-ORGAN mismatch, trivially separable if the matcher reads the organ in the trial title.</x:v>
       </x:c>
     </x:row>
     <x:row r="994" ht="58" customHeight="1">
@@ -28055,7 +28055,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I994" s="9" t="str">
-        <x:v>Postpartum microvascular physiology study (intradermal microdialysis) in women 12 weeks to 5 years after delivery, stratified by preeclampsia and prenatal low-dose aspirin exposure. Patient is 68 and not postpartum — the defining window is definitionally unreachable, and no obstetric history, preeclampsia, or prenatal aspirin exposure exists, so none of the four enrollment strata apply. Nearly every exclusion also fires: current daily aspirin use (long-term aspirin coded); CKD with eGFR &lt;60 — ESRD, hypertensive CKD stage V, dialysis status, AKI with tubular necrosis, transplanted kidney with complications; metabolic disease — insulin-treated T2DM with renal/ophthalmic/neurologic manifestations, background retinopathy, gastroparesis, obesity BMI 35.0–35.9, pure hypercholesterolemia, gout; current antihypertensive medication and pre-pregnancy hypertension (both high priority); likely statin therapy. BMI 35.0–35.9 is the opposite of the &lt;18.5 exclusion. Prior skin malignancy is worth noting given the intradermal technique. WEAKEST PAIRING IN THE PACKAGE — domain-level failure like PAIR-001016, should be filtered before criteria-level reasoning. Good sanity-check pair alongside that one.</x:v>
+        <x:v>Postpartum microvascular physiology study (intradermal microdialysis) in women 12 weeks to 5 years after delivery, stratified by preeclampsia and prenatal low-dose aspirin exposure. Patient is 68 and not postpartum, the defining window is definitionally unreachable, and no obstetric history, preeclampsia, or prenatal aspirin exposure exists, so none of the four enrollment strata apply. Nearly every exclusion also fires: current daily aspirin use (long-term aspirin coded); CKD with eGFR &lt;60, ESRD, hypertensive CKD stage V, dialysis status, AKI with tubular necrosis, transplanted kidney with complications; metabolic disease, insulin-treated T2DM with renal/ophthalmic/neurologic manifestations, background retinopathy, gastroparesis, obesity BMI 35.0–35.9, pure hypercholesterolemia, gout; current antihypertensive medication and pre-pregnancy hypertension (both high priority); likely statin therapy. BMI 35.0–35.9 is the opposite of the &lt;18.5 exclusion. Prior skin malignancy is worth noting given the intradermal technique. WEAKEST PAIRING IN THE PACKAGE, domain-level failure like PAIR-001016, should be filtered before criteria-level reasoning. Good sanity-check pair alongside that one.</x:v>
       </x:c>
     </x:row>
     <x:row r="995" ht="58" customHeight="1">
@@ -28084,7 +28084,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I995" s="9" t="str">
-        <x:v>Dara-CyBorD induction in NEWLY DIAGNOSED multiple myeloma with new-onset renal failure. Patient has the renal half emphatically — ESRD, hypertensive CKD stage V, dialysis status, AKI with tubular necrosis, transplanted kidney with complications — but NO multiple myeloma: no M protein, no free light chains, no SPEP/UPEP, no bone marrow biopsy, no PET-CT, no lytic lesions, no plasmacytoma. High-priority inclusion fails outright. Critically, her renal failure has a non-myeloma etiology — diabetic and hypertensive nephropathy progressing to ESRD — which is exactly the confounder the confirmed-MM requirement exists to exclude; the trial frames RI as a myeloma emergency requiring immediate antimyeloma therapy. Anemia and renal failure are attributable to her kidney disease, so they don't function as CRAB features. Only malignancy is a historical skin neoplasm, not active. Active infection requiring systemic therapy also excludes: Streptococcus infection, UTI, Norwalk virus, with hydronephrosis, ureteral calculus, and nephrostomy tube. Old MI is outside the 6-month window but ongoing angina bears on the uncontrolled-cardiac clause; diabetic neuropathy grade unspecified and relevant to bortezomib neurotoxicity. STRUCTURAL REPEAT OF PAIR-001000 — two myeloma trials, two patients without myeloma, both retrieved on non-oncologic features.</x:v>
+        <x:v>Dara-CyBorD induction in NEWLY DIAGNOSED multiple myeloma with new-onset renal failure. Patient has the renal half emphatically, ESRD, hypertensive CKD stage V, dialysis status, AKI with tubular necrosis, transplanted kidney with complications, but NO multiple myeloma: no M protein, no free light chains, no SPEP/UPEP, no bone marrow biopsy, no PET-CT, no lytic lesions, no plasmacytoma. High-priority inclusion fails outright. Critically, her renal failure has a non-myeloma etiology, diabetic and hypertensive nephropathy progressing to ESRD, which is exactly the confounder the confirmed-MM requirement exists to exclude; the trial frames RI as a myeloma emergency requiring immediate antimyeloma therapy. Anemia and renal failure are attributable to her kidney disease, so they don't function as CRAB features. Only malignancy is a historical skin neoplasm, not active. Active infection requiring systemic therapy also excludes: Streptococcus infection, UTI, Norwalk virus, with hydronephrosis, ureteral calculus, and nephrostomy tube. Old MI is outside the 6-month window but ongoing angina bears on the uncontrolled-cardiac clause; diabetic neuropathy grade unspecified and relevant to bortezomib neurotoxicity. STRUCTURAL REPEAT OF PAIR-001000, two myeloma trials, two patients without myeloma, both retrieved on non-oncologic features.</x:v>
       </x:c>
     </x:row>
     <x:row r="996" ht="58" customHeight="1">
@@ -28111,7 +28111,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I996" s="9" t="str">
-        <x:v>Phase 1 colchicine tolerability basket trial with permissive entry — age ≥18 plus either advanced CKD or chronic maintenance dialysis. Patient fits the Dialysis cohort: ESRD, renal dialysis status, hypertensive CKD stage V, and exactly the cardiovascular-risk-in-renal-disease profile targeted (old MI, angina, coronary atherosclerosis, PTCA status, PVD, insulin-treated diabetes, hypertension). No exclusion is affirmatively documented. THREE UNVERIFIED DISQUALIFIERS keep confidence low: (1) she is a kidney transplant recipient (kidney replaced by transplant, complications of transplanted kidney), so a strong P-gp/CYP3A4 inhibitor is likely — cyclosporine is a strong P-gp inhibitor and colchicine toxicity with CNIs in renal impairment is well described; this is the most important thing to check; (2) acute gouty arthropathy is coded and colchicine is first-line for gout, so she may already be on it — cuts both ways; (3) diabetes with neurological manifestations raises the pre-existing neuromuscular disease exclusion, relevant since colchicine causes myoneuropathy in renal impairment. Dialysis frequency and 90-day duration undocumented; transplant-then-dialysis sequence unclear. Norwalk virus is acute, NOT chronic diarrhea, so that exclusion doesn't fire — but gastroparesis, nausea, and dehydration bear on GI tolerability, which IS the primary endpoint. No CBC, LFTs, CK, or B12 available. Active infections and AKI/nephrostomy would need resolution first. LOW CONFIDENCE BY DESIGN — a reviewer assuming CNI use would reasonably score NO MATCH.</x:v>
+        <x:v>Phase 1 colchicine tolerability basket trial with permissive entry, age ≥18 plus either advanced CKD or chronic maintenance dialysis. Patient fits the Dialysis cohort: ESRD, renal dialysis status, hypertensive CKD stage V, and exactly the cardiovascular-risk-in-renal-disease profile targeted (old MI, angina, coronary atherosclerosis, PTCA status, PVD, insulin-treated diabetes, hypertension). No exclusion is affirmatively documented. THREE UNVERIFIED DISQUALIFIERS keep confidence low: (1) she is a kidney transplant recipient (kidney replaced by transplant, complications of transplanted kidney), so a strong P-gp/CYP3A4 inhibitor is likely, cyclosporine is a strong P-gp inhibitor and colchicine toxicity with CNIs in renal impairment is well described; this is the most important thing to check; (2) acute gouty arthropathy is coded and colchicine is first-line for gout, so she may already be on it, cuts both ways; (3) diabetes with neurological manifestations raises the pre-existing neuromuscular disease exclusion, relevant since colchicine causes myoneuropathy in renal impairment. Dialysis frequency and 90-day duration undocumented; transplant-then-dialysis sequence unclear. Norwalk virus is acute, NOT chronic diarrhea, so that exclusion doesn't fire, but gastroparesis, nausea, and dehydration bear on GI tolerability, which IS the primary endpoint. No CBC, LFTs, CK, or B12 available. Active infections and AKI/nephrostomy would need resolution first. LOW CONFIDENCE BY DESIGN, a reviewer assuming CNI use would reasonably score NO MATCH.</x:v>
       </x:c>
     </x:row>
     <x:row r="997" ht="58" customHeight="1">
@@ -28138,7 +28138,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I997" s="9" t="str">
-        <x:v>FFR vs IVUS-guided stenting after angiography-derived FFR decision-making. Patient has established symptomatic ischemic heart disease — angina pectoris, coronary atherosclerosis of NATIVE coronary artery, old MI, PTCA status, family history of IHD, PVD — so she is a reasonable candidate for angiography and, if a 50–90% lesion is found, for enrollment. CRITICALLY, NO CABG: the bypass-graft lesion exclusion that decided PAIR-001051 for the other patient does not apply here, making her a cleaner candidate for this protocol. No exclusion affirmatively documented — no bleeding diathesis (high-priority, doesn't fire; tolerates long-term aspirin), no STEMI culprit, no active GI/GU bleeding despite hydronephrosis, ureteral calculus, and nephrostomy. KEY GAP: no coronary angiography this encounter — documented procedure is pyelostomy/nephrostomy tube removal and the admission is urologic/renal — so the qualifying 50–90% stenosis is inferred, not demonstrated. MAIN CLINICAL CONCERN: life expectancy &lt;2 years exclusion against the 24-month POCO endpoint, given dialysis-dependent ESRD with failing transplant, insulin-treated diabetes with multi-organ complications, legal blindness, PVD, prior MI — 2-yr dialysis survival is roughly 75–80%, so not clearly disqualifying but an investigator could reasonably pause. Sequencing: active strep/UTI/Norwalk infections and AKI need resolution first; contrast timing is less of an issue since she is already dialysis-dependent. Consent needs accommodation for visual impairment. LOW CONFIDENCE — qualifying lesion inferred rather than shown.</x:v>
+        <x:v>FFR vs IVUS-guided stenting after angiography-derived FFR decision-making. Patient has established symptomatic ischemic heart disease, angina pectoris, coronary atherosclerosis of NATIVE coronary artery, old MI, PTCA status, family history of IHD, PVD, so she is a reasonable candidate for angiography and, if a 50–90% lesion is found, for enrollment. CRITICALLY, NO CABG: the bypass-graft lesion exclusion that decided PAIR-001051 for the other patient does not apply here, making her a cleaner candidate for this protocol. No exclusion affirmatively documented, no bleeding diathesis (high-priority, doesn't fire; tolerates long-term aspirin), no STEMI culprit, no active GI/GU bleeding despite hydronephrosis, ureteral calculus, and nephrostomy. KEY GAP: no coronary angiography this encounter, documented procedure is pyelostomy/nephrostomy tube removal and the admission is urologic/renal, so the qualifying 50–90% stenosis is inferred, not demonstrated. MAIN CLINICAL CONCERN: life expectancy &lt;2 years exclusion against the 24-month POCO endpoint, given dialysis-dependent ESRD with failing transplant, insulin-treated diabetes with multi-organ complications, legal blindness, PVD, prior MI, 2-yr dialysis survival is roughly 75–80%, so not clearly disqualifying but an investigator could reasonably pause. Sequencing: active strep/UTI/Norwalk infections and AKI need resolution first; contrast timing is less of an issue since she is already dialysis-dependent. Consent needs accommodation for visual impairment. LOW CONFIDENCE, qualifying lesion inferred rather than shown.</x:v>
       </x:c>
     </x:row>
     <x:row r="998" ht="58" customHeight="1">
@@ -28167,7 +28167,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I998" s="9" t="str">
-        <x:v>Post-PCI colchicine dosing RCT in China. Explicit numeric exclusion at eGFR &lt;30 — she has ESRD on maintenance dialysis (hypertensive CKD stage V/ESRD, renal dialysis status, AKI with tubular necrosis, transplant complications), far below the cutoff and the most severe renal impairment in the package. Two further failures: trial requires hospitalized CHD patients requiring PCI with ALL planned PCI completed during the admission, and her hospitalization is urologic/renal (hydronephrosis, ureteral calculus, UTI, pyelostomy and nephrostomy tube removal) with no PCI performed — her PTCA is historical, so there's no randomization anchor. And as a kidney transplant recipient she is almost certainly on maintenance immunosuppression, which the protocol excludes outright. Acute gouty arthropathy raises possible current colchicine use (10-day exclusion). Norwalk virus is acute, not chronic diarrhea, so that exclusion doesn't fire; gastroparesis and nausea bear on GI tolerability. Age 68 clears 18–80; no shock; skin malignancy historical not active; pregnancy exclusion moot. STRONG PROBE PAIRED WITH 001059: same drug, opposite renal criteria — REPAIR is designed FOR dialysis patients, this trial excludes them because colchicine accumulates in renal failure. Tests whether the model reads renal thresholds directionally rather than as generic topical overlap.</x:v>
+        <x:v>Post-PCI colchicine dosing RCT in China. Explicit numeric exclusion at eGFR &lt;30, she has ESRD on maintenance dialysis (hypertensive CKD stage V/ESRD, renal dialysis status, AKI with tubular necrosis, transplant complications), far below the cutoff and the most severe renal impairment in the package. Two further failures: trial requires hospitalized CHD patients requiring PCI with ALL planned PCI completed during the admission, and her hospitalization is urologic/renal (hydronephrosis, ureteral calculus, UTI, pyelostomy and nephrostomy tube removal) with no PCI performed, her PTCA is historical, so there's no randomization anchor. And as a kidney transplant recipient she is almost certainly on maintenance immunosuppression, which the protocol excludes outright. Acute gouty arthropathy raises possible current colchicine use (10-day exclusion). Norwalk virus is acute, not chronic diarrhea, so that exclusion doesn't fire; gastroparesis and nausea bear on GI tolerability. Age 68 clears 18–80; no shock; skin malignancy historical not active; pregnancy exclusion moot. STRONG PROBE PAIRED WITH 001059: same drug, opposite renal criteria, REPAIR is designed FOR dialysis patients, this trial excludes them because colchicine accumulates in renal failure. Tests whether the model reads renal thresholds directionally rather than as generic topical overlap.</x:v>
       </x:c>
     </x:row>
     <x:row r="999" ht="58" customHeight="1">
@@ -28194,7 +28194,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I999" s="9" t="str">
-        <x:v>Best-aimed trial in her series — IVUS-CKD exists specifically for CKD patients with CAD and she is both. Satisfies eGFR &lt;60 emphatically (ESRD, hypertensive CKD stage V, dialysis status, AKI with tubular necrosis, transplant complications) and has symptomatic native-vessel disease (angina pectoris, coronary atherosclerosis of native coronary artery, old MI, PTCA status). BOTH high-priority exclusions clear: no antiplatelet contraindication (tolerates long-term aspirin) and no intracranial/GI bleeding history. No anticoagulants — aspirin is antiplatelet and is explicitly carved out of the nephrotoxic-medication exclusion. Life expectancy &lt;1 yr likely clears (1-yr dialysis survival ~80–85%), a lower bar than FLAVOUR III's 2-year. THREE OPEN ITEMS: (1) PTCA is UNDATED and PCI within 12 months excludes — one chart detail resolves it; (2) "immune-related kidney disease OR ON HORMONE THERAPY" may capture maintenance corticosteroids, which most kidney transplant recipients take — her nephropathy itself is diabetic/hypertensive, not immune; (3) no angiography this encounter (documented procedure is pyelostomy/nephrostomy tube removal), so the de novo DES/IVUS-suitable lesion is inferred, and prior PTCA raises whether the target would be restenotic rather than de novo. CONCEPTUAL TENSION WORTH FLAGGING: IVUS guidance in CKD is premised on limiting contrast to preserve residual renal function, which has little purpose in a maintenance dialysis patient — an investigator could reasonably decline even though the written criteria permit her. Also check for planned urologic surgery within 12 months given hydronephrosis, ureteral calculus, and nephrostomy.</x:v>
+        <x:v>Best-aimed trial in her series, IVUS-CKD exists specifically for CKD patients with CAD and she is both. Satisfies eGFR &lt;60 emphatically (ESRD, hypertensive CKD stage V, dialysis status, AKI with tubular necrosis, transplant complications) and has symptomatic native-vessel disease (angina pectoris, coronary atherosclerosis of native coronary artery, old MI, PTCA status). BOTH high-priority exclusions clear: no antiplatelet contraindication (tolerates long-term aspirin) and no intracranial/GI bleeding history. No anticoagulants, aspirin is antiplatelet and is explicitly carved out of the nephrotoxic-medication exclusion. Life expectancy &lt;1 yr likely clears (1-yr dialysis survival ~80–85%), a lower bar than FLAVOUR III's 2-year. THREE OPEN ITEMS: (1) PTCA is UNDATED and PCI within 12 months excludes, one chart detail resolves it; (2) "immune-related kidney disease OR ON HORMONE THERAPY" may capture maintenance corticosteroids, which most kidney transplant recipients take, her nephropathy itself is diabetic/hypertensive, not immune; (3) no angiography this encounter (documented procedure is pyelostomy/nephrostomy tube removal), so the de novo DES/IVUS-suitable lesion is inferred, and prior PTCA raises whether the target would be restenotic rather than de novo. CONCEPTUAL TENSION WORTH FLAGGING: IVUS guidance in CKD is premised on limiting contrast to preserve residual renal function, which has little purpose in a maintenance dialysis patient, an investigator could reasonably decline even though the written criteria permit her. Also check for planned urologic surgery within 12 months given hydronephrosis, ureteral calculus, and nephrostomy.</x:v>
       </x:c>
     </x:row>
     <x:row r="1000" ht="58" customHeight="1">
@@ -28223,7 +28223,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I1000" s="9" t="str">
-        <x:v>Beet-nitrate supplement for prevention of contrast-induced nephropathy in high-risk patients undergoing planned PCI. Unqualified "infectious diseases" exclusion fires directly — Streptococcus infection, UTI, and Norwalk virus, with hydronephrosis, ureteral calculus, and nephrostomy tube. No planned PCI: this admission is urologic/renal (pyelostomy and nephrostomy tube removal), PTCA status is historical, and the intervention starts 24h before a scheduled PCI, so there is no dosing window. DEEPEST PROBLEM IS PREMISE FAILURE: she is on maintenance dialysis with ESRD, so there is no residual renal function to protect and the primary endpoints (eGFR decline, NGAL, cystatin C) are uninterpretable in an anuric patient. She technically satisfies the high-CIN-risk inclusion (eGFR far below 60, plus insulin-treated diabetes), but that criterion identifies patients at risk of DEVELOPING CIN and she has already reached end-stage disease. Nitrate use in the last 30 days unverifiable and realistic given angina. Angina coded as "other and unspecified" — if unstable, the ACS exclusion would also fire; MI is old, not acute. No hypotension, shock, or cognitive decline. PAIRS WITH 001063: both trials aim to preserve kidney function during contrast exposure, and in both her dialysis dependence makes her the highest-risk-LOOKING candidate on paper and the least appropriate clinically. That criterion-vs-clinical-logic gap is a valuable eval case.</x:v>
+        <x:v>Beet-nitrate supplement for prevention of contrast-induced nephropathy in high-risk patients undergoing planned PCI. Unqualified "infectious diseases" exclusion fires directly, Streptococcus infection, UTI, and Norwalk virus, with hydronephrosis, ureteral calculus, and nephrostomy tube. No planned PCI: this admission is urologic/renal (pyelostomy and nephrostomy tube removal), PTCA status is historical, and the intervention starts 24h before a scheduled PCI, so there is no dosing window. DEEPEST PROBLEM IS PREMISE FAILURE: she is on maintenance dialysis with ESRD, so there is no residual renal function to protect and the primary endpoints (eGFR decline, NGAL, cystatin C) are uninterpretable in an anuric patient. She technically satisfies the high-CIN-risk inclusion (eGFR far below 60, plus insulin-treated diabetes), but that criterion identifies patients at risk of DEVELOPING CIN and she has already reached end-stage disease. Nitrate use in the last 30 days unverifiable and realistic given angina. Angina coded as "other and unspecified", if unstable, the ACS exclusion would also fire; MI is old, not acute. No hypotension, shock, or cognitive decline. PAIRS WITH 001063: both trials aim to preserve kidney function during contrast exposure, and in both her dialysis dependence makes her the highest-risk-LOOKING candidate on paper and the least appropriate clinically. That criterion-vs-clinical-logic gap is a valuable eval case.</x:v>
       </x:c>
     </x:row>
     <x:row r="1001" ht="58" customHeight="1">
@@ -28252,7 +28252,7 @@
         <x:v>Sahil</x:v>
       </x:c>
       <x:c r="I1001" s="9" t="str">
-        <x:v>Same renal denervation trial as PAIR-001054, different failure. AGE ACTUALLY PASSES here — 68 is inside the 18–75 window that disqualified the 83F. Decisive exclusion is eGFR &lt;45: ESRD, hypertensive CKD stage V, renal dialysis status, AKI with tubular necrosis, transplant complications. Three compounding problems: (1) high-priority T1DM exclusion — her record carries "diabetes with ophthalmic manifestations, type I [juvenile type]" and "diabetes with renal manifestations, type I [juvenile type]" alongside multiple type II codes; internally inconsistent but type 1 codes are affirmatively present and need adjudication. (2) Kidney replaced by transplant — a transplanted kidney is anastomosed to iliac vessels, so the catheter-based renal artery ablation has no appropriate target; hydronephrosis and ureteral calculus indicate further abnormal anatomy. (3) Hypertension in dialysis-dependent ESRD is volume-dependent renoparenchymal and would likely be adjudicated SECONDARY, tripping that exclusion despite the essential hypertension code. Also the 4-week run-in requires valsartan/amlodipine ± HCTZ, and a thiazide is pharmacologically useless in an anuric patient whose BP is managed by ultrafiltration. Oxygen-support and contrast-allergy exclusions do NOT fire (unlike the prior patient). Old MI likely outside the 3-month window; unstable angina would fire if present. SAME TRIAL REJECTED TWO PATIENTS ON ENTIRELY DIFFERENT GROUNDS — good illustration of why criterion-by-criterion evaluation beats trial-level pattern matching.</x:v>
+        <x:v>Same renal denervation trial as PAIR-001054, different failure. AGE ACTUALLY PASSES here, 68 is inside the 18–75 window that disqualified the 83F. Decisive exclusion is eGFR &lt;45: ESRD, hypertensive CKD stage V, renal dialysis status, AKI with tubular necrosis, transplant complications. Three compounding problems: (1) high-priority T1DM exclusion, her record carries "diabetes with ophthalmic manifestations, type I [juvenile type]" and "diabetes with renal manifestations, type I [juvenile type]" alongside multiple type II codes; internally inconsistent but type 1 codes are affirmatively present and need adjudication. (2) Kidney replaced by transplant, a transplanted kidney is anastomosed to iliac vessels, so the catheter-based renal artery ablation has no appropriate target; hydronephrosis and ureteral calculus indicate further abnormal anatomy. (3) Hypertension in dialysis-dependent ESRD is volume-dependent renoparenchymal and would likely be adjudicated SECONDARY, tripping that exclusion despite the essential hypertension code. Also the 4-week run-in requires valsartan/amlodipine ± HCTZ, and a thiazide is pharmacologically useless in an anuric patient whose BP is managed by ultrafiltration. Oxygen-support and contrast-allergy exclusions do NOT fire (unlike the prior patient). Old MI likely outside the 3-month window; unstable angina would fire if present. SAME TRIAL REJECTED TWO PATIENTS ON ENTIRELY DIFFERENT GROUNDS, good illustration of why criterion-by-criterion evaluation beats trial-level pattern matching.</x:v>
       </x:c>
     </x:row>
     <x:row r="1002" ht="58" customHeight="1">
@@ -30622,8 +30622,8 @@
         <x:v>Tara Lam</x:v>
       </x:c>
       <x:c r="I1081" s="9" t="str">
-        <x:v>Established type 2 diabetes mellitus — explicitly prohibited by the trial, regardless of HbA1c. The diagnosis is corroborated by chronic insulin and oral hypoglycemic use.
-Established clinical heart failure — documented as hypertensive heart disease with heart failure and acute-on-chronic diastolic heart failure.</x:v>
+        <x:v>Established type 2 diabetes mellitus, explicitly prohibited by the trial, regardless of HbA1c. The diagnosis is corroborated by chronic insulin and oral hypoglycemic use.
+Established clinical heart failure, documented as hypertensive heart disease with heart failure and acute-on-chronic diastolic heart failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="1082" ht="58" customHeight="1">
@@ -33119,7 +33119,7 @@
         <x:v>Sachin</x:v>
       </x:c>
       <x:c r="I1167" s="9" t="str">
-        <x:v>Trial is a treatment trial for patients with advanced structural heart disease plus recurrent monomorphic ventricular tachycardia (VT). The patient clearly has qualifying-type structural disease—dilated cardiomyopathy/chronic systolic HF—but her documented rhythm diagnosis is ventricular premature depolarization, not recurrent monomorphic VT.</x:v>
+        <x:v>Trial is a treatment trial for patients with advanced structural heart disease plus recurrent monomorphic ventricular tachycardia (VT). The patient clearly has qualifying-type structural disease, dilated cardiomyopathy/chronic systolic HF, but her documented rhythm diagnosis is ventricular premature depolarization, not recurrent monomorphic VT.</x:v>
       </x:c>
     </x:row>
     <x:row r="1168" ht="58" customHeight="1">
@@ -33335,7 +33335,7 @@
         <x:v>Sachin</x:v>
       </x:c>
       <x:c r="I1175" s="9" t="str">
-        <x:v>trial requires fairly specific current target-lesion findings—OCT calcium arc ≥270°, defined stenosis/severity criteria, suitable vessel diameter, and inadequate preparation with a non-compliant balloon.</x:v>
+        <x:v>trial requires fairly specific current target-lesion findings, OCT calcium arc ≥270°, defined stenosis/severity criteria, suitable vessel diameter, and inadequate preparation with a non-compliant balloon.</x:v>
       </x:c>
     </x:row>
     <x:row r="1176" ht="58" customHeight="1">
@@ -33954,7 +33954,7 @@
         <x:v>Sachin</x:v>
       </x:c>
       <x:c r="I1197" s="9" t="str">
-        <x:v>Prior CABG — Definitively present. This is an explicit protocol exclusion</x:v>
+        <x:v>Prior CABG, Definitively present. This is an explicit protocol exclusion</x:v>
       </x:c>
     </x:row>
     <x:row r="1198" ht="58" customHeight="1">
@@ -34748,7 +34748,7 @@
         <x:v>Sachin</x:v>
       </x:c>
       <x:c r="I1225" s="9" t="str">
-        <x:v>Prior CABG — definite hard exclusion.</x:v>
+        <x:v>Prior CABG, definite hard exclusion.</x:v>
       </x:c>
     </x:row>
     <x:row r="1226" ht="58" customHeight="1">
@@ -34804,7 +34804,7 @@
         <x:v>Sachin</x:v>
       </x:c>
       <x:c r="I1227" s="9" t="str">
-        <x:v>If ultimately screen-failed, the most plausible mechanism would be a medication/timing mismatch—specifically inability to document &gt;5 years of stable antihypertensive, lipid-lowering, or type-2 diabetes therapy</x:v>
+        <x:v>If ultimately screen-failed, the most plausible mechanism would be a medication/timing mismatch, specifically inability to document &gt;5 years of stable antihypertensive, lipid-lowering, or type-2 diabetes therapy</x:v>
       </x:c>
     </x:row>
     <x:row r="1228" ht="58" customHeight="1">
@@ -53207,7 +53207,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc98a2cc6513483f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dc98c7af5f94b55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>